<commit_message>
Remove UPV affiliation for Leire Larizgoitia, leaving DIPC only
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sorel/next/next-exp/NEXTAuthorList/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B65F58-7CF5-854C-B147-13AB2C15A29B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D11A965-454F-F74F-A334-2AAEC49CFFB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11820" yWindow="3120" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11640" yWindow="3120" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AuthorList" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="475">
   <si>
     <t>LastName</t>
   </si>
@@ -3532,12 +3532,6 @@
       <c r="I54" t="s">
         <v>19</v>
       </c>
-      <c r="J54" t="s">
-        <v>297</v>
-      </c>
-      <c r="K54" t="s">
-        <v>293</v>
-      </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">

</xml_diff>

<commit_message>
removed C. Adams, A.I. Aranburu, K. Bailey, A. Bayo, L. Cid. Last active dates asdded for I.J. Arnquist, E. Church and P. Dietz. ORCIDs added for I. Osborne and L.M. Villar Padruno
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sorel/next/next-exp/NEXTAuthorList/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D11A965-454F-F74F-A334-2AAEC49CFFB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC5660A-F82B-A14F-AF90-C8BE4DAB2757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11640" yWindow="3120" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10940" yWindow="3640" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AuthorList" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="461">
   <si>
     <t>LastName</t>
   </si>
@@ -58,9 +58,6 @@
     <t>Address2</t>
   </si>
   <si>
-    <t>Adams</t>
-  </si>
-  <si>
     <t>C.</t>
   </si>
   <si>
@@ -94,12 +91,6 @@
     <t>San Sebasti\'an / Donostia, E-20018, Spain</t>
   </si>
   <si>
-    <t>Aranburu</t>
-  </si>
-  <si>
-    <t>A.I.</t>
-  </si>
-  <si>
     <t>Department of Applied Chemistry, Universidad del Pais Vasco (UPV/EHU), Manuel de Lardizabal 3</t>
   </si>
   <si>
@@ -142,9 +133,6 @@
     <t xml:space="preserve"> Aveiro, 3810-193, Portugal             </t>
   </si>
   <si>
-    <t xml:space="preserve">Bailey                       </t>
-  </si>
-  <si>
     <t xml:space="preserve">Ballester                    </t>
   </si>
   <si>
@@ -523,9 +511,6 @@
     <t>C.D.R.</t>
   </si>
   <si>
-    <t xml:space="preserve">K.         </t>
-  </si>
-  <si>
     <t xml:space="preserve">F.         </t>
   </si>
   <si>
@@ -664,9 +649,6 @@
     <t>vicente.alvarez@ific.uv.es</t>
   </si>
   <si>
-    <t>aneiaranburu.94@gmail.com</t>
-  </si>
-  <si>
     <t>larazi@bgu.ac.il</t>
   </si>
   <si>
@@ -682,9 +664,6 @@
     <t>cdazevedo@ua.pt</t>
   </si>
   <si>
-    <t>kevin_bailey@anl.gov</t>
-  </si>
-  <si>
     <t>fballest@eln.upv.es</t>
   </si>
   <si>
@@ -1042,12 +1021,6 @@
     <t>Ruiz-Ch\'oliz</t>
   </si>
   <si>
-    <t>Now at NVIDIA.</t>
-  </si>
-  <si>
-    <t>coreya@nvidia.com</t>
-  </si>
-  <si>
     <t>Vanga</t>
   </si>
   <si>
@@ -1057,30 +1030,15 @@
     <t>Cid</t>
   </si>
   <si>
-    <t>Bayo</t>
-  </si>
-  <si>
-    <t>abayo@lsc-canfranc.es</t>
-  </si>
-  <si>
-    <t>lcid@lsc-canfranc.es</t>
-  </si>
-  <si>
     <t>LastActiveDate</t>
   </si>
   <si>
-    <t>https://orcid.org/0000-0002-1327-0726</t>
-  </si>
-  <si>
     <t>https://orcid.org/0000-0003-1772-2598</t>
   </si>
   <si>
     <t>https://orcid.org/0000-0001-6938-8259</t>
   </si>
   <si>
-    <t>https://orcid.org/0000-0002-0373-4662</t>
-  </si>
-  <si>
     <t>https://orcid.org/0000-0002-7624-5827</t>
   </si>
   <si>
@@ -1096,9 +1054,6 @@
     <t>https://orcid.org/0000-0002-0012-9918</t>
   </si>
   <si>
-    <t>https://orcid.org/0000-0002-3773-5954</t>
-  </si>
-  <si>
     <t>https://orcid.org/0000-0002-2464-5116</t>
   </si>
   <si>
@@ -1108,9 +1063,6 @@
     <t>https://orcid.org/0009-0001-7036-6476</t>
   </si>
   <si>
-    <t>https://orcid.org/0000-0002-6469-0667</t>
-  </si>
-  <si>
     <t>https://orcid.org/0000-0002-8566-4804</t>
   </si>
   <si>
@@ -1129,9 +1081,6 @@
     <t>https://orcid.org/0000-0002-0155-5812</t>
   </si>
   <si>
-    <t>https://orcid.org/0000-0001-5426-8115</t>
-  </si>
-  <si>
     <t>https://orcid.org/0000-0002-1387-2161</t>
   </si>
   <si>
@@ -1457,6 +1406,15 @@
   </si>
   <si>
     <t>luismiguel.villarpadruno@postgrad.manchester.ac.uk</t>
+  </si>
+  <si>
+    <t>31/03/26</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0009-0002-2780-2399</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0009-0002-5335-0891</t>
   </si>
 </sst>
 </file>
@@ -1955,11 +1913,12 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="42" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2316,7 +2275,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="6" width="20.83203125" customWidth="1"/>
@@ -2336,13 +2295,13 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="F1" t="s">
-        <v>447</v>
+        <v>430</v>
       </c>
       <c r="G1" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="H1" t="s">
         <v>4</v>
@@ -2359,260 +2318,258 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>336</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>337</v>
+        <v>307</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="G2" s="2">
-        <v>45478</v>
-      </c>
+        <v>333</v>
+      </c>
+      <c r="G2" s="1"/>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="I2" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>155</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>314</v>
+        <v>204</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>157</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="G5" s="2">
-        <v>45597</v>
+        <v>46174</v>
       </c>
       <c r="H5" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>160</v>
+        <v>27</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" t="s">
-        <v>24</v>
+        <v>289</v>
       </c>
       <c r="I6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>161</v>
+        <v>29</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="I7" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>441</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>169</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>213</v>
+        <v>442</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>351</v>
+        <v>443</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" t="s">
-        <v>296</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>19</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>158</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>352</v>
+        <v>339</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>458</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>459</v>
+        <v>210</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>460</v>
+        <v>340</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" t="s">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="I10" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>324</v>
       </c>
       <c r="B11" t="s">
-        <v>162</v>
+        <v>325</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>215</v>
+        <v>326</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I11" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
+        <v>211</v>
+      </c>
+      <c r="F12" t="s">
+        <v>342</v>
+      </c>
+      <c r="H12" t="s">
         <v>36</v>
       </c>
-      <c r="B12" t="s">
-        <v>163</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="G12" s="2">
-        <v>45718</v>
-      </c>
-      <c r="H12" t="s">
-        <v>10</v>
-      </c>
       <c r="I12" t="s">
-        <v>11</v>
+        <v>18</v>
+      </c>
+      <c r="J12" t="s">
+        <v>290</v>
+      </c>
+      <c r="K12" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>164</v>
+        <v>41</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="I13" t="s">
         <v>18</v>
@@ -2620,745 +2577,739 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>331</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>332</v>
+        <v>160</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>333</v>
+        <v>213</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>346</v>
       </c>
       <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" t="s">
-        <v>218</v>
-      </c>
-      <c r="F15" t="s">
-        <v>357</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="G15" s="1"/>
       <c r="H15" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J15" t="s">
-        <v>297</v>
+        <v>45</v>
       </c>
       <c r="K15" t="s">
-        <v>293</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>341</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>154</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G16" s="2">
-        <v>45714</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
       <c r="H16" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="I16" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>190</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="G17" s="1"/>
+        <v>187</v>
+      </c>
+      <c r="E17" t="s">
+        <v>216</v>
+      </c>
+      <c r="F17" t="s">
+        <v>347</v>
+      </c>
       <c r="H17" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>360</v>
-      </c>
-      <c r="G18" s="1"/>
+        <v>348</v>
+      </c>
+      <c r="G18" s="2">
+        <v>46174</v>
+      </c>
       <c r="H18" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="I18" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>362</v>
+        <v>331</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>221</v>
+        <v>447</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="G19" s="1"/>
+        <v>448</v>
+      </c>
+      <c r="G19" s="2"/>
       <c r="H19" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="I19" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="J19" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="K19" t="s">
-        <v>19</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>50</v>
+        <v>331</v>
       </c>
       <c r="B20" t="s">
-        <v>158</v>
+        <v>444</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
+        <v>445</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="G20" s="2"/>
       <c r="H20" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="I20" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>195</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>192</v>
-      </c>
-      <c r="E21" t="s">
-        <v>223</v>
-      </c>
-      <c r="F21" t="s">
-        <v>363</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="C21" t="s">
+        <v>292</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="G21" s="1"/>
       <c r="H21" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I21" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>301</v>
       </c>
       <c r="B22" t="s">
-        <v>166</v>
+        <v>8</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>224</v>
+        <v>304</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="G22" s="1"/>
       <c r="H22" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="I22" t="s">
-        <v>28</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>340</v>
+        <v>55</v>
       </c>
       <c r="B23" t="s">
         <v>56</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>343</v>
+        <v>219</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="G23" s="2">
-        <v>45714</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G23" s="1"/>
       <c r="H23" t="s">
-        <v>42</v>
+        <v>289</v>
       </c>
       <c r="I23" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>340</v>
+        <v>294</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>464</v>
+        <v>295</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="G24" s="2"/>
+        <v>352</v>
+      </c>
+      <c r="G24" s="1"/>
       <c r="H24" t="s">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="I24" t="s">
-        <v>54</v>
-      </c>
-      <c r="J24" t="s">
-        <v>63</v>
-      </c>
-      <c r="K24" t="s">
-        <v>90</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>340</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>461</v>
+        <v>58</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>462</v>
+        <v>220</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="G25" s="2"/>
+        <v>353</v>
+      </c>
+      <c r="G25" s="1"/>
       <c r="H25" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="I25" t="s">
-        <v>90</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>322</v>
       </c>
       <c r="B26" t="s">
-        <v>157</v>
-      </c>
-      <c r="C26" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>225</v>
+        <v>323</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="G26" s="1"/>
+        <v>354</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>458</v>
+      </c>
       <c r="H26" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="I26" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>308</v>
+        <v>355</v>
       </c>
       <c r="B27" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>367</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="I27" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>226</v>
+        <v>35</v>
+      </c>
+      <c r="E28" t="s">
+        <v>222</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="G28" s="1"/>
+        <v>434</v>
+      </c>
       <c r="H28" t="s">
-        <v>296</v>
+        <v>36</v>
       </c>
       <c r="I28" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="J28" t="s">
+        <v>290</v>
+      </c>
+      <c r="K28" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>301</v>
+        <v>61</v>
       </c>
       <c r="B29" t="s">
-        <v>82</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="G29" s="1"/>
+        <v>163</v>
+      </c>
+      <c r="E29" t="s">
+        <v>223</v>
+      </c>
+      <c r="F29" t="s">
+        <v>356</v>
+      </c>
       <c r="H29" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I29" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>163</v>
+      </c>
+      <c r="C30" t="s">
+        <v>317</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="G30" s="1"/>
+        <v>357</v>
+      </c>
+      <c r="G30" s="2">
+        <v>45779</v>
+      </c>
       <c r="H30" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="I30" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>329</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
-        <v>305</v>
+        <v>164</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>330</v>
+        <v>313</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="G31" s="1"/>
       <c r="H31" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="I31" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>372</v>
+        <v>66</v>
       </c>
       <c r="B32" t="s">
-        <v>9</v>
+        <v>165</v>
+      </c>
+      <c r="C32" t="s">
+        <v>318</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
+        <v>225</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="G32" s="2">
+        <v>45496</v>
+      </c>
       <c r="H32" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I32" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="J32" t="s">
+        <v>67</v>
+      </c>
+      <c r="K32" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B33" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="E33" t="s">
-        <v>229</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>451</v>
+        <v>226</v>
+      </c>
+      <c r="F33" t="s">
+        <v>360</v>
       </c>
       <c r="H33" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="I33" t="s">
-        <v>19</v>
-      </c>
-      <c r="J33" t="s">
-        <v>297</v>
-      </c>
-      <c r="K33" t="s">
-        <v>293</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B34" t="s">
-        <v>168</v>
+        <v>74</v>
       </c>
       <c r="E34" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F34" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="H34" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I34" t="s">
         <v>18</v>
       </c>
+      <c r="J34" t="s">
+        <v>67</v>
+      </c>
+      <c r="K34" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>66</v>
+        <v>201</v>
       </c>
       <c r="B35" t="s">
-        <v>168</v>
-      </c>
-      <c r="C35" t="s">
-        <v>324</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="G35" s="2">
-        <v>45779</v>
+        <v>113</v>
+      </c>
+      <c r="E35" t="s">
+        <v>228</v>
+      </c>
+      <c r="F35" t="s">
+        <v>362</v>
       </c>
       <c r="H35" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="I35" t="s">
-        <v>67</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" t="s">
+        <v>77</v>
+      </c>
+      <c r="E36" t="s">
+        <v>229</v>
+      </c>
+      <c r="F36" t="s">
+        <v>363</v>
+      </c>
+      <c r="H36" t="s">
+        <v>36</v>
+      </c>
+      <c r="I36" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" t="s">
+        <v>67</v>
+      </c>
+      <c r="K36" t="s">
         <v>68</v>
-      </c>
-      <c r="B36" t="s">
-        <v>169</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>375</v>
-      </c>
-      <c r="G36" s="1"/>
-      <c r="H36" t="s">
-        <v>69</v>
-      </c>
-      <c r="I36" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="B37" t="s">
-        <v>170</v>
-      </c>
-      <c r="C37" t="s">
-        <v>325</v>
+        <v>191</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="G37" s="2">
-        <v>45496</v>
-      </c>
+        <v>364</v>
+      </c>
+      <c r="G37" s="1"/>
       <c r="H37" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="I37" t="s">
-        <v>19</v>
-      </c>
-      <c r="J37" t="s">
-        <v>71</v>
-      </c>
-      <c r="K37" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
-      </c>
-      <c r="E38" t="s">
-        <v>233</v>
-      </c>
-      <c r="F38" t="s">
-        <v>377</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="G38" s="1"/>
       <c r="H38" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="I38" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B39" t="s">
-        <v>78</v>
-      </c>
-      <c r="E39" t="s">
-        <v>234</v>
-      </c>
-      <c r="F39" t="s">
-        <v>378</v>
-      </c>
+        <v>162</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="G39" s="1"/>
       <c r="H39" t="s">
-        <v>22</v>
+        <v>82</v>
       </c>
       <c r="I39" t="s">
-        <v>19</v>
-      </c>
-      <c r="J39" t="s">
-        <v>71</v>
-      </c>
-      <c r="K39" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>206</v>
+        <v>84</v>
       </c>
       <c r="B40" t="s">
-        <v>117</v>
-      </c>
-      <c r="E40" t="s">
-        <v>235</v>
-      </c>
-      <c r="F40" t="s">
-        <v>379</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="G40" s="1"/>
       <c r="H40" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="I40" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B41" t="s">
-        <v>80</v>
-      </c>
-      <c r="C41" t="s">
-        <v>81</v>
-      </c>
-      <c r="E41" t="s">
-        <v>236</v>
-      </c>
-      <c r="F41" t="s">
-        <v>380</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="G41" s="1"/>
       <c r="H41" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="I41" t="s">
-        <v>19</v>
-      </c>
-      <c r="J41" t="s">
-        <v>71</v>
-      </c>
-      <c r="K41" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s">
-        <v>196</v>
+        <v>95</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>237</v>
+        <v>282</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" t="s">
-        <v>14</v>
+        <v>284</v>
       </c>
       <c r="I42" t="s">
-        <v>15</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B43" t="s">
         <v>168</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I43" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B44" t="s">
-        <v>167</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="G44" s="1"/>
+        <v>8</v>
+      </c>
+      <c r="E44" t="s">
+        <v>234</v>
+      </c>
+      <c r="F44" t="s">
+        <v>371</v>
+      </c>
       <c r="H44" t="s">
+        <v>59</v>
+      </c>
+      <c r="I44" t="s">
         <v>86</v>
-      </c>
-      <c r="I44" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B45" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>321</v>
+        <v>235</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="I45" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>436</v>
       </c>
       <c r="B46" t="s">
-        <v>172</v>
+        <v>437</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>288</v>
+        <v>438</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>385</v>
+        <v>439</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="I46" t="s">
-        <v>90</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
@@ -3366,378 +3317,379 @@
         <v>91</v>
       </c>
       <c r="B47" t="s">
-        <v>99</v>
+        <v>170</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="G47" s="1"/>
+        <v>440</v>
+      </c>
+      <c r="F47" t="s">
+        <v>373</v>
+      </c>
       <c r="H47" t="s">
-        <v>291</v>
+        <v>47</v>
       </c>
       <c r="I47" t="s">
-        <v>292</v>
+        <v>48</v>
+      </c>
+      <c r="J47" t="s">
+        <v>13</v>
+      </c>
+      <c r="K47" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>92</v>
+        <v>196</v>
       </c>
       <c r="B48" t="s">
-        <v>173</v>
+        <v>27</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="G48" s="1"/>
       <c r="H48" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="I48" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>92</v>
+      </c>
+      <c r="B49" t="s">
+        <v>52</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="G49" s="1"/>
+      <c r="H49" t="s">
+        <v>36</v>
+      </c>
+      <c r="I49" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>93</v>
       </c>
-      <c r="B49" t="s">
-        <v>9</v>
-      </c>
-      <c r="E49" t="s">
-        <v>241</v>
-      </c>
-      <c r="F49" t="s">
-        <v>388</v>
-      </c>
-      <c r="H49" t="s">
-        <v>63</v>
-      </c>
-      <c r="I49" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>94</v>
-      </c>
       <c r="B50" t="s">
-        <v>174</v>
+        <v>37</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" t="s">
-        <v>24</v>
+        <v>289</v>
       </c>
       <c r="I50" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>453</v>
+        <v>94</v>
       </c>
       <c r="B51" t="s">
-        <v>454</v>
+        <v>95</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>455</v>
+        <v>239</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>456</v>
+        <v>377</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
       <c r="I51" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B52" t="s">
-        <v>175</v>
+        <v>27</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="F52" t="s">
-        <v>390</v>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="G52" s="1"/>
       <c r="H52" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="I52" t="s">
-        <v>52</v>
-      </c>
-      <c r="J52" t="s">
-        <v>14</v>
-      </c>
-      <c r="K52" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>201</v>
+        <v>99</v>
       </c>
       <c r="B53" t="s">
-        <v>30</v>
+        <v>172</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I53" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B54" t="s">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="G54" s="1"/>
       <c r="H54" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="I54" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>173</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="G55" s="1"/>
       <c r="H55" t="s">
-        <v>296</v>
+        <v>65</v>
       </c>
       <c r="I55" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>98</v>
+        <v>312</v>
       </c>
       <c r="B56" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>246</v>
+        <v>321</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="G56" s="1"/>
       <c r="H56" t="s">
-        <v>100</v>
+        <v>289</v>
       </c>
       <c r="I56" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>102</v>
       </c>
       <c r="B57" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="G57" s="1"/>
       <c r="H57" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I57" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B58" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I58" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>104</v>
+        <v>305</v>
       </c>
       <c r="B59" t="s">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>249</v>
+        <v>306</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="G59" s="1"/>
       <c r="H59" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I59" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B60" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="G60" s="1"/>
       <c r="H60" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="I60" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>319</v>
+        <v>107</v>
       </c>
       <c r="B61" t="s">
-        <v>41</v>
+        <v>176</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>328</v>
+        <v>452</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="G61" s="1"/>
       <c r="H61" t="s">
-        <v>296</v>
+        <v>49</v>
       </c>
       <c r="I61" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B62" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="G62" s="1"/>
       <c r="H62" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="I62" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B63" t="s">
-        <v>179</v>
+        <v>111</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I63" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>312</v>
+        <v>112</v>
       </c>
       <c r="B64" t="s">
-        <v>41</v>
+        <v>113</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>313</v>
+        <v>249</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
       <c r="G64" s="1"/>
       <c r="H64" t="s">
-        <v>17</v>
+        <v>289</v>
       </c>
       <c r="I64" t="s">
         <v>18</v>
@@ -3745,41 +3697,47 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B65" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="I65" t="s">
-        <v>25</v>
+        <v>18</v>
+      </c>
+      <c r="J65" t="s">
+        <v>67</v>
+      </c>
+      <c r="K65" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B66" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>469</v>
+        <v>251</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="G66" s="1"/>
       <c r="H66" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="I66" t="s">
         <v>54</v>
@@ -3787,155 +3745,149 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B67" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="G67" s="1"/>
       <c r="H67" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I67" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B68" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
       <c r="G68" s="1"/>
       <c r="H68" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I68" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B69" t="s">
-        <v>117</v>
+        <v>180</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>407</v>
+        <v>394</v>
       </c>
       <c r="G69" s="1"/>
       <c r="H69" t="s">
-        <v>296</v>
+        <v>49</v>
       </c>
       <c r="I69" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B70" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>408</v>
+        <v>395</v>
       </c>
       <c r="G70" s="1"/>
       <c r="H70" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="I70" t="s">
-        <v>19</v>
-      </c>
-      <c r="J70" t="s">
-        <v>71</v>
-      </c>
-      <c r="K70" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B71" t="s">
-        <v>183</v>
+        <v>58</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
       <c r="G71" s="1"/>
       <c r="H71" t="s">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="I71" t="s">
-        <v>58</v>
+        <v>18</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>120</v>
+        <v>453</v>
       </c>
       <c r="B72" t="s">
-        <v>184</v>
+        <v>126</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>259</v>
+        <v>454</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>410</v>
+        <v>459</v>
       </c>
       <c r="G72" s="1"/>
       <c r="H72" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="I72" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B73" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>450</v>
+        <v>397</v>
       </c>
       <c r="G73" s="1"/>
       <c r="H73" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="I73" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
@@ -3943,20 +3895,20 @@
         <v>123</v>
       </c>
       <c r="B74" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>411</v>
+        <v>398</v>
       </c>
       <c r="G74" s="1"/>
       <c r="H74" t="s">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="I74" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
@@ -3964,20 +3916,18 @@
         <v>124</v>
       </c>
       <c r="B75" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>412</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="F75" s="1"/>
       <c r="G75" s="1"/>
       <c r="H75" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="I75" t="s">
-        <v>52</v>
+        <v>97</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
@@ -3985,463 +3935,471 @@
         <v>125</v>
       </c>
       <c r="B76" t="s">
-        <v>62</v>
+        <v>126</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="G76" s="1"/>
       <c r="H76" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="I76" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>470</v>
+        <v>195</v>
       </c>
       <c r="B77" t="s">
-        <v>130</v>
+        <v>37</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="F77" s="1"/>
+        <v>261</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>400</v>
+      </c>
       <c r="G77" s="1"/>
       <c r="H77" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="I77" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B78" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>414</v>
+        <v>401</v>
       </c>
       <c r="G78" s="1"/>
       <c r="H78" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I78" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B79" t="s">
-        <v>187</v>
+        <v>35</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>415</v>
+        <v>402</v>
       </c>
       <c r="G79" s="1"/>
       <c r="H79" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="I79" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B80" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F80" s="1"/>
+        <v>264</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>403</v>
+      </c>
       <c r="G80" s="1"/>
       <c r="H80" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="I80" t="s">
-        <v>101</v>
+        <v>50</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B81" t="s">
-        <v>130</v>
+        <v>174</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>267</v>
+        <v>296</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="G81" s="1"/>
       <c r="H81" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I81" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>200</v>
+        <v>131</v>
       </c>
       <c r="B82" t="s">
-        <v>41</v>
+        <v>126</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="G82" s="1"/>
       <c r="H82" t="s">
-        <v>22</v>
+        <v>289</v>
       </c>
       <c r="I82" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="J82" t="s">
+        <v>36</v>
+      </c>
+      <c r="K82" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B83" t="s">
-        <v>117</v>
+        <v>8</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
       <c r="G83" s="1"/>
       <c r="H83" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I83" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B84" t="s">
-        <v>39</v>
+        <v>171</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>270</v>
+        <v>311</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="G84" s="1"/>
+        <v>407</v>
+      </c>
+      <c r="G84" s="2">
+        <v>45718</v>
+      </c>
       <c r="H84" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
       <c r="I84" t="s">
-        <v>90</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B85" t="s">
-        <v>181</v>
+        <v>182</v>
+      </c>
+      <c r="C85" t="s">
+        <v>293</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="G85" s="1"/>
+        <v>408</v>
+      </c>
+      <c r="G85" s="2">
+        <v>45779</v>
+      </c>
       <c r="H85" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="I85" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="K85" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B86" t="s">
-        <v>179</v>
+        <v>184</v>
+      </c>
+      <c r="C86" t="s">
+        <v>291</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="G86" s="1"/>
+        <v>409</v>
+      </c>
+      <c r="G86" s="2">
+        <v>45779</v>
+      </c>
       <c r="H86" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I86" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>135</v>
+        <v>328</v>
       </c>
       <c r="B87" t="s">
-        <v>130</v>
+        <v>58</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>272</v>
+        <v>319</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="G87" s="1"/>
       <c r="H87" t="s">
-        <v>296</v>
+        <v>38</v>
       </c>
       <c r="I87" t="s">
-        <v>19</v>
-      </c>
-      <c r="J87" t="s">
-        <v>40</v>
-      </c>
-      <c r="K87" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>136</v>
+        <v>297</v>
       </c>
       <c r="B88" t="s">
-        <v>9</v>
+        <v>298</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="G88" s="1"/>
       <c r="H88" t="s">
         <v>49</v>
       </c>
       <c r="I88" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B89" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="G89" s="2">
-        <v>45718</v>
-      </c>
+        <v>411</v>
+      </c>
+      <c r="G89" s="1"/>
       <c r="H89" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="I89" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B90" t="s">
-        <v>187</v>
-      </c>
-      <c r="C90" t="s">
-        <v>300</v>
+        <v>186</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>274</v>
+        <v>315</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="G90" s="2">
-        <v>45779</v>
-      </c>
+        <v>412</v>
+      </c>
+      <c r="G90" s="1"/>
       <c r="H90" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="I90" t="s">
-        <v>19</v>
-      </c>
-      <c r="K90" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>139</v>
+        <v>192</v>
       </c>
       <c r="B91" t="s">
-        <v>189</v>
-      </c>
-      <c r="C91" t="s">
-        <v>298</v>
+        <v>35</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>317</v>
+        <v>268</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="G91" s="2">
-        <v>45779</v>
-      </c>
+        <v>413</v>
+      </c>
+      <c r="G91" s="1"/>
       <c r="H91" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="I91" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="J91" t="s">
+        <v>290</v>
+      </c>
+      <c r="K91" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>335</v>
+        <v>137</v>
       </c>
       <c r="B92" t="s">
-        <v>62</v>
+        <v>126</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>326</v>
+        <v>269</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>427</v>
+        <v>414</v>
       </c>
       <c r="G92" s="1"/>
       <c r="H92" t="s">
-        <v>42</v>
+        <v>284</v>
       </c>
       <c r="I92" t="s">
-        <v>43</v>
+        <v>285</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>304</v>
+        <v>198</v>
       </c>
       <c r="B93" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>309</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>448</v>
+        <v>435</v>
       </c>
       <c r="G93" s="1"/>
       <c r="H93" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="I93" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>140</v>
+        <v>198</v>
       </c>
       <c r="B94" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="F94" s="1" t="s">
-        <v>428</v>
-      </c>
+        <v>316</v>
+      </c>
+      <c r="F94" s="1"/>
       <c r="G94" s="1"/>
       <c r="H94" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="I94" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B95" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>429</v>
+        <v>415</v>
       </c>
       <c r="G95" s="1"/>
       <c r="H95" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="I95" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>197</v>
+        <v>139</v>
       </c>
       <c r="B96" t="s">
-        <v>39</v>
+        <v>140</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>430</v>
+        <v>416</v>
       </c>
       <c r="G96" s="1"/>
       <c r="H96" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I96" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J96" t="s">
-        <v>297</v>
+        <v>67</v>
       </c>
       <c r="K96" t="s">
-        <v>293</v>
+        <v>68</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
@@ -4449,253 +4407,265 @@
         <v>141</v>
       </c>
       <c r="B97" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>431</v>
+        <v>417</v>
       </c>
       <c r="G97" s="1"/>
       <c r="H97" t="s">
-        <v>291</v>
+        <v>49</v>
       </c>
       <c r="I97" t="s">
-        <v>292</v>
+        <v>50</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>203</v>
+        <v>142</v>
       </c>
       <c r="B98" t="s">
-        <v>315</v>
+        <v>113</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>316</v>
+        <v>283</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>452</v>
+        <v>418</v>
       </c>
       <c r="G98" s="1"/>
       <c r="H98" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="I98" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>203</v>
+        <v>143</v>
       </c>
       <c r="B99" t="s">
-        <v>204</v>
+        <v>144</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>323</v>
+        <v>271</v>
       </c>
       <c r="F99" s="1"/>
       <c r="G99" s="1"/>
       <c r="H99" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="I99" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>142</v>
+        <v>200</v>
       </c>
       <c r="B100" t="s">
-        <v>192</v>
+        <v>29</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>327</v>
+        <v>272</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>432</v>
+        <v>419</v>
       </c>
       <c r="G100" s="1"/>
       <c r="H100" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I100" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B101" t="s">
-        <v>144</v>
+        <v>188</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>433</v>
+        <v>420</v>
       </c>
       <c r="G101" s="1"/>
       <c r="H101" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="I101" t="s">
-        <v>19</v>
-      </c>
-      <c r="J101" t="s">
-        <v>71</v>
-      </c>
-      <c r="K101" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>145</v>
+        <v>197</v>
       </c>
       <c r="B102" t="s">
-        <v>181</v>
+        <v>8</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>434</v>
+        <v>421</v>
       </c>
       <c r="G102" s="1"/>
       <c r="H102" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="I102" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>146</v>
+        <v>287</v>
       </c>
       <c r="B103" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>435</v>
+        <v>422</v>
       </c>
       <c r="G103" s="1"/>
       <c r="H103" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="I103" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B104" t="s">
-        <v>148</v>
+        <v>174</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="F104" s="1"/>
+        <v>275</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>423</v>
+      </c>
       <c r="G104" s="1"/>
       <c r="H104" t="s">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="I104" t="s">
-        <v>58</v>
+        <v>18</v>
+      </c>
+      <c r="J104" t="s">
+        <v>147</v>
+      </c>
+      <c r="K104" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>205</v>
+        <v>149</v>
       </c>
       <c r="B105" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>279</v>
+        <v>432</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
       <c r="G105" s="1"/>
       <c r="H105" t="s">
-        <v>53</v>
+        <v>13</v>
       </c>
       <c r="I105" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>149</v>
+        <v>193</v>
       </c>
       <c r="B106" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="F106" s="1" t="s">
-        <v>437</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="F106" s="1"/>
       <c r="G106" s="1"/>
       <c r="H106" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="I106" t="s">
         <v>18</v>
       </c>
+      <c r="J106" t="s">
+        <v>19</v>
+      </c>
+      <c r="K106" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>202</v>
+        <v>329</v>
       </c>
       <c r="B107" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>281</v>
+        <v>330</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>438</v>
+        <v>425</v>
       </c>
       <c r="G107" s="1"/>
       <c r="H107" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="I107" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>294</v>
+        <v>449</v>
       </c>
       <c r="B108" t="s">
-        <v>32</v>
+        <v>298</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>295</v>
+        <v>450</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>439</v>
+        <v>451</v>
       </c>
       <c r="G108" s="1"/>
       <c r="H108" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I108" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="J108" t="s">
+        <v>59</v>
+      </c>
+      <c r="K108" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.2">
@@ -4703,351 +4673,228 @@
         <v>150</v>
       </c>
       <c r="B109" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>440</v>
+        <v>426</v>
       </c>
       <c r="G109" s="1"/>
       <c r="H109" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="I109" t="s">
-        <v>19</v>
-      </c>
-      <c r="J109" t="s">
-        <v>151</v>
-      </c>
-      <c r="K109" t="s">
-        <v>152</v>
+        <v>69</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>153</v>
+        <v>299</v>
       </c>
       <c r="B110" t="s">
-        <v>41</v>
+        <v>300</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>449</v>
+        <v>303</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>441</v>
+        <v>427</v>
       </c>
       <c r="G110" s="1"/>
       <c r="H110" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="I110" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>198</v>
+      <c r="A111" s="3" t="s">
+        <v>455</v>
       </c>
       <c r="B111" t="s">
-        <v>199</v>
+        <v>456</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="F111" s="1"/>
+        <v>457</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>460</v>
+      </c>
       <c r="G111" s="1"/>
       <c r="H111" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="I111" t="s">
-        <v>19</v>
-      </c>
-      <c r="J111" t="s">
-        <v>22</v>
-      </c>
-      <c r="K111" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>338</v>
+        <v>151</v>
       </c>
       <c r="B112" t="s">
-        <v>39</v>
+        <v>152</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>339</v>
+        <v>278</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>442</v>
+        <v>428</v>
       </c>
       <c r="G112" s="1"/>
       <c r="H112" t="s">
-        <v>76</v>
+        <v>13</v>
       </c>
       <c r="I112" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>466</v>
+        <v>202</v>
       </c>
       <c r="B113" t="s">
-        <v>305</v>
+        <v>37</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>467</v>
+        <v>279</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>468</v>
+        <v>429</v>
       </c>
       <c r="G113" s="1"/>
       <c r="H113" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="I113" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J113" t="s">
-        <v>63</v>
+        <v>290</v>
       </c>
       <c r="K113" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>154</v>
-      </c>
-      <c r="B114" t="s">
-        <v>194</v>
-      </c>
-      <c r="E114" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="G114" s="1"/>
-      <c r="H114" t="s">
-        <v>34</v>
-      </c>
-      <c r="I114" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>306</v>
-      </c>
-      <c r="B115" t="s">
-        <v>307</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>444</v>
-      </c>
-      <c r="G115" s="1"/>
-      <c r="H115" t="s">
-        <v>53</v>
-      </c>
-      <c r="I115" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A116" s="3" t="s">
-        <v>472</v>
-      </c>
-      <c r="B116" t="s">
-        <v>473</v>
-      </c>
-      <c r="E116" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="F116" s="1"/>
-      <c r="G116" s="1"/>
-      <c r="H116" t="s">
-        <v>14</v>
-      </c>
-      <c r="I116" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
-        <v>155</v>
-      </c>
-      <c r="B117" t="s">
-        <v>156</v>
-      </c>
-      <c r="E117" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="F117" s="1" t="s">
-        <v>445</v>
-      </c>
-      <c r="G117" s="1"/>
-      <c r="H117" t="s">
-        <v>14</v>
-      </c>
-      <c r="I117" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
-        <v>207</v>
-      </c>
-      <c r="B118" t="s">
-        <v>41</v>
-      </c>
-      <c r="E118" s="1" t="s">
         <v>286</v>
-      </c>
-      <c r="F118" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="G118" s="1"/>
-      <c r="H118" t="s">
-        <v>40</v>
-      </c>
-      <c r="I118" t="s">
-        <v>19</v>
-      </c>
-      <c r="J118" t="s">
-        <v>297</v>
-      </c>
-      <c r="K118" t="s">
-        <v>293</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{0FF3DA65-AAFE-A544-B83F-3B8DBBA655D2}"/>
-    <hyperlink ref="E6" r:id="rId2" xr:uid="{D72FCA14-EA08-4749-BB11-D24B8A62C2FD}"/>
-    <hyperlink ref="E9" r:id="rId3" xr:uid="{E6DBC748-9C42-444A-9719-EDB7AD21ED31}"/>
-    <hyperlink ref="E11" r:id="rId4" xr:uid="{D72F2EFB-3573-5D41-9B63-CA5C8A903FE7}"/>
-    <hyperlink ref="E17" r:id="rId5" xr:uid="{7BA53910-2895-8546-8C78-4ADAECEB1354}"/>
-    <hyperlink ref="E18" r:id="rId6" xr:uid="{5B370D66-5FA2-8A4A-A92C-48946FC643B8}"/>
-    <hyperlink ref="E19" r:id="rId7" xr:uid="{E1E20BC8-2BB4-C34E-8CA8-2ED92BB0838B}"/>
-    <hyperlink ref="E20" r:id="rId8" xr:uid="{77E75D5E-F948-2248-A233-77176542B4F7}"/>
-    <hyperlink ref="E26" r:id="rId9" xr:uid="{D9028AA5-E4C8-9E40-BF28-A681BB8D6B4F}"/>
-    <hyperlink ref="E30" r:id="rId10" xr:uid="{221B0995-0A38-FC4A-A9DC-9EFA0954E180}"/>
-    <hyperlink ref="E32" r:id="rId11" xr:uid="{2B53C67F-39F7-4A49-99C5-3CED9DB96DF6}"/>
-    <hyperlink ref="E35" r:id="rId12" xr:uid="{B022962F-480B-E242-A4EB-4B4743EC7105}"/>
-    <hyperlink ref="E37" r:id="rId13" xr:uid="{3503F030-FF3A-A74C-AECE-58009DA1DD3E}"/>
-    <hyperlink ref="E42" r:id="rId14" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
-    <hyperlink ref="E43" r:id="rId15" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
-    <hyperlink ref="E44" r:id="rId16" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
-    <hyperlink ref="E45" r:id="rId17" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
-    <hyperlink ref="E46" r:id="rId18" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
-    <hyperlink ref="E47" r:id="rId19" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
-    <hyperlink ref="E48" r:id="rId20" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
-    <hyperlink ref="E50" r:id="rId21" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
-    <hyperlink ref="E53" r:id="rId22" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
-    <hyperlink ref="E54" r:id="rId23" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
-    <hyperlink ref="E56" r:id="rId24" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
-    <hyperlink ref="E60" r:id="rId25" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
-    <hyperlink ref="E67" r:id="rId26" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
-    <hyperlink ref="E63" r:id="rId27" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
-    <hyperlink ref="E68" r:id="rId28" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
-    <hyperlink ref="E70" r:id="rId29" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
-    <hyperlink ref="E72" r:id="rId30" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
-    <hyperlink ref="E73" r:id="rId31" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
-    <hyperlink ref="E3" r:id="rId32" xr:uid="{3A3CFB2D-9550-DB47-876D-1CF2172ED36B}"/>
-    <hyperlink ref="E65" r:id="rId33" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
-    <hyperlink ref="E74" r:id="rId34" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
-    <hyperlink ref="E75" r:id="rId35" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
-    <hyperlink ref="E28" r:id="rId36" xr:uid="{403F5279-8F67-B64C-A27C-18563FED25F5}"/>
-    <hyperlink ref="E76" r:id="rId37" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
-    <hyperlink ref="E78" r:id="rId38" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
-    <hyperlink ref="E79" r:id="rId39" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
-    <hyperlink ref="E80" r:id="rId40" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
-    <hyperlink ref="E81" r:id="rId41" xr:uid="{C651F08A-4556-B04E-BEC5-BBBA98A040F7}"/>
-    <hyperlink ref="E82" r:id="rId42" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
-    <hyperlink ref="E83" r:id="rId43" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
-    <hyperlink ref="E85" r:id="rId44" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
-    <hyperlink ref="E87" r:id="rId45" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
-    <hyperlink ref="E88" r:id="rId46" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
-    <hyperlink ref="E89" r:id="rId47" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
-    <hyperlink ref="E90" r:id="rId48" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
-    <hyperlink ref="E94" r:id="rId49" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
-    <hyperlink ref="E96" r:id="rId50" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
-    <hyperlink ref="E101" r:id="rId51" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
-    <hyperlink ref="E103" r:id="rId52" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
-    <hyperlink ref="E104" r:id="rId53" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
-    <hyperlink ref="E105" r:id="rId54" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
-    <hyperlink ref="E106" r:id="rId55" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
-    <hyperlink ref="E107" r:id="rId56" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
-    <hyperlink ref="E109" r:id="rId57" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
-    <hyperlink ref="E110" r:id="rId58" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
-    <hyperlink ref="E114" r:id="rId59" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
-    <hyperlink ref="E117" r:id="rId60" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
-    <hyperlink ref="E118" r:id="rId61" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
-    <hyperlink ref="E59" r:id="rId62" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
-    <hyperlink ref="E71" r:id="rId63" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
-    <hyperlink ref="E95" r:id="rId64" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
-    <hyperlink ref="E102" r:id="rId65" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
-    <hyperlink ref="E5" r:id="rId66" xr:uid="{F868C6CA-568C-E347-BF39-833BED9A84ED}"/>
-    <hyperlink ref="E13" r:id="rId67" xr:uid="{464857C2-993C-4144-9F79-68780529C7BD}"/>
-    <hyperlink ref="E62" r:id="rId68" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
-    <hyperlink ref="E7" r:id="rId69" display="mailto:isaac.arnquist@pnnl.gov" xr:uid="{308E6526-5B60-F34F-A8F5-559BEC15710C}"/>
-    <hyperlink ref="E12" r:id="rId70" display="mailto:kevin_bailey@anl.gov" xr:uid="{C7A6318C-B3D3-A24F-A8E4-7E9174A7398D}"/>
-    <hyperlink ref="E57" r:id="rId71" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
-    <hyperlink ref="E58" r:id="rId72" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
-    <hyperlink ref="E8" r:id="rId73" xr:uid="{2D0C47D7-E74D-EA48-8223-B97B97694F84}"/>
-    <hyperlink ref="E55" r:id="rId74" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
-    <hyperlink ref="E69" r:id="rId75" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
-    <hyperlink ref="E97" r:id="rId76" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
-    <hyperlink ref="E111" r:id="rId77" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
-    <hyperlink ref="E84" r:id="rId78" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
-    <hyperlink ref="E4" r:id="rId79" xr:uid="{1407FD31-5939-8E40-B9DC-A0AC164EEEA9}"/>
-    <hyperlink ref="E108" r:id="rId80" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
-    <hyperlink ref="E29" r:id="rId81" xr:uid="{A1BB8086-1232-764F-9321-DBAFA8F4E6BC}"/>
-    <hyperlink ref="E86" r:id="rId82" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
-    <hyperlink ref="E93" r:id="rId83" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
-    <hyperlink ref="E115" r:id="rId84" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
-    <hyperlink ref="E27" r:id="rId85" xr:uid="{D75012BC-D5E3-6D46-B329-96A4CB35BA96}"/>
-    <hyperlink ref="E64" r:id="rId86" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
-    <hyperlink ref="E98" r:id="rId87" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
-    <hyperlink ref="E91" r:id="rId88" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
-    <hyperlink ref="E36" r:id="rId89" xr:uid="{137601BF-06D1-F948-9D79-A5FEE0032F25}"/>
-    <hyperlink ref="E99" r:id="rId90" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
-    <hyperlink ref="E92" r:id="rId91" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
-    <hyperlink ref="E100" r:id="rId92" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
-    <hyperlink ref="E61" r:id="rId93" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
-    <hyperlink ref="E31" r:id="rId94" xr:uid="{E24B841F-2272-CA43-9614-50B7F36AD8C5}"/>
-    <hyperlink ref="E14" r:id="rId95" xr:uid="{29460556-99EB-6943-BF02-EAF45B9A2438}"/>
-    <hyperlink ref="E112" r:id="rId96" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
-    <hyperlink ref="E22" r:id="rId97" xr:uid="{BFCD233B-85C4-684A-9E1F-CFD7E946453F}"/>
-    <hyperlink ref="E16" r:id="rId98" tooltip="abayo@lsc-canfranc.es" display="mailto:abayo@lsc-canfranc.es" xr:uid="{9D231E2D-796B-5044-A575-DB475A1F4009}"/>
-    <hyperlink ref="E23" r:id="rId99" tooltip="lcid@lsc-canfranc.es" display="mailto:lcid@lsc-canfranc.es" xr:uid="{2505E3E3-5341-1F45-B64F-DF1C414EDC59}"/>
-    <hyperlink ref="F93" r:id="rId100" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
-    <hyperlink ref="F73" r:id="rId101" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
-    <hyperlink ref="F33" r:id="rId102" xr:uid="{232B5F00-F258-A24E-BDEA-CF2F2635A32D}"/>
-    <hyperlink ref="F98" r:id="rId103" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
-    <hyperlink ref="E51" r:id="rId104" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
-    <hyperlink ref="F51" r:id="rId105" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
-    <hyperlink ref="E52" r:id="rId106" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
-    <hyperlink ref="E10" r:id="rId107" xr:uid="{E4C80A26-9BBE-CE4E-A398-4F9C5F4955F3}"/>
-    <hyperlink ref="F10" r:id="rId108" xr:uid="{5914BE48-1B32-6F46-B075-BC630F5D8608}"/>
-    <hyperlink ref="E25" r:id="rId109" xr:uid="{D5AF8CE0-2466-6647-B572-C377DB7C2F3F}"/>
-    <hyperlink ref="F25" r:id="rId110" xr:uid="{0DDC6C1F-4537-7C4D-A53D-0EA66E740063}"/>
-    <hyperlink ref="E24" r:id="rId111" xr:uid="{7651A9F0-0FB9-AD45-8536-6DA2DBA419D4}"/>
-    <hyperlink ref="F23" r:id="rId112" xr:uid="{EF908708-D656-CC4E-AA5B-142D3510D559}"/>
-    <hyperlink ref="F24" r:id="rId113" xr:uid="{89D30D76-781B-4C4A-9D08-40BF96ECDA97}"/>
-    <hyperlink ref="E113" r:id="rId114" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
-    <hyperlink ref="F113" r:id="rId115" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
-    <hyperlink ref="E66" r:id="rId116" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
-    <hyperlink ref="E77" r:id="rId117" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
-    <hyperlink ref="E116" r:id="rId118" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
+    <hyperlink ref="E4" r:id="rId1" xr:uid="{D72FCA14-EA08-4749-BB11-D24B8A62C2FD}"/>
+    <hyperlink ref="E7" r:id="rId2" xr:uid="{E6DBC748-9C42-444A-9719-EDB7AD21ED31}"/>
+    <hyperlink ref="E9" r:id="rId3" xr:uid="{D72F2EFB-3573-5D41-9B63-CA5C8A903FE7}"/>
+    <hyperlink ref="E13" r:id="rId4" xr:uid="{7BA53910-2895-8546-8C78-4ADAECEB1354}"/>
+    <hyperlink ref="E14" r:id="rId5" xr:uid="{5B370D66-5FA2-8A4A-A92C-48946FC643B8}"/>
+    <hyperlink ref="E15" r:id="rId6" xr:uid="{E1E20BC8-2BB4-C34E-8CA8-2ED92BB0838B}"/>
+    <hyperlink ref="E16" r:id="rId7" xr:uid="{77E75D5E-F948-2248-A233-77176542B4F7}"/>
+    <hyperlink ref="E21" r:id="rId8" xr:uid="{D9028AA5-E4C8-9E40-BF28-A681BB8D6B4F}"/>
+    <hyperlink ref="E25" r:id="rId9" xr:uid="{221B0995-0A38-FC4A-A9DC-9EFA0954E180}"/>
+    <hyperlink ref="E27" r:id="rId10" xr:uid="{2B53C67F-39F7-4A49-99C5-3CED9DB96DF6}"/>
+    <hyperlink ref="E30" r:id="rId11" xr:uid="{B022962F-480B-E242-A4EB-4B4743EC7105}"/>
+    <hyperlink ref="E32" r:id="rId12" xr:uid="{3503F030-FF3A-A74C-AECE-58009DA1DD3E}"/>
+    <hyperlink ref="E37" r:id="rId13" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
+    <hyperlink ref="E38" r:id="rId14" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
+    <hyperlink ref="E39" r:id="rId15" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
+    <hyperlink ref="E40" r:id="rId16" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
+    <hyperlink ref="E41" r:id="rId17" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
+    <hyperlink ref="E42" r:id="rId18" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
+    <hyperlink ref="E43" r:id="rId19" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
+    <hyperlink ref="E45" r:id="rId20" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
+    <hyperlink ref="E48" r:id="rId21" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
+    <hyperlink ref="E49" r:id="rId22" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
+    <hyperlink ref="E51" r:id="rId23" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
+    <hyperlink ref="E55" r:id="rId24" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
+    <hyperlink ref="E62" r:id="rId25" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
+    <hyperlink ref="E58" r:id="rId26" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
+    <hyperlink ref="E63" r:id="rId27" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
+    <hyperlink ref="E65" r:id="rId28" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
+    <hyperlink ref="E67" r:id="rId29" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
+    <hyperlink ref="E68" r:id="rId30" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
+    <hyperlink ref="E2" r:id="rId31" xr:uid="{3A3CFB2D-9550-DB47-876D-1CF2172ED36B}"/>
+    <hyperlink ref="E60" r:id="rId32" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
+    <hyperlink ref="E69" r:id="rId33" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
+    <hyperlink ref="E70" r:id="rId34" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
+    <hyperlink ref="E23" r:id="rId35" xr:uid="{403F5279-8F67-B64C-A27C-18563FED25F5}"/>
+    <hyperlink ref="E71" r:id="rId36" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
+    <hyperlink ref="E73" r:id="rId37" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
+    <hyperlink ref="E74" r:id="rId38" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
+    <hyperlink ref="E75" r:id="rId39" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
+    <hyperlink ref="E76" r:id="rId40" xr:uid="{C651F08A-4556-B04E-BEC5-BBBA98A040F7}"/>
+    <hyperlink ref="E77" r:id="rId41" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
+    <hyperlink ref="E78" r:id="rId42" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
+    <hyperlink ref="E80" r:id="rId43" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
+    <hyperlink ref="E82" r:id="rId44" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
+    <hyperlink ref="E83" r:id="rId45" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
+    <hyperlink ref="E84" r:id="rId46" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
+    <hyperlink ref="E85" r:id="rId47" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
+    <hyperlink ref="E89" r:id="rId48" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
+    <hyperlink ref="E91" r:id="rId49" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
+    <hyperlink ref="E96" r:id="rId50" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
+    <hyperlink ref="E98" r:id="rId51" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
+    <hyperlink ref="E99" r:id="rId52" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
+    <hyperlink ref="E100" r:id="rId53" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
+    <hyperlink ref="E101" r:id="rId54" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
+    <hyperlink ref="E102" r:id="rId55" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
+    <hyperlink ref="E104" r:id="rId56" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
+    <hyperlink ref="E105" r:id="rId57" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
+    <hyperlink ref="E109" r:id="rId58" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
+    <hyperlink ref="E112" r:id="rId59" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
+    <hyperlink ref="E113" r:id="rId60" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
+    <hyperlink ref="E54" r:id="rId61" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
+    <hyperlink ref="E66" r:id="rId62" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
+    <hyperlink ref="E90" r:id="rId63" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
+    <hyperlink ref="E97" r:id="rId64" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
+    <hyperlink ref="E10" r:id="rId65" xr:uid="{464857C2-993C-4144-9F79-68780529C7BD}"/>
+    <hyperlink ref="E57" r:id="rId66" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
+    <hyperlink ref="E5" r:id="rId67" display="mailto:isaac.arnquist@pnnl.gov" xr:uid="{308E6526-5B60-F34F-A8F5-559BEC15710C}"/>
+    <hyperlink ref="E52" r:id="rId68" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
+    <hyperlink ref="E53" r:id="rId69" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
+    <hyperlink ref="E6" r:id="rId70" xr:uid="{2D0C47D7-E74D-EA48-8223-B97B97694F84}"/>
+    <hyperlink ref="E50" r:id="rId71" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
+    <hyperlink ref="E64" r:id="rId72" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
+    <hyperlink ref="E92" r:id="rId73" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
+    <hyperlink ref="E106" r:id="rId74" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
+    <hyperlink ref="E79" r:id="rId75" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
+    <hyperlink ref="E3" r:id="rId76" xr:uid="{1407FD31-5939-8E40-B9DC-A0AC164EEEA9}"/>
+    <hyperlink ref="E103" r:id="rId77" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
+    <hyperlink ref="E24" r:id="rId78" xr:uid="{A1BB8086-1232-764F-9321-DBAFA8F4E6BC}"/>
+    <hyperlink ref="E81" r:id="rId79" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
+    <hyperlink ref="E88" r:id="rId80" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
+    <hyperlink ref="E110" r:id="rId81" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
+    <hyperlink ref="E22" r:id="rId82" xr:uid="{D75012BC-D5E3-6D46-B329-96A4CB35BA96}"/>
+    <hyperlink ref="E59" r:id="rId83" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
+    <hyperlink ref="E93" r:id="rId84" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
+    <hyperlink ref="E86" r:id="rId85" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
+    <hyperlink ref="E31" r:id="rId86" xr:uid="{137601BF-06D1-F948-9D79-A5FEE0032F25}"/>
+    <hyperlink ref="E94" r:id="rId87" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
+    <hyperlink ref="E87" r:id="rId88" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
+    <hyperlink ref="E95" r:id="rId89" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
+    <hyperlink ref="E56" r:id="rId90" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
+    <hyperlink ref="E26" r:id="rId91" xr:uid="{E24B841F-2272-CA43-9614-50B7F36AD8C5}"/>
+    <hyperlink ref="E11" r:id="rId92" xr:uid="{29460556-99EB-6943-BF02-EAF45B9A2438}"/>
+    <hyperlink ref="E107" r:id="rId93" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
+    <hyperlink ref="E18" r:id="rId94" xr:uid="{BFCD233B-85C4-684A-9E1F-CFD7E946453F}"/>
+    <hyperlink ref="F88" r:id="rId95" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
+    <hyperlink ref="F68" r:id="rId96" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
+    <hyperlink ref="F28" r:id="rId97" xr:uid="{232B5F00-F258-A24E-BDEA-CF2F2635A32D}"/>
+    <hyperlink ref="F93" r:id="rId98" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
+    <hyperlink ref="E46" r:id="rId99" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
+    <hyperlink ref="F46" r:id="rId100" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
+    <hyperlink ref="E47" r:id="rId101" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
+    <hyperlink ref="E8" r:id="rId102" xr:uid="{E4C80A26-9BBE-CE4E-A398-4F9C5F4955F3}"/>
+    <hyperlink ref="F8" r:id="rId103" xr:uid="{5914BE48-1B32-6F46-B075-BC630F5D8608}"/>
+    <hyperlink ref="E20" r:id="rId104" xr:uid="{D5AF8CE0-2466-6647-B572-C377DB7C2F3F}"/>
+    <hyperlink ref="F20" r:id="rId105" xr:uid="{0DDC6C1F-4537-7C4D-A53D-0EA66E740063}"/>
+    <hyperlink ref="E19" r:id="rId106" xr:uid="{7651A9F0-0FB9-AD45-8536-6DA2DBA419D4}"/>
+    <hyperlink ref="F19" r:id="rId107" xr:uid="{89D30D76-781B-4C4A-9D08-40BF96ECDA97}"/>
+    <hyperlink ref="E108" r:id="rId108" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
+    <hyperlink ref="F108" r:id="rId109" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
+    <hyperlink ref="E61" r:id="rId110" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
+    <hyperlink ref="E72" r:id="rId111" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
+    <hyperlink ref="E111" r:id="rId112" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
+    <hyperlink ref="F72" r:id="rId113" xr:uid="{22B55A5B-C73B-1740-B6AA-6B10A8B349F2}"/>
+    <hyperlink ref="F111" r:id="rId114" xr:uid="{E3192BBD-0D35-6F46-BD87-F7D47501BD47}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
dipc update: add p. ferrero mancheno
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sorel/next/next-exp/NEXTAuthorList/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC5660A-F82B-A14F-AF90-C8BE4DAB2757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B305C8-DD4C-874D-8504-637DA9A6C8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10940" yWindow="3640" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="463">
   <si>
     <t>LastName</t>
   </si>
@@ -1415,6 +1415,12 @@
   </si>
   <si>
     <t>https://orcid.org/0009-0002-5335-0891</t>
+  </si>
+  <si>
+    <t>Ferrero Manche\~{n}o</t>
+  </si>
+  <si>
+    <t>pablo.ferrero@dipc.org</t>
   </si>
 </sst>
 </file>
@@ -2275,7 +2281,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="6" width="20.83203125" customWidth="1"/>
@@ -3010,132 +3016,130 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>461</v>
       </c>
       <c r="B33" t="s">
-        <v>71</v>
-      </c>
-      <c r="E33" t="s">
-        <v>226</v>
-      </c>
-      <c r="F33" t="s">
-        <v>360</v>
-      </c>
+        <v>298</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="F33" s="1"/>
+      <c r="G33" s="2"/>
       <c r="H33" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="I33" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E34" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F34" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H34" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="I34" t="s">
-        <v>18</v>
-      </c>
-      <c r="J34" t="s">
-        <v>67</v>
-      </c>
-      <c r="K34" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>201</v>
+        <v>73</v>
       </c>
       <c r="B35" t="s">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F35" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H35" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I35" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="J35" t="s">
+        <v>67</v>
+      </c>
+      <c r="K35" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
-      </c>
-      <c r="C36" t="s">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="E36" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F36" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="H36" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="I36" t="s">
-        <v>18</v>
-      </c>
-      <c r="J36" t="s">
-        <v>67</v>
-      </c>
-      <c r="K36" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B37" t="s">
-        <v>191</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="G37" s="1"/>
+        <v>76</v>
+      </c>
+      <c r="C37" t="s">
+        <v>77</v>
+      </c>
+      <c r="E37" t="s">
+        <v>229</v>
+      </c>
+      <c r="F37" t="s">
+        <v>363</v>
+      </c>
       <c r="H37" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I37" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="J37" t="s">
+        <v>67</v>
+      </c>
+      <c r="K37" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B38" t="s">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" t="s">
@@ -3147,255 +3151,255 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B39" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G39" s="1"/>
       <c r="H39" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
       <c r="I39" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B40" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>314</v>
+        <v>232</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="I40" t="s">
-        <v>54</v>
+        <v>83</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B41" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>281</v>
+        <v>314</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I41" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B42" t="s">
-        <v>95</v>
+        <v>167</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" t="s">
-        <v>284</v>
+        <v>59</v>
       </c>
       <c r="I42" t="s">
-        <v>285</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B43" t="s">
-        <v>168</v>
+        <v>95</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>233</v>
+        <v>282</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" t="s">
-        <v>16</v>
+        <v>284</v>
       </c>
       <c r="I43" t="s">
-        <v>17</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B44" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" t="s">
-        <v>234</v>
-      </c>
-      <c r="F44" t="s">
-        <v>371</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="G44" s="1"/>
       <c r="H44" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="I44" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B45" t="s">
-        <v>169</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="G45" s="1"/>
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
+        <v>234</v>
+      </c>
+      <c r="F45" t="s">
+        <v>371</v>
+      </c>
       <c r="H45" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="I45" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>436</v>
+        <v>90</v>
       </c>
       <c r="B46" t="s">
-        <v>437</v>
+        <v>169</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>438</v>
+        <v>235</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>439</v>
+        <v>372</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" t="s">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="I46" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>436</v>
       </c>
       <c r="B47" t="s">
-        <v>170</v>
+        <v>437</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="F47" t="s">
-        <v>373</v>
-      </c>
+        <v>438</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="G47" s="1"/>
       <c r="H47" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="I47" t="s">
-        <v>48</v>
-      </c>
-      <c r="J47" t="s">
-        <v>13</v>
-      </c>
-      <c r="K47" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>196</v>
+        <v>91</v>
       </c>
       <c r="B48" t="s">
-        <v>27</v>
+        <v>170</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="G48" s="1"/>
+        <v>440</v>
+      </c>
+      <c r="F48" t="s">
+        <v>373</v>
+      </c>
       <c r="H48" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I48" t="s">
-        <v>50</v>
+        <v>48</v>
+      </c>
+      <c r="J48" t="s">
+        <v>13</v>
+      </c>
+      <c r="K48" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>92</v>
+        <v>196</v>
       </c>
       <c r="B49" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="G49" s="1"/>
       <c r="H49" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="I49" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B50" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" t="s">
-        <v>289</v>
+        <v>36</v>
       </c>
       <c r="I50" t="s">
         <v>18</v>
@@ -3403,272 +3407,272 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B51" t="s">
-        <v>95</v>
+        <v>37</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" t="s">
-        <v>96</v>
+        <v>289</v>
       </c>
       <c r="I51" t="s">
-        <v>97</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B52" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" t="s">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="I52" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B53" t="s">
-        <v>172</v>
+        <v>27</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I53" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B54" t="s">
-        <v>78</v>
+        <v>172</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G54" s="1"/>
       <c r="H54" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="I54" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B55" t="s">
-        <v>173</v>
+        <v>78</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G55" s="1"/>
       <c r="H55" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="I55" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>312</v>
+        <v>101</v>
       </c>
       <c r="B56" t="s">
-        <v>37</v>
+        <v>173</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>321</v>
+        <v>243</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="G56" s="1"/>
       <c r="H56" t="s">
-        <v>289</v>
+        <v>65</v>
       </c>
       <c r="I56" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>102</v>
+        <v>312</v>
       </c>
       <c r="B57" t="s">
-        <v>103</v>
+        <v>37</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>244</v>
+        <v>321</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="G57" s="1"/>
       <c r="H57" t="s">
-        <v>43</v>
+        <v>289</v>
       </c>
       <c r="I57" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B58" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I58" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>305</v>
+        <v>104</v>
       </c>
       <c r="B59" t="s">
-        <v>37</v>
+        <v>174</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>306</v>
+        <v>245</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="G59" s="1"/>
       <c r="H59" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="I59" t="s">
-        <v>17</v>
+        <v>105</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>106</v>
+        <v>305</v>
       </c>
       <c r="B60" t="s">
-        <v>175</v>
+        <v>37</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>246</v>
+        <v>306</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G60" s="1"/>
       <c r="H60" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I60" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B61" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>452</v>
+        <v>246</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G61" s="1"/>
       <c r="H61" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="I61" t="s">
-        <v>50</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B62" t="s">
-        <v>109</v>
+        <v>176</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>247</v>
+        <v>452</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G62" s="1"/>
       <c r="H62" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="I62" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B63" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="I63" t="s">
         <v>48</v>
@@ -3676,318 +3680,318 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B64" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G64" s="1"/>
       <c r="H64" t="s">
-        <v>289</v>
+        <v>47</v>
       </c>
       <c r="I64" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B65" t="s">
-        <v>177</v>
+        <v>113</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" t="s">
-        <v>36</v>
+        <v>289</v>
       </c>
       <c r="I65" t="s">
         <v>18</v>
       </c>
-      <c r="J65" t="s">
-        <v>67</v>
-      </c>
-      <c r="K65" t="s">
-        <v>68</v>
-      </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B66" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="G66" s="1"/>
       <c r="H66" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="I66" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="J66" t="s">
+        <v>67</v>
+      </c>
+      <c r="K66" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B67" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="G67" s="1"/>
       <c r="H67" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="I67" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B68" t="s">
-        <v>118</v>
+        <v>179</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>433</v>
+        <v>393</v>
       </c>
       <c r="G68" s="1"/>
       <c r="H68" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="I68" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B69" t="s">
-        <v>180</v>
+        <v>118</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>394</v>
+        <v>433</v>
       </c>
       <c r="G69" s="1"/>
       <c r="H69" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I69" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B70" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="G70" s="1"/>
       <c r="H70" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I70" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B71" t="s">
-        <v>58</v>
+        <v>181</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G71" s="1"/>
       <c r="H71" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="I71" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>453</v>
+        <v>121</v>
       </c>
       <c r="B72" t="s">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>454</v>
+        <v>256</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>459</v>
+        <v>396</v>
       </c>
       <c r="G72" s="1"/>
       <c r="H72" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I72" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>453</v>
       </c>
       <c r="B73" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>257</v>
+        <v>454</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>397</v>
+        <v>459</v>
       </c>
       <c r="G73" s="1"/>
       <c r="H73" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="I73" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B74" t="s">
-        <v>182</v>
+        <v>113</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G74" s="1"/>
       <c r="H74" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="I74" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B75" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="F75" s="1"/>
+        <v>258</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>398</v>
+      </c>
       <c r="G75" s="1"/>
       <c r="H75" t="s">
-        <v>96</v>
+        <v>13</v>
       </c>
       <c r="I75" t="s">
-        <v>97</v>
+        <v>14</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B76" t="s">
-        <v>126</v>
+        <v>183</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>399</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="F76" s="1"/>
       <c r="G76" s="1"/>
       <c r="H76" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="I76" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>195</v>
+        <v>125</v>
       </c>
       <c r="B77" t="s">
-        <v>37</v>
+        <v>126</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G77" s="1"/>
       <c r="H77" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="I77" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>195</v>
       </c>
       <c r="B78" t="s">
-        <v>113</v>
+        <v>37</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G78" s="1"/>
       <c r="H78" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="I78" t="s">
         <v>18</v>
@@ -3995,58 +3999,58 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B79" t="s">
-        <v>35</v>
+        <v>113</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G79" s="1"/>
       <c r="H79" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="I79" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B80" t="s">
-        <v>176</v>
+        <v>35</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="G80" s="1"/>
       <c r="H80" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="I80" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B81" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>296</v>
+        <v>264</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G81" s="1"/>
       <c r="H81" t="s">
@@ -4058,191 +4062,191 @@
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B82" t="s">
-        <v>126</v>
+        <v>174</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G82" s="1"/>
       <c r="H82" t="s">
-        <v>289</v>
+        <v>49</v>
       </c>
       <c r="I82" t="s">
-        <v>18</v>
-      </c>
-      <c r="J82" t="s">
-        <v>36</v>
-      </c>
-      <c r="K82" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B83" t="s">
-        <v>8</v>
+        <v>126</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G83" s="1"/>
       <c r="H83" t="s">
-        <v>45</v>
+        <v>289</v>
       </c>
       <c r="I83" t="s">
         <v>18</v>
       </c>
+      <c r="J83" t="s">
+        <v>36</v>
+      </c>
+      <c r="K83" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B84" t="s">
-        <v>171</v>
+        <v>8</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>311</v>
+        <v>266</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="G84" s="2">
-        <v>45718</v>
-      </c>
+        <v>406</v>
+      </c>
+      <c r="G84" s="1"/>
       <c r="H84" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="I84" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B85" t="s">
-        <v>182</v>
-      </c>
-      <c r="C85" t="s">
-        <v>293</v>
+        <v>171</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>267</v>
+        <v>311</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="G85" s="2">
-        <v>45779</v>
+        <v>45718</v>
       </c>
       <c r="H85" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="I85" t="s">
-        <v>18</v>
-      </c>
-      <c r="K85" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B86" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C86" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>310</v>
+        <v>267</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G86" s="2">
         <v>45779</v>
       </c>
       <c r="H86" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I86" t="s">
-        <v>50</v>
+        <v>18</v>
+      </c>
+      <c r="K86" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>328</v>
+        <v>135</v>
       </c>
       <c r="B87" t="s">
-        <v>58</v>
+        <v>184</v>
+      </c>
+      <c r="C87" t="s">
+        <v>291</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="G87" s="1"/>
+        <v>409</v>
+      </c>
+      <c r="G87" s="2">
+        <v>45779</v>
+      </c>
       <c r="H87" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="I87" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>297</v>
+        <v>328</v>
       </c>
       <c r="B88" t="s">
-        <v>298</v>
+        <v>58</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>302</v>
+        <v>319</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>431</v>
+        <v>410</v>
       </c>
       <c r="G88" s="1"/>
       <c r="H88" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="I88" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>136</v>
+        <v>297</v>
       </c>
       <c r="B89" t="s">
-        <v>185</v>
+        <v>298</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>327</v>
+        <v>302</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>411</v>
+        <v>431</v>
       </c>
       <c r="G89" s="1"/>
       <c r="H89" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I89" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
@@ -4250,17 +4254,17 @@
         <v>136</v>
       </c>
       <c r="B90" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G90" s="1"/>
       <c r="H90" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="I90" t="s">
         <v>54</v>
@@ -4268,71 +4272,71 @@
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>192</v>
+        <v>136</v>
       </c>
       <c r="B91" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>268</v>
+        <v>315</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G91" s="1"/>
       <c r="H91" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="I91" t="s">
-        <v>18</v>
-      </c>
-      <c r="J91" t="s">
-        <v>290</v>
-      </c>
-      <c r="K91" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>137</v>
+        <v>192</v>
       </c>
       <c r="B92" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="G92" s="1"/>
       <c r="H92" t="s">
-        <v>284</v>
+        <v>36</v>
       </c>
       <c r="I92" t="s">
-        <v>285</v>
+        <v>18</v>
+      </c>
+      <c r="J92" t="s">
+        <v>290</v>
+      </c>
+      <c r="K92" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>198</v>
+        <v>137</v>
       </c>
       <c r="B93" t="s">
-        <v>308</v>
+        <v>126</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>309</v>
+        <v>269</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>435</v>
+        <v>414</v>
       </c>
       <c r="G93" s="1"/>
       <c r="H93" t="s">
-        <v>31</v>
+        <v>284</v>
       </c>
       <c r="I93" t="s">
-        <v>32</v>
+        <v>285</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
@@ -4340,101 +4344,101 @@
         <v>198</v>
       </c>
       <c r="B94" t="s">
-        <v>199</v>
+        <v>308</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="F94" s="1"/>
+        <v>309</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>435</v>
+      </c>
       <c r="G94" s="1"/>
       <c r="H94" t="s">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="I94" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>138</v>
+        <v>198</v>
       </c>
       <c r="B95" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="F95" s="1" t="s">
-        <v>415</v>
-      </c>
+        <v>316</v>
+      </c>
+      <c r="F95" s="1"/>
       <c r="G95" s="1"/>
       <c r="H95" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="I95" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B96" t="s">
-        <v>140</v>
+        <v>187</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>270</v>
+        <v>320</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G96" s="1"/>
       <c r="H96" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="I96" t="s">
-        <v>18</v>
-      </c>
-      <c r="J96" t="s">
-        <v>67</v>
-      </c>
-      <c r="K96" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B97" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="G97" s="1"/>
       <c r="H97" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I97" t="s">
-        <v>50</v>
+        <v>18</v>
+      </c>
+      <c r="J97" t="s">
+        <v>67</v>
+      </c>
+      <c r="K97" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B98" t="s">
-        <v>113</v>
+        <v>176</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="G98" s="1"/>
       <c r="H98" t="s">
@@ -4446,98 +4450,98 @@
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B99" t="s">
-        <v>144</v>
+        <v>113</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="F99" s="1"/>
+        <v>283</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>418</v>
+      </c>
       <c r="G99" s="1"/>
       <c r="H99" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="I99" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>200</v>
+        <v>143</v>
       </c>
       <c r="B100" t="s">
-        <v>29</v>
+        <v>144</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="F100" s="1" t="s">
-        <v>419</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="F100" s="1"/>
       <c r="G100" s="1"/>
       <c r="H100" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="I100" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>145</v>
+        <v>200</v>
       </c>
       <c r="B101" t="s">
-        <v>188</v>
+        <v>29</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="G101" s="1"/>
       <c r="H101" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="I101" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>197</v>
+        <v>145</v>
       </c>
       <c r="B102" t="s">
-        <v>8</v>
+        <v>188</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="G102" s="1"/>
       <c r="H102" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="I102" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>287</v>
+        <v>197</v>
       </c>
       <c r="B103" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="G103" s="1"/>
       <c r="H103" t="s">
@@ -4549,16 +4553,16 @@
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>146</v>
+        <v>287</v>
       </c>
       <c r="B104" t="s">
-        <v>174</v>
+        <v>29</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="G104" s="1"/>
       <c r="H104" t="s">
@@ -4567,182 +4571,182 @@
       <c r="I104" t="s">
         <v>18</v>
       </c>
-      <c r="J104" t="s">
-        <v>147</v>
-      </c>
-      <c r="K104" t="s">
-        <v>148</v>
-      </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B105" t="s">
-        <v>37</v>
+        <v>174</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>432</v>
+        <v>275</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G105" s="1"/>
       <c r="H105" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I105" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="J105" t="s">
+        <v>147</v>
+      </c>
+      <c r="K105" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>193</v>
+        <v>149</v>
       </c>
       <c r="B106" t="s">
-        <v>194</v>
+        <v>37</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="F106" s="1"/>
+        <v>432</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>424</v>
+      </c>
       <c r="G106" s="1"/>
       <c r="H106" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="I106" t="s">
-        <v>18</v>
-      </c>
-      <c r="J106" t="s">
-        <v>19</v>
-      </c>
-      <c r="K106" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>329</v>
+        <v>193</v>
       </c>
       <c r="B107" t="s">
-        <v>35</v>
+        <v>194</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="F107" s="1" t="s">
-        <v>425</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="F107" s="1"/>
       <c r="G107" s="1"/>
       <c r="H107" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="I107" t="s">
-        <v>48</v>
+        <v>18</v>
+      </c>
+      <c r="J107" t="s">
+        <v>19</v>
+      </c>
+      <c r="K107" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>449</v>
+        <v>329</v>
       </c>
       <c r="B108" t="s">
-        <v>298</v>
+        <v>35</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>450</v>
+        <v>330</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>451</v>
+        <v>425</v>
       </c>
       <c r="G108" s="1"/>
       <c r="H108" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="I108" t="s">
-        <v>18</v>
-      </c>
-      <c r="J108" t="s">
-        <v>59</v>
-      </c>
-      <c r="K108" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>150</v>
+        <v>449</v>
       </c>
       <c r="B109" t="s">
-        <v>189</v>
+        <v>298</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>277</v>
+        <v>450</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>426</v>
+        <v>451</v>
       </c>
       <c r="G109" s="1"/>
       <c r="H109" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="I109" t="s">
-        <v>69</v>
+        <v>18</v>
+      </c>
+      <c r="J109" t="s">
+        <v>59</v>
+      </c>
+      <c r="K109" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>299</v>
+        <v>150</v>
       </c>
       <c r="B110" t="s">
-        <v>300</v>
+        <v>189</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>303</v>
+        <v>277</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="G110" s="1"/>
       <c r="H110" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="I110" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A111" s="3" t="s">
-        <v>455</v>
+      <c r="A111" t="s">
+        <v>299</v>
       </c>
       <c r="B111" t="s">
-        <v>456</v>
+        <v>300</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>457</v>
+        <v>303</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>460</v>
+        <v>427</v>
       </c>
       <c r="G111" s="1"/>
       <c r="H111" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="I111" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
-        <v>151</v>
+      <c r="A112" s="3" t="s">
+        <v>455</v>
       </c>
       <c r="B112" t="s">
-        <v>152</v>
+        <v>456</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>278</v>
+        <v>457</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>428</v>
+        <v>460</v>
       </c>
       <c r="G112" s="1"/>
       <c r="H112" t="s">
@@ -4754,28 +4758,49 @@
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>202</v>
+        <v>151</v>
       </c>
       <c r="B113" t="s">
-        <v>37</v>
+        <v>152</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="G113" s="1"/>
       <c r="H113" t="s">
+        <v>13</v>
+      </c>
+      <c r="I113" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>202</v>
+      </c>
+      <c r="B114" t="s">
+        <v>37</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="G114" s="1"/>
+      <c r="H114" t="s">
         <v>36</v>
       </c>
-      <c r="I113" t="s">
+      <c r="I114" t="s">
         <v>18</v>
       </c>
-      <c r="J113" t="s">
+      <c r="J114" t="s">
         <v>290</v>
       </c>
-      <c r="K113" t="s">
+      <c r="K114" t="s">
         <v>286</v>
       </c>
     </row>
@@ -4793,108 +4818,108 @@
     <hyperlink ref="E27" r:id="rId10" xr:uid="{2B53C67F-39F7-4A49-99C5-3CED9DB96DF6}"/>
     <hyperlink ref="E30" r:id="rId11" xr:uid="{B022962F-480B-E242-A4EB-4B4743EC7105}"/>
     <hyperlink ref="E32" r:id="rId12" xr:uid="{3503F030-FF3A-A74C-AECE-58009DA1DD3E}"/>
-    <hyperlink ref="E37" r:id="rId13" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
-    <hyperlink ref="E38" r:id="rId14" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
-    <hyperlink ref="E39" r:id="rId15" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
-    <hyperlink ref="E40" r:id="rId16" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
-    <hyperlink ref="E41" r:id="rId17" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
-    <hyperlink ref="E42" r:id="rId18" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
-    <hyperlink ref="E43" r:id="rId19" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
-    <hyperlink ref="E45" r:id="rId20" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
-    <hyperlink ref="E48" r:id="rId21" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
-    <hyperlink ref="E49" r:id="rId22" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
-    <hyperlink ref="E51" r:id="rId23" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
-    <hyperlink ref="E55" r:id="rId24" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
-    <hyperlink ref="E62" r:id="rId25" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
-    <hyperlink ref="E58" r:id="rId26" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
-    <hyperlink ref="E63" r:id="rId27" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
-    <hyperlink ref="E65" r:id="rId28" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
-    <hyperlink ref="E67" r:id="rId29" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
-    <hyperlink ref="E68" r:id="rId30" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
+    <hyperlink ref="E38" r:id="rId13" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
+    <hyperlink ref="E39" r:id="rId14" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
+    <hyperlink ref="E40" r:id="rId15" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
+    <hyperlink ref="E41" r:id="rId16" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
+    <hyperlink ref="E42" r:id="rId17" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
+    <hyperlink ref="E43" r:id="rId18" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
+    <hyperlink ref="E44" r:id="rId19" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
+    <hyperlink ref="E46" r:id="rId20" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
+    <hyperlink ref="E49" r:id="rId21" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
+    <hyperlink ref="E50" r:id="rId22" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
+    <hyperlink ref="E52" r:id="rId23" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
+    <hyperlink ref="E56" r:id="rId24" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
+    <hyperlink ref="E63" r:id="rId25" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
+    <hyperlink ref="E59" r:id="rId26" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
+    <hyperlink ref="E64" r:id="rId27" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
+    <hyperlink ref="E66" r:id="rId28" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
+    <hyperlink ref="E68" r:id="rId29" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
+    <hyperlink ref="E69" r:id="rId30" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
     <hyperlink ref="E2" r:id="rId31" xr:uid="{3A3CFB2D-9550-DB47-876D-1CF2172ED36B}"/>
-    <hyperlink ref="E60" r:id="rId32" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
-    <hyperlink ref="E69" r:id="rId33" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
-    <hyperlink ref="E70" r:id="rId34" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
+    <hyperlink ref="E61" r:id="rId32" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
+    <hyperlink ref="E70" r:id="rId33" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
+    <hyperlink ref="E71" r:id="rId34" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
     <hyperlink ref="E23" r:id="rId35" xr:uid="{403F5279-8F67-B64C-A27C-18563FED25F5}"/>
-    <hyperlink ref="E71" r:id="rId36" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
-    <hyperlink ref="E73" r:id="rId37" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
-    <hyperlink ref="E74" r:id="rId38" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
-    <hyperlink ref="E75" r:id="rId39" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
-    <hyperlink ref="E76" r:id="rId40" xr:uid="{C651F08A-4556-B04E-BEC5-BBBA98A040F7}"/>
-    <hyperlink ref="E77" r:id="rId41" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
-    <hyperlink ref="E78" r:id="rId42" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
-    <hyperlink ref="E80" r:id="rId43" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
-    <hyperlink ref="E82" r:id="rId44" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
-    <hyperlink ref="E83" r:id="rId45" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
-    <hyperlink ref="E84" r:id="rId46" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
-    <hyperlink ref="E85" r:id="rId47" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
-    <hyperlink ref="E89" r:id="rId48" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
-    <hyperlink ref="E91" r:id="rId49" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
-    <hyperlink ref="E96" r:id="rId50" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
-    <hyperlink ref="E98" r:id="rId51" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
-    <hyperlink ref="E99" r:id="rId52" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
-    <hyperlink ref="E100" r:id="rId53" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
-    <hyperlink ref="E101" r:id="rId54" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
-    <hyperlink ref="E102" r:id="rId55" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
-    <hyperlink ref="E104" r:id="rId56" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
-    <hyperlink ref="E105" r:id="rId57" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
-    <hyperlink ref="E109" r:id="rId58" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
-    <hyperlink ref="E112" r:id="rId59" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
-    <hyperlink ref="E113" r:id="rId60" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
-    <hyperlink ref="E54" r:id="rId61" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
-    <hyperlink ref="E66" r:id="rId62" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
-    <hyperlink ref="E90" r:id="rId63" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
-    <hyperlink ref="E97" r:id="rId64" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
+    <hyperlink ref="E72" r:id="rId36" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
+    <hyperlink ref="E74" r:id="rId37" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
+    <hyperlink ref="E75" r:id="rId38" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
+    <hyperlink ref="E76" r:id="rId39" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
+    <hyperlink ref="E77" r:id="rId40" xr:uid="{C651F08A-4556-B04E-BEC5-BBBA98A040F7}"/>
+    <hyperlink ref="E78" r:id="rId41" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
+    <hyperlink ref="E79" r:id="rId42" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
+    <hyperlink ref="E81" r:id="rId43" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
+    <hyperlink ref="E83" r:id="rId44" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
+    <hyperlink ref="E84" r:id="rId45" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
+    <hyperlink ref="E85" r:id="rId46" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
+    <hyperlink ref="E86" r:id="rId47" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
+    <hyperlink ref="E90" r:id="rId48" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
+    <hyperlink ref="E92" r:id="rId49" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
+    <hyperlink ref="E97" r:id="rId50" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
+    <hyperlink ref="E99" r:id="rId51" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
+    <hyperlink ref="E100" r:id="rId52" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
+    <hyperlink ref="E101" r:id="rId53" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
+    <hyperlink ref="E102" r:id="rId54" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
+    <hyperlink ref="E103" r:id="rId55" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
+    <hyperlink ref="E105" r:id="rId56" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
+    <hyperlink ref="E106" r:id="rId57" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
+    <hyperlink ref="E110" r:id="rId58" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
+    <hyperlink ref="E113" r:id="rId59" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
+    <hyperlink ref="E114" r:id="rId60" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
+    <hyperlink ref="E55" r:id="rId61" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
+    <hyperlink ref="E67" r:id="rId62" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
+    <hyperlink ref="E91" r:id="rId63" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
+    <hyperlink ref="E98" r:id="rId64" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
     <hyperlink ref="E10" r:id="rId65" xr:uid="{464857C2-993C-4144-9F79-68780529C7BD}"/>
-    <hyperlink ref="E57" r:id="rId66" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
+    <hyperlink ref="E58" r:id="rId66" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
     <hyperlink ref="E5" r:id="rId67" display="mailto:isaac.arnquist@pnnl.gov" xr:uid="{308E6526-5B60-F34F-A8F5-559BEC15710C}"/>
-    <hyperlink ref="E52" r:id="rId68" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
-    <hyperlink ref="E53" r:id="rId69" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
+    <hyperlink ref="E53" r:id="rId68" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
+    <hyperlink ref="E54" r:id="rId69" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
     <hyperlink ref="E6" r:id="rId70" xr:uid="{2D0C47D7-E74D-EA48-8223-B97B97694F84}"/>
-    <hyperlink ref="E50" r:id="rId71" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
-    <hyperlink ref="E64" r:id="rId72" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
-    <hyperlink ref="E92" r:id="rId73" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
-    <hyperlink ref="E106" r:id="rId74" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
-    <hyperlink ref="E79" r:id="rId75" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
+    <hyperlink ref="E51" r:id="rId71" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
+    <hyperlink ref="E65" r:id="rId72" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
+    <hyperlink ref="E93" r:id="rId73" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
+    <hyperlink ref="E107" r:id="rId74" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
+    <hyperlink ref="E80" r:id="rId75" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
     <hyperlink ref="E3" r:id="rId76" xr:uid="{1407FD31-5939-8E40-B9DC-A0AC164EEEA9}"/>
-    <hyperlink ref="E103" r:id="rId77" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
+    <hyperlink ref="E104" r:id="rId77" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
     <hyperlink ref="E24" r:id="rId78" xr:uid="{A1BB8086-1232-764F-9321-DBAFA8F4E6BC}"/>
-    <hyperlink ref="E81" r:id="rId79" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
-    <hyperlink ref="E88" r:id="rId80" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
-    <hyperlink ref="E110" r:id="rId81" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
+    <hyperlink ref="E82" r:id="rId79" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
+    <hyperlink ref="E89" r:id="rId80" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
+    <hyperlink ref="E111" r:id="rId81" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
     <hyperlink ref="E22" r:id="rId82" xr:uid="{D75012BC-D5E3-6D46-B329-96A4CB35BA96}"/>
-    <hyperlink ref="E59" r:id="rId83" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
-    <hyperlink ref="E93" r:id="rId84" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
-    <hyperlink ref="E86" r:id="rId85" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
+    <hyperlink ref="E60" r:id="rId83" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
+    <hyperlink ref="E94" r:id="rId84" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
+    <hyperlink ref="E87" r:id="rId85" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
     <hyperlink ref="E31" r:id="rId86" xr:uid="{137601BF-06D1-F948-9D79-A5FEE0032F25}"/>
-    <hyperlink ref="E94" r:id="rId87" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
-    <hyperlink ref="E87" r:id="rId88" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
-    <hyperlink ref="E95" r:id="rId89" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
-    <hyperlink ref="E56" r:id="rId90" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
+    <hyperlink ref="E95" r:id="rId87" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
+    <hyperlink ref="E88" r:id="rId88" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
+    <hyperlink ref="E96" r:id="rId89" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
+    <hyperlink ref="E57" r:id="rId90" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
     <hyperlink ref="E26" r:id="rId91" xr:uid="{E24B841F-2272-CA43-9614-50B7F36AD8C5}"/>
     <hyperlink ref="E11" r:id="rId92" xr:uid="{29460556-99EB-6943-BF02-EAF45B9A2438}"/>
-    <hyperlink ref="E107" r:id="rId93" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
+    <hyperlink ref="E108" r:id="rId93" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
     <hyperlink ref="E18" r:id="rId94" xr:uid="{BFCD233B-85C4-684A-9E1F-CFD7E946453F}"/>
-    <hyperlink ref="F88" r:id="rId95" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
-    <hyperlink ref="F68" r:id="rId96" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
+    <hyperlink ref="F89" r:id="rId95" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
+    <hyperlink ref="F69" r:id="rId96" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
     <hyperlink ref="F28" r:id="rId97" xr:uid="{232B5F00-F258-A24E-BDEA-CF2F2635A32D}"/>
-    <hyperlink ref="F93" r:id="rId98" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
-    <hyperlink ref="E46" r:id="rId99" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
-    <hyperlink ref="F46" r:id="rId100" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
-    <hyperlink ref="E47" r:id="rId101" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
+    <hyperlink ref="F94" r:id="rId98" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
+    <hyperlink ref="E47" r:id="rId99" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
+    <hyperlink ref="F47" r:id="rId100" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
+    <hyperlink ref="E48" r:id="rId101" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
     <hyperlink ref="E8" r:id="rId102" xr:uid="{E4C80A26-9BBE-CE4E-A398-4F9C5F4955F3}"/>
     <hyperlink ref="F8" r:id="rId103" xr:uid="{5914BE48-1B32-6F46-B075-BC630F5D8608}"/>
     <hyperlink ref="E20" r:id="rId104" xr:uid="{D5AF8CE0-2466-6647-B572-C377DB7C2F3F}"/>
     <hyperlink ref="F20" r:id="rId105" xr:uid="{0DDC6C1F-4537-7C4D-A53D-0EA66E740063}"/>
     <hyperlink ref="E19" r:id="rId106" xr:uid="{7651A9F0-0FB9-AD45-8536-6DA2DBA419D4}"/>
     <hyperlink ref="F19" r:id="rId107" xr:uid="{89D30D76-781B-4C4A-9D08-40BF96ECDA97}"/>
-    <hyperlink ref="E108" r:id="rId108" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
-    <hyperlink ref="F108" r:id="rId109" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
-    <hyperlink ref="E61" r:id="rId110" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
-    <hyperlink ref="E72" r:id="rId111" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
-    <hyperlink ref="E111" r:id="rId112" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
-    <hyperlink ref="F72" r:id="rId113" xr:uid="{22B55A5B-C73B-1740-B6AA-6B10A8B349F2}"/>
-    <hyperlink ref="F111" r:id="rId114" xr:uid="{E3192BBD-0D35-6F46-BD87-F7D47501BD47}"/>
+    <hyperlink ref="E109" r:id="rId108" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
+    <hyperlink ref="F109" r:id="rId109" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
+    <hyperlink ref="E62" r:id="rId110" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
+    <hyperlink ref="E73" r:id="rId111" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
+    <hyperlink ref="E112" r:id="rId112" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
+    <hyperlink ref="F73" r:id="rId113" xr:uid="{22B55A5B-C73B-1740-B6AA-6B10A8B349F2}"/>
+    <hyperlink ref="F112" r:id="rId114" xr:uid="{E3192BBD-0D35-6F46-BD87-F7D47501BD47}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
IGFAE update: add C. Cabo
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sorel/next/next-exp/NEXTAuthorList/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B305C8-DD4C-874D-8504-637DA9A6C8DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E134048C-F619-154D-8634-DB50C3E35DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10940" yWindow="3640" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8140" yWindow="9080" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AuthorList" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="466">
   <si>
     <t>LastName</t>
   </si>
@@ -1421,6 +1421,15 @@
   </si>
   <si>
     <t>pablo.ferrero@dipc.org</t>
+  </si>
+  <si>
+    <t>Cabo</t>
+  </si>
+  <si>
+    <t>cristina.cabo@usc.es</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-4149-0208</t>
   </si>
 </sst>
 </file>
@@ -2281,7 +2290,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="6" width="20.83203125" customWidth="1"/>
@@ -2650,72 +2659,66 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>190</v>
+        <v>463</v>
       </c>
       <c r="B17" t="s">
-        <v>187</v>
-      </c>
-      <c r="E17" t="s">
-        <v>216</v>
-      </c>
-      <c r="F17" t="s">
-        <v>347</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="G17" s="1"/>
       <c r="H17" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="I17" t="s">
-        <v>18</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>190</v>
       </c>
       <c r="B18" t="s">
-        <v>161</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="G18" s="2">
-        <v>46174</v>
+        <v>187</v>
+      </c>
+      <c r="E18" t="s">
+        <v>216</v>
+      </c>
+      <c r="F18" t="s">
+        <v>347</v>
       </c>
       <c r="H18" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="I18" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>331</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>161</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>447</v>
+        <v>217</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>448</v>
-      </c>
-      <c r="G19" s="2"/>
+        <v>348</v>
+      </c>
+      <c r="G19" s="2">
+        <v>46174</v>
+      </c>
       <c r="H19" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="I19" t="s">
-        <v>50</v>
-      </c>
-      <c r="J19" t="s">
-        <v>59</v>
-      </c>
-      <c r="K19" t="s">
-        <v>86</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -2723,165 +2726,173 @@
         <v>331</v>
       </c>
       <c r="B20" t="s">
-        <v>444</v>
+        <v>35</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" t="s">
+        <v>49</v>
+      </c>
+      <c r="I20" t="s">
+        <v>50</v>
+      </c>
+      <c r="J20" t="s">
         <v>59</v>
       </c>
-      <c r="I20" t="s">
+      <c r="K20" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>331</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
-      </c>
-      <c r="C21" t="s">
-        <v>292</v>
+        <v>444</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>218</v>
+        <v>445</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="G21" s="1"/>
+        <v>446</v>
+      </c>
+      <c r="G21" s="2"/>
       <c r="H21" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="I21" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>301</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>153</v>
+      </c>
+      <c r="C22" t="s">
+        <v>292</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>304</v>
+        <v>218</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G22" s="1"/>
       <c r="H22" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I22" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>301</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>219</v>
+        <v>304</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="G23" s="1"/>
       <c r="H23" t="s">
-        <v>289</v>
+        <v>49</v>
       </c>
       <c r="I23" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>294</v>
+        <v>55</v>
       </c>
       <c r="B24" t="s">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>295</v>
+        <v>219</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G24" s="1"/>
       <c r="H24" t="s">
-        <v>13</v>
+        <v>289</v>
       </c>
       <c r="I24" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>294</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>220</v>
+        <v>295</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" t="s">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="I25" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>322</v>
+        <v>57</v>
       </c>
       <c r="B26" t="s">
-        <v>298</v>
+        <v>58</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>323</v>
+        <v>220</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>458</v>
-      </c>
+        <v>353</v>
+      </c>
+      <c r="G26" s="1"/>
       <c r="H26" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="I26" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>355</v>
+        <v>322</v>
       </c>
       <c r="B27" t="s">
-        <v>8</v>
+        <v>298</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
+        <v>323</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>458</v>
+      </c>
       <c r="H27" t="s">
         <v>36</v>
       </c>
@@ -2891,276 +2902,274 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>355</v>
       </c>
       <c r="B28" t="s">
-        <v>35</v>
-      </c>
-      <c r="E28" t="s">
-        <v>222</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>434</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
       <c r="H28" t="s">
         <v>36</v>
       </c>
       <c r="I28" t="s">
         <v>18</v>
       </c>
-      <c r="J28" t="s">
-        <v>290</v>
-      </c>
-      <c r="K28" t="s">
-        <v>286</v>
-      </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B29" t="s">
-        <v>163</v>
+        <v>35</v>
       </c>
       <c r="E29" t="s">
-        <v>223</v>
-      </c>
-      <c r="F29" t="s">
-        <v>356</v>
+        <v>222</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>434</v>
       </c>
       <c r="H29" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="I29" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="J29" t="s">
+        <v>290</v>
+      </c>
+      <c r="K29" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B30" t="s">
         <v>163</v>
       </c>
-      <c r="C30" t="s">
-        <v>317</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="G30" s="2">
-        <v>45779</v>
+      <c r="E30" t="s">
+        <v>223</v>
+      </c>
+      <c r="F30" t="s">
+        <v>356</v>
       </c>
       <c r="H30" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I30" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>164</v>
+        <v>163</v>
+      </c>
+      <c r="C31" t="s">
+        <v>317</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>313</v>
+        <v>224</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G31" s="1"/>
+        <v>357</v>
+      </c>
+      <c r="G31" s="2">
+        <v>45779</v>
+      </c>
       <c r="H31" t="s">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="I31" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B32" t="s">
-        <v>165</v>
-      </c>
-      <c r="C32" t="s">
-        <v>318</v>
+        <v>164</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>225</v>
+        <v>313</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="G32" s="2">
-        <v>45496</v>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="G32" s="1"/>
       <c r="H32" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="I32" t="s">
-        <v>18</v>
-      </c>
-      <c r="J32" t="s">
-        <v>67</v>
-      </c>
-      <c r="K32" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>461</v>
+        <v>66</v>
       </c>
       <c r="B33" t="s">
-        <v>298</v>
+        <v>165</v>
+      </c>
+      <c r="C33" t="s">
+        <v>318</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="F33" s="1"/>
-      <c r="G33" s="2"/>
+        <v>225</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="G33" s="2">
+        <v>45496</v>
+      </c>
       <c r="H33" t="s">
         <v>36</v>
       </c>
       <c r="I33" t="s">
         <v>18</v>
       </c>
+      <c r="J33" t="s">
+        <v>67</v>
+      </c>
+      <c r="K33" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>461</v>
       </c>
       <c r="B34" t="s">
-        <v>71</v>
-      </c>
-      <c r="E34" t="s">
-        <v>226</v>
-      </c>
-      <c r="F34" t="s">
-        <v>360</v>
-      </c>
+        <v>298</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="F34" s="1"/>
+      <c r="G34" s="2"/>
       <c r="H34" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="I34" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B35" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E35" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F35" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H35" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="I35" t="s">
-        <v>18</v>
-      </c>
-      <c r="J35" t="s">
-        <v>67</v>
-      </c>
-      <c r="K35" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>201</v>
+        <v>73</v>
       </c>
       <c r="B36" t="s">
-        <v>113</v>
+        <v>74</v>
       </c>
       <c r="E36" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F36" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H36" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I36" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="J36" t="s">
+        <v>67</v>
+      </c>
+      <c r="K36" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>201</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
-      </c>
-      <c r="C37" t="s">
-        <v>77</v>
+        <v>113</v>
       </c>
       <c r="E37" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F37" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="H37" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="I37" t="s">
-        <v>18</v>
-      </c>
-      <c r="J37" t="s">
-        <v>67</v>
-      </c>
-      <c r="K37" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
-        <v>191</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="G38" s="1"/>
+        <v>76</v>
+      </c>
+      <c r="C38" t="s">
+        <v>77</v>
+      </c>
+      <c r="E38" t="s">
+        <v>229</v>
+      </c>
+      <c r="F38" t="s">
+        <v>363</v>
+      </c>
       <c r="H38" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I38" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="J38" t="s">
+        <v>67</v>
+      </c>
+      <c r="K38" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B39" t="s">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="G39" s="1"/>
       <c r="H39" t="s">
@@ -3172,528 +3181,528 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B40" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
       <c r="I40" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>314</v>
+        <v>232</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="I41" t="s">
-        <v>54</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B42" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>281</v>
+        <v>314</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="I42" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
+        <v>167</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" t="s">
-        <v>284</v>
+        <v>59</v>
       </c>
       <c r="I43" t="s">
-        <v>285</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B44" t="s">
-        <v>168</v>
+        <v>95</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>233</v>
+        <v>282</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" t="s">
-        <v>16</v>
+        <v>284</v>
       </c>
       <c r="I44" t="s">
-        <v>17</v>
+        <v>285</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B45" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" t="s">
-        <v>234</v>
-      </c>
-      <c r="F45" t="s">
-        <v>371</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="G45" s="1"/>
       <c r="H45" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="I45" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>169</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="G46" s="1"/>
+        <v>8</v>
+      </c>
+      <c r="E46" t="s">
+        <v>234</v>
+      </c>
+      <c r="F46" t="s">
+        <v>371</v>
+      </c>
       <c r="H46" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="I46" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>436</v>
+        <v>90</v>
       </c>
       <c r="B47" t="s">
-        <v>437</v>
+        <v>169</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>438</v>
+        <v>235</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>439</v>
+        <v>372</v>
       </c>
       <c r="G47" s="1"/>
       <c r="H47" t="s">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="I47" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>436</v>
+      </c>
+      <c r="B48" t="s">
+        <v>437</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="G48" s="1"/>
+      <c r="H48" t="s">
+        <v>65</v>
+      </c>
+      <c r="I48" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>91</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>170</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E49" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="F48" t="s">
+      <c r="F49" t="s">
         <v>373</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H49" t="s">
         <v>47</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I49" t="s">
         <v>48</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J49" t="s">
         <v>13</v>
       </c>
-      <c r="K48" t="s">
+      <c r="K49" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>196</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>27</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E50" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F50" s="1" t="s">
         <v>374</v>
-      </c>
-      <c r="G49" s="1"/>
-      <c r="H49" t="s">
-        <v>49</v>
-      </c>
-      <c r="I49" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>92</v>
-      </c>
-      <c r="B50" t="s">
-        <v>52</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>375</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="I50" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" t="s">
-        <v>289</v>
+        <v>36</v>
       </c>
       <c r="I51" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B52" t="s">
-        <v>95</v>
+        <v>37</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" t="s">
-        <v>96</v>
+        <v>289</v>
       </c>
       <c r="I52" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B53" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" t="s">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="I53" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B54" t="s">
-        <v>172</v>
+        <v>27</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G54" s="1"/>
       <c r="H54" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I54" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B55" t="s">
-        <v>78</v>
+        <v>172</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="G55" s="1"/>
       <c r="H55" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="I55" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B56" t="s">
-        <v>173</v>
+        <v>78</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="G56" s="1"/>
       <c r="H56" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="I56" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>312</v>
+        <v>101</v>
       </c>
       <c r="B57" t="s">
-        <v>37</v>
+        <v>173</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>321</v>
+        <v>243</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="G57" s="1"/>
       <c r="H57" t="s">
-        <v>289</v>
+        <v>65</v>
       </c>
       <c r="I57" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>102</v>
+        <v>312</v>
       </c>
       <c r="B58" t="s">
-        <v>103</v>
+        <v>37</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>244</v>
+        <v>321</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" t="s">
-        <v>43</v>
+        <v>289</v>
       </c>
       <c r="I58" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B59" t="s">
-        <v>174</v>
+        <v>103</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="G59" s="1"/>
       <c r="H59" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="I59" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>305</v>
+        <v>104</v>
       </c>
       <c r="B60" t="s">
-        <v>37</v>
+        <v>174</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>306</v>
+        <v>245</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="G60" s="1"/>
       <c r="H60" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="I60" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>106</v>
+        <v>305</v>
       </c>
       <c r="B61" t="s">
-        <v>175</v>
+        <v>37</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>246</v>
+        <v>306</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="G61" s="1"/>
       <c r="H61" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I61" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B62" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>452</v>
+        <v>246</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G62" s="1"/>
       <c r="H62" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="I62" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B63" t="s">
-        <v>109</v>
+        <v>176</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>247</v>
+        <v>452</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="I63" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B64" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="G64" s="1"/>
       <c r="H64" t="s">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="I64" t="s">
         <v>48</v>
@@ -3701,318 +3710,318 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B65" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" t="s">
-        <v>289</v>
+        <v>47</v>
       </c>
       <c r="I65" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B66" t="s">
-        <v>177</v>
+        <v>113</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="G66" s="1"/>
       <c r="H66" t="s">
-        <v>36</v>
+        <v>289</v>
       </c>
       <c r="I66" t="s">
         <v>18</v>
       </c>
-      <c r="J66" t="s">
-        <v>67</v>
-      </c>
-      <c r="K66" t="s">
-        <v>68</v>
-      </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B67" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="G67" s="1"/>
       <c r="H67" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="I67" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="J67" t="s">
+        <v>67</v>
+      </c>
+      <c r="K67" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B68" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="G68" s="1"/>
       <c r="H68" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="I68" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B69" t="s">
-        <v>118</v>
+        <v>179</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>433</v>
+        <v>393</v>
       </c>
       <c r="G69" s="1"/>
       <c r="H69" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="I69" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B70" t="s">
-        <v>180</v>
+        <v>118</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>394</v>
+        <v>433</v>
       </c>
       <c r="G70" s="1"/>
       <c r="H70" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="I70" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B71" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="G71" s="1"/>
       <c r="H71" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="I71" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B72" t="s">
-        <v>58</v>
+        <v>181</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G72" s="1"/>
       <c r="H72" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="I72" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>453</v>
+        <v>121</v>
       </c>
       <c r="B73" t="s">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>454</v>
+        <v>256</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>459</v>
+        <v>396</v>
       </c>
       <c r="G73" s="1"/>
       <c r="H73" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I73" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>122</v>
+        <v>453</v>
       </c>
       <c r="B74" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>257</v>
+        <v>454</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>397</v>
+        <v>459</v>
       </c>
       <c r="G74" s="1"/>
       <c r="H74" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="I74" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B75" t="s">
-        <v>182</v>
+        <v>113</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G75" s="1"/>
       <c r="H75" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="I75" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B76" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="F76" s="1"/>
+        <v>258</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>398</v>
+      </c>
       <c r="G76" s="1"/>
       <c r="H76" t="s">
-        <v>96</v>
+        <v>13</v>
       </c>
       <c r="I76" t="s">
-        <v>97</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B77" t="s">
-        <v>126</v>
+        <v>183</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="F77" s="1" t="s">
-        <v>399</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="F77" s="1"/>
       <c r="G77" s="1"/>
       <c r="H77" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="I77" t="s">
-        <v>48</v>
+        <v>97</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>195</v>
+        <v>125</v>
       </c>
       <c r="B78" t="s">
-        <v>37</v>
+        <v>126</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G78" s="1"/>
       <c r="H78" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="I78" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>127</v>
+        <v>195</v>
       </c>
       <c r="B79" t="s">
-        <v>113</v>
+        <v>37</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G79" s="1"/>
       <c r="H79" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="I79" t="s">
         <v>18</v>
@@ -4020,58 +4029,58 @@
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B80" t="s">
-        <v>35</v>
+        <v>113</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G80" s="1"/>
       <c r="H80" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="I80" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B81" t="s">
-        <v>176</v>
+        <v>35</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="G81" s="1"/>
       <c r="H81" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="I81" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B82" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>296</v>
+        <v>264</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G82" s="1"/>
       <c r="H82" t="s">
@@ -4083,191 +4092,191 @@
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B83" t="s">
-        <v>126</v>
+        <v>174</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G83" s="1"/>
       <c r="H83" t="s">
-        <v>289</v>
+        <v>49</v>
       </c>
       <c r="I83" t="s">
-        <v>18</v>
-      </c>
-      <c r="J83" t="s">
-        <v>36</v>
-      </c>
-      <c r="K83" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B84" t="s">
-        <v>8</v>
+        <v>126</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G84" s="1"/>
       <c r="H84" t="s">
-        <v>45</v>
+        <v>289</v>
       </c>
       <c r="I84" t="s">
         <v>18</v>
       </c>
+      <c r="J84" t="s">
+        <v>36</v>
+      </c>
+      <c r="K84" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B85" t="s">
-        <v>171</v>
+        <v>8</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>311</v>
+        <v>266</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="G85" s="2">
-        <v>45718</v>
-      </c>
+        <v>406</v>
+      </c>
+      <c r="G85" s="1"/>
       <c r="H85" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="I85" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B86" t="s">
-        <v>182</v>
-      </c>
-      <c r="C86" t="s">
-        <v>293</v>
+        <v>171</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>267</v>
+        <v>311</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="G86" s="2">
-        <v>45779</v>
+        <v>45718</v>
       </c>
       <c r="H86" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="I86" t="s">
-        <v>18</v>
-      </c>
-      <c r="K86" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B87" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C87" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>310</v>
+        <v>267</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G87" s="2">
         <v>45779</v>
       </c>
       <c r="H87" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I87" t="s">
-        <v>50</v>
+        <v>18</v>
+      </c>
+      <c r="K87" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>328</v>
+        <v>135</v>
       </c>
       <c r="B88" t="s">
-        <v>58</v>
+        <v>184</v>
+      </c>
+      <c r="C88" t="s">
+        <v>291</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="G88" s="1"/>
+        <v>409</v>
+      </c>
+      <c r="G88" s="2">
+        <v>45779</v>
+      </c>
       <c r="H88" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="I88" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>297</v>
+        <v>328</v>
       </c>
       <c r="B89" t="s">
-        <v>298</v>
+        <v>58</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>302</v>
+        <v>319</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>431</v>
+        <v>410</v>
       </c>
       <c r="G89" s="1"/>
       <c r="H89" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="I89" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>136</v>
+        <v>297</v>
       </c>
       <c r="B90" t="s">
-        <v>185</v>
+        <v>298</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>327</v>
+        <v>302</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>411</v>
+        <v>431</v>
       </c>
       <c r="G90" s="1"/>
       <c r="H90" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I90" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
@@ -4275,17 +4284,17 @@
         <v>136</v>
       </c>
       <c r="B91" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="G91" s="1"/>
       <c r="H91" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="I91" t="s">
         <v>54</v>
@@ -4293,71 +4302,71 @@
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>192</v>
+        <v>136</v>
       </c>
       <c r="B92" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>268</v>
+        <v>315</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="G92" s="1"/>
       <c r="H92" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="I92" t="s">
-        <v>18</v>
-      </c>
-      <c r="J92" t="s">
-        <v>290</v>
-      </c>
-      <c r="K92" t="s">
-        <v>286</v>
+        <v>54</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>137</v>
+        <v>192</v>
       </c>
       <c r="B93" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="G93" s="1"/>
       <c r="H93" t="s">
-        <v>284</v>
+        <v>36</v>
       </c>
       <c r="I93" t="s">
-        <v>285</v>
+        <v>18</v>
+      </c>
+      <c r="J93" t="s">
+        <v>290</v>
+      </c>
+      <c r="K93" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>198</v>
+        <v>137</v>
       </c>
       <c r="B94" t="s">
-        <v>308</v>
+        <v>126</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>309</v>
+        <v>269</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>435</v>
+        <v>414</v>
       </c>
       <c r="G94" s="1"/>
       <c r="H94" t="s">
-        <v>31</v>
+        <v>284</v>
       </c>
       <c r="I94" t="s">
-        <v>32</v>
+        <v>285</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
@@ -4365,101 +4374,101 @@
         <v>198</v>
       </c>
       <c r="B95" t="s">
-        <v>199</v>
+        <v>308</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="F95" s="1"/>
+        <v>309</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>435</v>
+      </c>
       <c r="G95" s="1"/>
       <c r="H95" t="s">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="I95" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>138</v>
+        <v>198</v>
       </c>
       <c r="B96" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="F96" s="1" t="s">
-        <v>415</v>
-      </c>
+        <v>316</v>
+      </c>
+      <c r="F96" s="1"/>
       <c r="G96" s="1"/>
       <c r="H96" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="I96" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B97" t="s">
-        <v>140</v>
+        <v>187</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>270</v>
+        <v>320</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G97" s="1"/>
       <c r="H97" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="I97" t="s">
-        <v>18</v>
-      </c>
-      <c r="J97" t="s">
-        <v>67</v>
-      </c>
-      <c r="K97" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B98" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="G98" s="1"/>
       <c r="H98" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I98" t="s">
-        <v>50</v>
+        <v>18</v>
+      </c>
+      <c r="J98" t="s">
+        <v>67</v>
+      </c>
+      <c r="K98" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B99" t="s">
-        <v>113</v>
+        <v>176</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="G99" s="1"/>
       <c r="H99" t="s">
@@ -4471,98 +4480,98 @@
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B100" t="s">
-        <v>144</v>
+        <v>113</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="F100" s="1"/>
+        <v>283</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>418</v>
+      </c>
       <c r="G100" s="1"/>
       <c r="H100" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="I100" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>200</v>
+        <v>143</v>
       </c>
       <c r="B101" t="s">
-        <v>29</v>
+        <v>144</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="F101" s="1" t="s">
-        <v>419</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="F101" s="1"/>
       <c r="G101" s="1"/>
       <c r="H101" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="I101" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>145</v>
+        <v>200</v>
       </c>
       <c r="B102" t="s">
-        <v>188</v>
+        <v>29</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="G102" s="1"/>
       <c r="H102" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="I102" t="s">
-        <v>17</v>
+        <v>50</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>197</v>
+        <v>145</v>
       </c>
       <c r="B103" t="s">
-        <v>8</v>
+        <v>188</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="G103" s="1"/>
       <c r="H103" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="I103" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>287</v>
+        <v>197</v>
       </c>
       <c r="B104" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="G104" s="1"/>
       <c r="H104" t="s">
@@ -4574,16 +4583,16 @@
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>146</v>
+        <v>287</v>
       </c>
       <c r="B105" t="s">
-        <v>174</v>
+        <v>29</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="G105" s="1"/>
       <c r="H105" t="s">
@@ -4592,182 +4601,182 @@
       <c r="I105" t="s">
         <v>18</v>
       </c>
-      <c r="J105" t="s">
-        <v>147</v>
-      </c>
-      <c r="K105" t="s">
-        <v>148</v>
-      </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B106" t="s">
-        <v>37</v>
+        <v>174</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>432</v>
+        <v>275</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G106" s="1"/>
       <c r="H106" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I106" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="J106" t="s">
+        <v>147</v>
+      </c>
+      <c r="K106" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>193</v>
+        <v>149</v>
       </c>
       <c r="B107" t="s">
-        <v>194</v>
+        <v>37</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="F107" s="1"/>
+        <v>432</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>424</v>
+      </c>
       <c r="G107" s="1"/>
       <c r="H107" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="I107" t="s">
-        <v>18</v>
-      </c>
-      <c r="J107" t="s">
-        <v>19</v>
-      </c>
-      <c r="K107" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>329</v>
+        <v>193</v>
       </c>
       <c r="B108" t="s">
-        <v>35</v>
+        <v>194</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="F108" s="1" t="s">
-        <v>425</v>
-      </c>
+        <v>276</v>
+      </c>
+      <c r="F108" s="1"/>
       <c r="G108" s="1"/>
       <c r="H108" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="I108" t="s">
-        <v>48</v>
+        <v>18</v>
+      </c>
+      <c r="J108" t="s">
+        <v>19</v>
+      </c>
+      <c r="K108" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>449</v>
+        <v>329</v>
       </c>
       <c r="B109" t="s">
-        <v>298</v>
+        <v>35</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>450</v>
+        <v>330</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>451</v>
+        <v>425</v>
       </c>
       <c r="G109" s="1"/>
       <c r="H109" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="I109" t="s">
-        <v>18</v>
-      </c>
-      <c r="J109" t="s">
-        <v>59</v>
-      </c>
-      <c r="K109" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>150</v>
+        <v>449</v>
       </c>
       <c r="B110" t="s">
-        <v>189</v>
+        <v>298</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>277</v>
+        <v>450</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>426</v>
+        <v>451</v>
       </c>
       <c r="G110" s="1"/>
       <c r="H110" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="I110" t="s">
-        <v>69</v>
+        <v>18</v>
+      </c>
+      <c r="J110" t="s">
+        <v>59</v>
+      </c>
+      <c r="K110" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>299</v>
+        <v>150</v>
       </c>
       <c r="B111" t="s">
-        <v>300</v>
+        <v>189</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>303</v>
+        <v>277</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="G111" s="1"/>
       <c r="H111" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="I111" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A112" s="3" t="s">
-        <v>455</v>
+      <c r="A112" t="s">
+        <v>299</v>
       </c>
       <c r="B112" t="s">
-        <v>456</v>
+        <v>300</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>457</v>
+        <v>303</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>460</v>
+        <v>427</v>
       </c>
       <c r="G112" s="1"/>
       <c r="H112" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="I112" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
-        <v>151</v>
+      <c r="A113" s="3" t="s">
+        <v>455</v>
       </c>
       <c r="B113" t="s">
-        <v>152</v>
+        <v>456</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>278</v>
+        <v>457</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>428</v>
+        <v>460</v>
       </c>
       <c r="G113" s="1"/>
       <c r="H113" t="s">
@@ -4779,28 +4788,49 @@
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>202</v>
+        <v>151</v>
       </c>
       <c r="B114" t="s">
-        <v>37</v>
+        <v>152</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="G114" s="1"/>
       <c r="H114" t="s">
+        <v>13</v>
+      </c>
+      <c r="I114" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>202</v>
+      </c>
+      <c r="B115" t="s">
+        <v>37</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="G115" s="1"/>
+      <c r="H115" t="s">
         <v>36</v>
       </c>
-      <c r="I114" t="s">
+      <c r="I115" t="s">
         <v>18</v>
       </c>
-      <c r="J114" t="s">
+      <c r="J115" t="s">
         <v>290</v>
       </c>
-      <c r="K114" t="s">
+      <c r="K115" t="s">
         <v>286</v>
       </c>
     </row>
@@ -4813,113 +4843,115 @@
     <hyperlink ref="E14" r:id="rId5" xr:uid="{5B370D66-5FA2-8A4A-A92C-48946FC643B8}"/>
     <hyperlink ref="E15" r:id="rId6" xr:uid="{E1E20BC8-2BB4-C34E-8CA8-2ED92BB0838B}"/>
     <hyperlink ref="E16" r:id="rId7" xr:uid="{77E75D5E-F948-2248-A233-77176542B4F7}"/>
-    <hyperlink ref="E21" r:id="rId8" xr:uid="{D9028AA5-E4C8-9E40-BF28-A681BB8D6B4F}"/>
-    <hyperlink ref="E25" r:id="rId9" xr:uid="{221B0995-0A38-FC4A-A9DC-9EFA0954E180}"/>
-    <hyperlink ref="E27" r:id="rId10" xr:uid="{2B53C67F-39F7-4A49-99C5-3CED9DB96DF6}"/>
-    <hyperlink ref="E30" r:id="rId11" xr:uid="{B022962F-480B-E242-A4EB-4B4743EC7105}"/>
-    <hyperlink ref="E32" r:id="rId12" xr:uid="{3503F030-FF3A-A74C-AECE-58009DA1DD3E}"/>
-    <hyperlink ref="E38" r:id="rId13" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
-    <hyperlink ref="E39" r:id="rId14" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
-    <hyperlink ref="E40" r:id="rId15" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
-    <hyperlink ref="E41" r:id="rId16" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
-    <hyperlink ref="E42" r:id="rId17" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
-    <hyperlink ref="E43" r:id="rId18" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
-    <hyperlink ref="E44" r:id="rId19" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
-    <hyperlink ref="E46" r:id="rId20" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
-    <hyperlink ref="E49" r:id="rId21" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
-    <hyperlink ref="E50" r:id="rId22" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
-    <hyperlink ref="E52" r:id="rId23" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
-    <hyperlink ref="E56" r:id="rId24" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
-    <hyperlink ref="E63" r:id="rId25" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
-    <hyperlink ref="E59" r:id="rId26" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
-    <hyperlink ref="E64" r:id="rId27" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
-    <hyperlink ref="E66" r:id="rId28" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
-    <hyperlink ref="E68" r:id="rId29" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
-    <hyperlink ref="E69" r:id="rId30" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
+    <hyperlink ref="E22" r:id="rId8" xr:uid="{D9028AA5-E4C8-9E40-BF28-A681BB8D6B4F}"/>
+    <hyperlink ref="E26" r:id="rId9" xr:uid="{221B0995-0A38-FC4A-A9DC-9EFA0954E180}"/>
+    <hyperlink ref="E28" r:id="rId10" xr:uid="{2B53C67F-39F7-4A49-99C5-3CED9DB96DF6}"/>
+    <hyperlink ref="E31" r:id="rId11" xr:uid="{B022962F-480B-E242-A4EB-4B4743EC7105}"/>
+    <hyperlink ref="E33" r:id="rId12" xr:uid="{3503F030-FF3A-A74C-AECE-58009DA1DD3E}"/>
+    <hyperlink ref="E39" r:id="rId13" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
+    <hyperlink ref="E40" r:id="rId14" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
+    <hyperlink ref="E41" r:id="rId15" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
+    <hyperlink ref="E42" r:id="rId16" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
+    <hyperlink ref="E43" r:id="rId17" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
+    <hyperlink ref="E44" r:id="rId18" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
+    <hyperlink ref="E45" r:id="rId19" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
+    <hyperlink ref="E47" r:id="rId20" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
+    <hyperlink ref="E50" r:id="rId21" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
+    <hyperlink ref="E51" r:id="rId22" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
+    <hyperlink ref="E53" r:id="rId23" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
+    <hyperlink ref="E57" r:id="rId24" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
+    <hyperlink ref="E64" r:id="rId25" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
+    <hyperlink ref="E60" r:id="rId26" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
+    <hyperlink ref="E65" r:id="rId27" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
+    <hyperlink ref="E67" r:id="rId28" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
+    <hyperlink ref="E69" r:id="rId29" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
+    <hyperlink ref="E70" r:id="rId30" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
     <hyperlink ref="E2" r:id="rId31" xr:uid="{3A3CFB2D-9550-DB47-876D-1CF2172ED36B}"/>
-    <hyperlink ref="E61" r:id="rId32" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
-    <hyperlink ref="E70" r:id="rId33" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
-    <hyperlink ref="E71" r:id="rId34" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
-    <hyperlink ref="E23" r:id="rId35" xr:uid="{403F5279-8F67-B64C-A27C-18563FED25F5}"/>
-    <hyperlink ref="E72" r:id="rId36" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
-    <hyperlink ref="E74" r:id="rId37" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
-    <hyperlink ref="E75" r:id="rId38" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
-    <hyperlink ref="E76" r:id="rId39" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
-    <hyperlink ref="E77" r:id="rId40" xr:uid="{C651F08A-4556-B04E-BEC5-BBBA98A040F7}"/>
-    <hyperlink ref="E78" r:id="rId41" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
-    <hyperlink ref="E79" r:id="rId42" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
-    <hyperlink ref="E81" r:id="rId43" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
-    <hyperlink ref="E83" r:id="rId44" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
-    <hyperlink ref="E84" r:id="rId45" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
-    <hyperlink ref="E85" r:id="rId46" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
-    <hyperlink ref="E86" r:id="rId47" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
-    <hyperlink ref="E90" r:id="rId48" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
-    <hyperlink ref="E92" r:id="rId49" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
-    <hyperlink ref="E97" r:id="rId50" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
-    <hyperlink ref="E99" r:id="rId51" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
-    <hyperlink ref="E100" r:id="rId52" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
-    <hyperlink ref="E101" r:id="rId53" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
-    <hyperlink ref="E102" r:id="rId54" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
-    <hyperlink ref="E103" r:id="rId55" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
-    <hyperlink ref="E105" r:id="rId56" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
-    <hyperlink ref="E106" r:id="rId57" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
-    <hyperlink ref="E110" r:id="rId58" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
-    <hyperlink ref="E113" r:id="rId59" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
-    <hyperlink ref="E114" r:id="rId60" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
-    <hyperlink ref="E55" r:id="rId61" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
-    <hyperlink ref="E67" r:id="rId62" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
-    <hyperlink ref="E91" r:id="rId63" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
-    <hyperlink ref="E98" r:id="rId64" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
+    <hyperlink ref="E62" r:id="rId32" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
+    <hyperlink ref="E71" r:id="rId33" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
+    <hyperlink ref="E72" r:id="rId34" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
+    <hyperlink ref="E24" r:id="rId35" xr:uid="{403F5279-8F67-B64C-A27C-18563FED25F5}"/>
+    <hyperlink ref="E73" r:id="rId36" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
+    <hyperlink ref="E75" r:id="rId37" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
+    <hyperlink ref="E76" r:id="rId38" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
+    <hyperlink ref="E77" r:id="rId39" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
+    <hyperlink ref="E78" r:id="rId40" xr:uid="{C651F08A-4556-B04E-BEC5-BBBA98A040F7}"/>
+    <hyperlink ref="E79" r:id="rId41" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
+    <hyperlink ref="E80" r:id="rId42" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
+    <hyperlink ref="E82" r:id="rId43" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
+    <hyperlink ref="E84" r:id="rId44" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
+    <hyperlink ref="E85" r:id="rId45" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
+    <hyperlink ref="E86" r:id="rId46" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
+    <hyperlink ref="E87" r:id="rId47" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
+    <hyperlink ref="E91" r:id="rId48" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
+    <hyperlink ref="E93" r:id="rId49" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
+    <hyperlink ref="E98" r:id="rId50" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
+    <hyperlink ref="E100" r:id="rId51" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
+    <hyperlink ref="E101" r:id="rId52" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
+    <hyperlink ref="E102" r:id="rId53" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
+    <hyperlink ref="E103" r:id="rId54" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
+    <hyperlink ref="E104" r:id="rId55" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
+    <hyperlink ref="E106" r:id="rId56" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
+    <hyperlink ref="E107" r:id="rId57" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
+    <hyperlink ref="E111" r:id="rId58" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
+    <hyperlink ref="E114" r:id="rId59" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
+    <hyperlink ref="E115" r:id="rId60" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
+    <hyperlink ref="E56" r:id="rId61" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
+    <hyperlink ref="E68" r:id="rId62" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
+    <hyperlink ref="E92" r:id="rId63" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
+    <hyperlink ref="E99" r:id="rId64" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
     <hyperlink ref="E10" r:id="rId65" xr:uid="{464857C2-993C-4144-9F79-68780529C7BD}"/>
-    <hyperlink ref="E58" r:id="rId66" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
+    <hyperlink ref="E59" r:id="rId66" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
     <hyperlink ref="E5" r:id="rId67" display="mailto:isaac.arnquist@pnnl.gov" xr:uid="{308E6526-5B60-F34F-A8F5-559BEC15710C}"/>
-    <hyperlink ref="E53" r:id="rId68" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
-    <hyperlink ref="E54" r:id="rId69" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
+    <hyperlink ref="E54" r:id="rId68" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
+    <hyperlink ref="E55" r:id="rId69" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
     <hyperlink ref="E6" r:id="rId70" xr:uid="{2D0C47D7-E74D-EA48-8223-B97B97694F84}"/>
-    <hyperlink ref="E51" r:id="rId71" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
-    <hyperlink ref="E65" r:id="rId72" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
-    <hyperlink ref="E93" r:id="rId73" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
-    <hyperlink ref="E107" r:id="rId74" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
-    <hyperlink ref="E80" r:id="rId75" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
+    <hyperlink ref="E52" r:id="rId71" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
+    <hyperlink ref="E66" r:id="rId72" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
+    <hyperlink ref="E94" r:id="rId73" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
+    <hyperlink ref="E108" r:id="rId74" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
+    <hyperlink ref="E81" r:id="rId75" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
     <hyperlink ref="E3" r:id="rId76" xr:uid="{1407FD31-5939-8E40-B9DC-A0AC164EEEA9}"/>
-    <hyperlink ref="E104" r:id="rId77" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
-    <hyperlink ref="E24" r:id="rId78" xr:uid="{A1BB8086-1232-764F-9321-DBAFA8F4E6BC}"/>
-    <hyperlink ref="E82" r:id="rId79" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
-    <hyperlink ref="E89" r:id="rId80" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
-    <hyperlink ref="E111" r:id="rId81" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
-    <hyperlink ref="E22" r:id="rId82" xr:uid="{D75012BC-D5E3-6D46-B329-96A4CB35BA96}"/>
-    <hyperlink ref="E60" r:id="rId83" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
-    <hyperlink ref="E94" r:id="rId84" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
-    <hyperlink ref="E87" r:id="rId85" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
-    <hyperlink ref="E31" r:id="rId86" xr:uid="{137601BF-06D1-F948-9D79-A5FEE0032F25}"/>
-    <hyperlink ref="E95" r:id="rId87" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
-    <hyperlink ref="E88" r:id="rId88" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
-    <hyperlink ref="E96" r:id="rId89" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
-    <hyperlink ref="E57" r:id="rId90" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
-    <hyperlink ref="E26" r:id="rId91" xr:uid="{E24B841F-2272-CA43-9614-50B7F36AD8C5}"/>
+    <hyperlink ref="E105" r:id="rId77" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
+    <hyperlink ref="E25" r:id="rId78" xr:uid="{A1BB8086-1232-764F-9321-DBAFA8F4E6BC}"/>
+    <hyperlink ref="E83" r:id="rId79" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
+    <hyperlink ref="E90" r:id="rId80" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
+    <hyperlink ref="E112" r:id="rId81" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
+    <hyperlink ref="E23" r:id="rId82" xr:uid="{D75012BC-D5E3-6D46-B329-96A4CB35BA96}"/>
+    <hyperlink ref="E61" r:id="rId83" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
+    <hyperlink ref="E95" r:id="rId84" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
+    <hyperlink ref="E88" r:id="rId85" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
+    <hyperlink ref="E32" r:id="rId86" xr:uid="{137601BF-06D1-F948-9D79-A5FEE0032F25}"/>
+    <hyperlink ref="E96" r:id="rId87" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
+    <hyperlink ref="E89" r:id="rId88" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
+    <hyperlink ref="E97" r:id="rId89" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
+    <hyperlink ref="E58" r:id="rId90" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
+    <hyperlink ref="E27" r:id="rId91" xr:uid="{E24B841F-2272-CA43-9614-50B7F36AD8C5}"/>
     <hyperlink ref="E11" r:id="rId92" xr:uid="{29460556-99EB-6943-BF02-EAF45B9A2438}"/>
-    <hyperlink ref="E108" r:id="rId93" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
-    <hyperlink ref="E18" r:id="rId94" xr:uid="{BFCD233B-85C4-684A-9E1F-CFD7E946453F}"/>
-    <hyperlink ref="F89" r:id="rId95" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
-    <hyperlink ref="F69" r:id="rId96" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
-    <hyperlink ref="F28" r:id="rId97" xr:uid="{232B5F00-F258-A24E-BDEA-CF2F2635A32D}"/>
-    <hyperlink ref="F94" r:id="rId98" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
-    <hyperlink ref="E47" r:id="rId99" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
-    <hyperlink ref="F47" r:id="rId100" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
-    <hyperlink ref="E48" r:id="rId101" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
+    <hyperlink ref="E109" r:id="rId93" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
+    <hyperlink ref="E19" r:id="rId94" xr:uid="{BFCD233B-85C4-684A-9E1F-CFD7E946453F}"/>
+    <hyperlink ref="F90" r:id="rId95" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
+    <hyperlink ref="F70" r:id="rId96" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
+    <hyperlink ref="F29" r:id="rId97" xr:uid="{232B5F00-F258-A24E-BDEA-CF2F2635A32D}"/>
+    <hyperlink ref="F95" r:id="rId98" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
+    <hyperlink ref="E48" r:id="rId99" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
+    <hyperlink ref="F48" r:id="rId100" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
+    <hyperlink ref="E49" r:id="rId101" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
     <hyperlink ref="E8" r:id="rId102" xr:uid="{E4C80A26-9BBE-CE4E-A398-4F9C5F4955F3}"/>
     <hyperlink ref="F8" r:id="rId103" xr:uid="{5914BE48-1B32-6F46-B075-BC630F5D8608}"/>
-    <hyperlink ref="E20" r:id="rId104" xr:uid="{D5AF8CE0-2466-6647-B572-C377DB7C2F3F}"/>
-    <hyperlink ref="F20" r:id="rId105" xr:uid="{0DDC6C1F-4537-7C4D-A53D-0EA66E740063}"/>
-    <hyperlink ref="E19" r:id="rId106" xr:uid="{7651A9F0-0FB9-AD45-8536-6DA2DBA419D4}"/>
-    <hyperlink ref="F19" r:id="rId107" xr:uid="{89D30D76-781B-4C4A-9D08-40BF96ECDA97}"/>
-    <hyperlink ref="E109" r:id="rId108" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
-    <hyperlink ref="F109" r:id="rId109" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
-    <hyperlink ref="E62" r:id="rId110" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
-    <hyperlink ref="E73" r:id="rId111" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
-    <hyperlink ref="E112" r:id="rId112" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
-    <hyperlink ref="F73" r:id="rId113" xr:uid="{22B55A5B-C73B-1740-B6AA-6B10A8B349F2}"/>
-    <hyperlink ref="F112" r:id="rId114" xr:uid="{E3192BBD-0D35-6F46-BD87-F7D47501BD47}"/>
+    <hyperlink ref="E21" r:id="rId104" xr:uid="{D5AF8CE0-2466-6647-B572-C377DB7C2F3F}"/>
+    <hyperlink ref="F21" r:id="rId105" xr:uid="{0DDC6C1F-4537-7C4D-A53D-0EA66E740063}"/>
+    <hyperlink ref="E20" r:id="rId106" xr:uid="{7651A9F0-0FB9-AD45-8536-6DA2DBA419D4}"/>
+    <hyperlink ref="F20" r:id="rId107" xr:uid="{89D30D76-781B-4C4A-9D08-40BF96ECDA97}"/>
+    <hyperlink ref="E110" r:id="rId108" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
+    <hyperlink ref="F110" r:id="rId109" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
+    <hyperlink ref="E63" r:id="rId110" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
+    <hyperlink ref="E74" r:id="rId111" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
+    <hyperlink ref="E113" r:id="rId112" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
+    <hyperlink ref="F74" r:id="rId113" xr:uid="{22B55A5B-C73B-1740-B6AA-6B10A8B349F2}"/>
+    <hyperlink ref="F113" r:id="rId114" xr:uid="{E3192BBD-0D35-6F46-BD87-F7D47501BD47}"/>
+    <hyperlink ref="E17" r:id="rId115" xr:uid="{7282A957-59C7-2242-9B5C-B8EF75D9F7B7}"/>
+    <hyperlink ref="F17" r:id="rId116" xr:uid="{46335B35-EC75-1748-B7EA-F17851F56424}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
remove n.byrnes and i.parmaksiz from uta, lastactivedate for p.ferrero at dipc
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sorel/next/next-exp/NEXTAuthorList/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E134048C-F619-154D-8634-DB50C3E35DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5043996-05A8-9146-A544-C9AAFBF6F3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8140" yWindow="9080" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8140" yWindow="5360" windowWidth="22920" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AuthorList" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="462">
   <si>
     <t>LastName</t>
   </si>
@@ -172,9 +172,6 @@
     <t>Centro de F\'isica de Materiales (CFM), CSIC \&amp; Universidad del Pais Vasco (UPV/EHU), Manuel de Lardizabal 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Byrnes                       </t>
-  </si>
-  <si>
     <t xml:space="preserve">Department of Physics, University of Texas at Arlington </t>
   </si>
   <si>
@@ -409,9 +406,6 @@
     <t xml:space="preserve">Para                        </t>
   </si>
   <si>
-    <t>Parmaksiz</t>
-  </si>
-  <si>
     <t>I.</t>
   </si>
   <si>
@@ -496,9 +490,6 @@
     <t xml:space="preserve">C.A.N.     </t>
   </si>
   <si>
-    <t xml:space="preserve">N.         </t>
-  </si>
-  <si>
     <t xml:space="preserve">V.         </t>
   </si>
   <si>
@@ -679,9 +670,6 @@
     <t>alexey.brodoline@dipc.org</t>
   </si>
   <si>
-    <t>byrnes.nicholas@mavs.uta.edu</t>
-  </si>
-  <si>
     <t>asier.castillo@dipc.org</t>
   </si>
   <si>
@@ -814,9 +802,6 @@
     <t>para@fnal.gov</t>
   </si>
   <si>
-    <t>ilker.parmaksiz@mavs.uta.edu</t>
-  </si>
-  <si>
     <t>ariadna.pazos@ehu.eus</t>
   </si>
   <si>
@@ -1231,9 +1216,6 @@
     <t>https://orcid.org/0000-0001-5878-650X</t>
   </si>
   <si>
-    <t>https://orcid.org/0009-0002-1478-3977</t>
-  </si>
-  <si>
     <t>https://orcid.org/0000-0002-6074-6213</t>
   </si>
   <si>
@@ -1430,6 +1412,12 @@
   </si>
   <si>
     <t>https://orcid.org/0000-0002-4149-0208</t>
+  </si>
+  <si>
+    <t>23/07/24</t>
+  </si>
+  <si>
+    <t>30/04/26</t>
   </si>
 </sst>
 </file>
@@ -2290,7 +2278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="6" width="20.83203125" customWidth="1"/>
@@ -2310,13 +2298,13 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="F1" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="G1" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="H1" t="s">
         <v>4</v>
@@ -2339,10 +2327,10 @@
         <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" t="s">
@@ -2357,13 +2345,13 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" t="s">
@@ -2378,13 +2366,13 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" t="s">
@@ -2399,13 +2387,13 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="G5" s="2">
         <v>46174</v>
@@ -2425,14 +2413,14 @@
         <v>27</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="I6" t="s">
         <v>18</v>
@@ -2446,38 +2434,38 @@
         <v>29</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" t="s">
         <v>49</v>
-      </c>
-      <c r="I7" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="B8" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -2485,13 +2473,13 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" t="s">
@@ -2506,13 +2494,13 @@
         <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" t="s">
@@ -2524,16 +2512,16 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B11" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="G11" s="1"/>
       <c r="H11" t="s">
@@ -2551,10 +2539,10 @@
         <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F12" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="H12" t="s">
         <v>36</v>
@@ -2563,10 +2551,10 @@
         <v>18</v>
       </c>
       <c r="J12" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="K12" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -2577,10 +2565,10 @@
         <v>41</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" t="s">
@@ -2595,13 +2583,13 @@
         <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" t="s">
@@ -2613,16 +2601,16 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="B15" t="s">
         <v>37</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" t="s">
@@ -2640,259 +2628,259 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>457</v>
       </c>
       <c r="B16" t="s">
-        <v>154</v>
+        <v>8</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="F16" s="1"/>
+        <v>458</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>459</v>
+      </c>
       <c r="G16" s="1"/>
       <c r="H16" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="I16" t="s">
-        <v>48</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>463</v>
+        <v>187</v>
       </c>
       <c r="B17" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="G17" s="1"/>
+        <v>184</v>
+      </c>
+      <c r="E17" t="s">
+        <v>212</v>
+      </c>
+      <c r="F17" t="s">
+        <v>342</v>
+      </c>
       <c r="H17" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="I17" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>190</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>187</v>
-      </c>
-      <c r="E18" t="s">
-        <v>216</v>
-      </c>
-      <c r="F18" t="s">
-        <v>347</v>
+        <v>158</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="G18" s="2">
+        <v>46174</v>
       </c>
       <c r="H18" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="I18" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>326</v>
       </c>
       <c r="B19" t="s">
-        <v>161</v>
+        <v>35</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>217</v>
+        <v>441</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="G19" s="2">
-        <v>46174</v>
-      </c>
+        <v>442</v>
+      </c>
+      <c r="G19" s="2"/>
       <c r="H19" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="I19" t="s">
-        <v>25</v>
+        <v>49</v>
+      </c>
+      <c r="J19" t="s">
+        <v>58</v>
+      </c>
+      <c r="K19" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>438</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="I20" t="s">
-        <v>50</v>
-      </c>
-      <c r="J20" t="s">
-        <v>59</v>
-      </c>
-      <c r="K20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>331</v>
+        <v>52</v>
       </c>
       <c r="B21" t="s">
-        <v>444</v>
+        <v>151</v>
+      </c>
+      <c r="C21" t="s">
+        <v>287</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>445</v>
+        <v>214</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="G21" s="2"/>
+        <v>344</v>
+      </c>
+      <c r="G21" s="1"/>
       <c r="H21" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="I21" t="s">
-        <v>86</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>296</v>
       </c>
       <c r="B22" t="s">
-        <v>153</v>
-      </c>
-      <c r="C22" t="s">
-        <v>292</v>
+        <v>8</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>218</v>
+        <v>299</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="G22" s="1"/>
       <c r="H22" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I22" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>301</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>304</v>
+        <v>215</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="G23" s="1"/>
       <c r="H23" t="s">
-        <v>49</v>
+        <v>284</v>
       </c>
       <c r="I23" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>289</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>219</v>
+        <v>290</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="G24" s="1"/>
       <c r="H24" t="s">
-        <v>289</v>
+        <v>13</v>
       </c>
       <c r="I24" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>294</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>295</v>
+        <v>216</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="I25" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>317</v>
       </c>
       <c r="B26" t="s">
-        <v>58</v>
+        <v>293</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>220</v>
+        <v>318</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="G26" s="1"/>
+        <v>349</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>452</v>
+      </c>
       <c r="H26" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="I26" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>322</v>
+        <v>350</v>
       </c>
       <c r="B27" t="s">
-        <v>298</v>
+        <v>8</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>458</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
       <c r="H27" t="s">
         <v>36</v>
       </c>
@@ -2902,21 +2890,28 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>355</v>
+        <v>59</v>
       </c>
       <c r="B28" t="s">
-        <v>8</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
+        <v>35</v>
+      </c>
+      <c r="E28" t="s">
+        <v>218</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>428</v>
+      </c>
       <c r="H28" t="s">
         <v>36</v>
       </c>
       <c r="I28" t="s">
         <v>18</v>
+      </c>
+      <c r="J28" t="s">
+        <v>285</v>
+      </c>
+      <c r="K28" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -2924,25 +2919,19 @@
         <v>60</v>
       </c>
       <c r="B29" t="s">
-        <v>35</v>
+        <v>160</v>
       </c>
       <c r="E29" t="s">
-        <v>222</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>434</v>
+        <v>219</v>
+      </c>
+      <c r="F29" t="s">
+        <v>351</v>
       </c>
       <c r="H29" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="I29" t="s">
-        <v>18</v>
-      </c>
-      <c r="J29" t="s">
-        <v>290</v>
-      </c>
-      <c r="K29" t="s">
-        <v>286</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
@@ -2950,86 +2939,93 @@
         <v>61</v>
       </c>
       <c r="B30" t="s">
-        <v>163</v>
-      </c>
-      <c r="E30" t="s">
-        <v>223</v>
-      </c>
-      <c r="F30" t="s">
-        <v>356</v>
+        <v>160</v>
+      </c>
+      <c r="C30" t="s">
+        <v>312</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="G30" s="2">
+        <v>45779</v>
       </c>
       <c r="H30" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="I30" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B31" t="s">
-        <v>163</v>
-      </c>
-      <c r="C31" t="s">
-        <v>317</v>
+        <v>161</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>224</v>
+        <v>308</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="G31" s="2">
-        <v>45779</v>
-      </c>
+        <v>353</v>
+      </c>
+      <c r="G31" s="1"/>
       <c r="H31" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="I31" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
-        <v>164</v>
+        <v>162</v>
+      </c>
+      <c r="C32" t="s">
+        <v>313</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>313</v>
+        <v>221</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G32" s="1"/>
+        <v>354</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>460</v>
+      </c>
       <c r="H32" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="I32" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="J32" t="s">
+        <v>66</v>
+      </c>
+      <c r="K32" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>66</v>
+        <v>455</v>
       </c>
       <c r="B33" t="s">
-        <v>165</v>
-      </c>
-      <c r="C33" t="s">
-        <v>318</v>
+        <v>293</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="G33" s="2">
-        <v>45496</v>
+        <v>456</v>
+      </c>
+      <c r="F33" s="1"/>
+      <c r="G33" s="2" t="s">
+        <v>461</v>
       </c>
       <c r="H33" t="s">
         <v>36</v>
@@ -3037,125 +3033,121 @@
       <c r="I33" t="s">
         <v>18</v>
       </c>
-      <c r="J33" t="s">
-        <v>67</v>
-      </c>
-      <c r="K33" t="s">
-        <v>68</v>
-      </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>461</v>
+        <v>69</v>
       </c>
       <c r="B34" t="s">
-        <v>298</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="F34" s="1"/>
-      <c r="G34" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="E34" t="s">
+        <v>222</v>
+      </c>
+      <c r="F34" t="s">
+        <v>355</v>
+      </c>
       <c r="H34" t="s">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="I34" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B35" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E35" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F35" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="H35" t="s">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="I35" t="s">
-        <v>48</v>
+        <v>18</v>
+      </c>
+      <c r="J35" t="s">
+        <v>66</v>
+      </c>
+      <c r="K35" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>198</v>
       </c>
       <c r="B36" t="s">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="E36" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F36" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="H36" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I36" t="s">
-        <v>18</v>
-      </c>
-      <c r="J36" t="s">
-        <v>67</v>
-      </c>
-      <c r="K36" t="s">
-        <v>68</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>201</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
-        <v>113</v>
+        <v>75</v>
+      </c>
+      <c r="C37" t="s">
+        <v>76</v>
       </c>
       <c r="E37" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F37" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="H37" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="I37" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="J37" t="s">
+        <v>66</v>
+      </c>
+      <c r="K37" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
-      </c>
-      <c r="C38" t="s">
-        <v>77</v>
-      </c>
-      <c r="E38" t="s">
-        <v>229</v>
-      </c>
-      <c r="F38" t="s">
-        <v>363</v>
-      </c>
+        <v>188</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="G38" s="1"/>
       <c r="H38" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="I38" t="s">
-        <v>18</v>
-      </c>
-      <c r="J38" t="s">
-        <v>67</v>
-      </c>
-      <c r="K38" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
@@ -3163,13 +3155,13 @@
         <v>79</v>
       </c>
       <c r="B39" t="s">
-        <v>191</v>
+        <v>160</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="G39" s="1"/>
       <c r="H39" t="s">
@@ -3184,41 +3176,41 @@
         <v>80</v>
       </c>
       <c r="B40" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="I40" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B41" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>232</v>
+        <v>309</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="I41" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
@@ -3226,41 +3218,41 @@
         <v>84</v>
       </c>
       <c r="B42" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>314</v>
+        <v>276</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="I42" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B43" t="s">
-        <v>167</v>
+        <v>94</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" t="s">
-        <v>59</v>
+        <v>279</v>
       </c>
       <c r="I43" t="s">
-        <v>86</v>
+        <v>280</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -3268,20 +3260,20 @@
         <v>87</v>
       </c>
       <c r="B44" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>282</v>
+        <v>229</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" t="s">
-        <v>284</v>
+        <v>16</v>
       </c>
       <c r="I44" t="s">
-        <v>285</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -3289,20 +3281,19 @@
         <v>88</v>
       </c>
       <c r="B45" t="s">
-        <v>168</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="G45" s="1"/>
+        <v>8</v>
+      </c>
+      <c r="E45" t="s">
+        <v>230</v>
+      </c>
+      <c r="F45" t="s">
+        <v>366</v>
+      </c>
       <c r="H45" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="I45" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -3310,444 +3301,451 @@
         <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>8</v>
-      </c>
-      <c r="E46" t="s">
-        <v>234</v>
-      </c>
-      <c r="F46" t="s">
-        <v>371</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="G46" s="1"/>
       <c r="H46" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="I46" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>90</v>
+        <v>430</v>
       </c>
       <c r="B47" t="s">
-        <v>169</v>
+        <v>431</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>235</v>
+        <v>432</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>372</v>
+        <v>433</v>
       </c>
       <c r="G47" s="1"/>
       <c r="H47" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="I47" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>436</v>
+        <v>90</v>
       </c>
       <c r="B48" t="s">
-        <v>437</v>
+        <v>167</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="F48" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="G48" s="1"/>
+        <v>434</v>
+      </c>
+      <c r="F48" t="s">
+        <v>368</v>
+      </c>
       <c r="H48" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="I48" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+      <c r="J48" t="s">
+        <v>13</v>
+      </c>
+      <c r="K48" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
+        <v>193</v>
+      </c>
+      <c r="B49" t="s">
+        <v>27</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="G49" s="1"/>
+      <c r="H49" t="s">
+        <v>48</v>
+      </c>
+      <c r="I49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
         <v>91</v>
       </c>
-      <c r="B49" t="s">
-        <v>170</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="F49" t="s">
-        <v>373</v>
-      </c>
-      <c r="H49" t="s">
-        <v>47</v>
-      </c>
-      <c r="I49" t="s">
-        <v>48</v>
-      </c>
-      <c r="J49" t="s">
-        <v>13</v>
-      </c>
-      <c r="K49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>196</v>
-      </c>
       <c r="B50" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I50" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>92</v>
       </c>
       <c r="B51" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="G51" s="1"/>
       <c r="H51" t="s">
-        <v>36</v>
+        <v>284</v>
       </c>
       <c r="I51" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>93</v>
       </c>
       <c r="B52" t="s">
-        <v>37</v>
+        <v>94</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" t="s">
-        <v>289</v>
+        <v>95</v>
       </c>
       <c r="I52" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B53" t="s">
-        <v>95</v>
+        <v>27</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="G53" s="1"/>
       <c r="H53" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="I53" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>98</v>
       </c>
       <c r="B54" t="s">
-        <v>27</v>
+        <v>169</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="G54" s="1"/>
       <c r="H54" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="I54" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>99</v>
       </c>
       <c r="B55" t="s">
-        <v>172</v>
+        <v>77</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="G55" s="1"/>
       <c r="H55" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="I55" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>100</v>
       </c>
       <c r="B56" t="s">
-        <v>78</v>
+        <v>170</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="G56" s="1"/>
       <c r="H56" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="I56" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>101</v>
+        <v>307</v>
       </c>
       <c r="B57" t="s">
-        <v>173</v>
+        <v>37</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>243</v>
+        <v>316</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="G57" s="1"/>
       <c r="H57" t="s">
-        <v>65</v>
+        <v>284</v>
       </c>
       <c r="I57" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>312</v>
+        <v>101</v>
       </c>
       <c r="B58" t="s">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>321</v>
+        <v>240</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="G58" s="1"/>
       <c r="H58" t="s">
-        <v>289</v>
+        <v>43</v>
       </c>
       <c r="I58" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B59" t="s">
-        <v>103</v>
+        <v>171</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="G59" s="1"/>
       <c r="H59" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I59" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>104</v>
+        <v>300</v>
       </c>
       <c r="B60" t="s">
-        <v>174</v>
+        <v>37</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>245</v>
+        <v>301</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="G60" s="1"/>
       <c r="H60" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="I60" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>305</v>
-      </c>
       <c r="B61" t="s">
-        <v>37</v>
+        <v>172</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>306</v>
+        <v>242</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="G61" s="1"/>
       <c r="H61" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="I61" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>106</v>
       </c>
       <c r="B62" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>246</v>
+        <v>446</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="G62" s="1"/>
       <c r="H62" t="s">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="I62" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>107</v>
       </c>
       <c r="B63" t="s">
-        <v>176</v>
+        <v>108</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>452</v>
+        <v>243</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="G63" s="1"/>
       <c r="H63" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="I63" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B64" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="G64" s="1"/>
       <c r="H64" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="I64" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B65" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" t="s">
-        <v>47</v>
+        <v>284</v>
       </c>
       <c r="I65" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B66" t="s">
-        <v>113</v>
+        <v>174</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="G66" s="1"/>
       <c r="H66" t="s">
-        <v>289</v>
+        <v>36</v>
       </c>
       <c r="I66" t="s">
         <v>18</v>
+      </c>
+      <c r="J66" t="s">
+        <v>66</v>
+      </c>
+      <c r="K66" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
@@ -3755,26 +3753,20 @@
         <v>114</v>
       </c>
       <c r="B67" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="G67" s="1"/>
       <c r="H67" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="I67" t="s">
-        <v>18</v>
-      </c>
-      <c r="J67" t="s">
-        <v>67</v>
-      </c>
-      <c r="K67" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.2">
@@ -3782,20 +3774,20 @@
         <v>115</v>
       </c>
       <c r="B68" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="G68" s="1"/>
       <c r="H68" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="I68" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
@@ -3803,41 +3795,41 @@
         <v>116</v>
       </c>
       <c r="B69" t="s">
-        <v>179</v>
+        <v>117</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>393</v>
+        <v>427</v>
       </c>
       <c r="G69" s="1"/>
       <c r="H69" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="I69" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B70" t="s">
-        <v>118</v>
+        <v>177</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>433</v>
+        <v>389</v>
       </c>
       <c r="G70" s="1"/>
       <c r="H70" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I70" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
@@ -3845,20 +3837,20 @@
         <v>119</v>
       </c>
       <c r="B71" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="G71" s="1"/>
       <c r="H71" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I71" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
@@ -3866,62 +3858,62 @@
         <v>120</v>
       </c>
       <c r="B72" t="s">
-        <v>181</v>
+        <v>57</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="G72" s="1"/>
       <c r="H72" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="I72" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>121</v>
+        <v>447</v>
       </c>
       <c r="B73" t="s">
-        <v>58</v>
+        <v>124</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>256</v>
+        <v>448</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>396</v>
+        <v>453</v>
       </c>
       <c r="G73" s="1"/>
       <c r="H73" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="I73" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>453</v>
+        <v>121</v>
       </c>
       <c r="B74" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>454</v>
+        <v>253</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>459</v>
+        <v>392</v>
       </c>
       <c r="G74" s="1"/>
       <c r="H74" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="I74" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
@@ -3929,20 +3921,20 @@
         <v>122</v>
       </c>
       <c r="B75" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="G75" s="1"/>
       <c r="H75" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="I75" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
@@ -3950,39 +3942,39 @@
         <v>123</v>
       </c>
       <c r="B76" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>398</v>
-      </c>
+        <v>255</v>
+      </c>
+      <c r="F76" s="1"/>
       <c r="G76" s="1"/>
       <c r="H76" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="I76" t="s">
-        <v>14</v>
+        <v>96</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>124</v>
+        <v>192</v>
       </c>
       <c r="B77" t="s">
-        <v>183</v>
+        <v>37</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="F77" s="1"/>
+        <v>256</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>394</v>
+      </c>
       <c r="G77" s="1"/>
       <c r="H77" t="s">
-        <v>96</v>
+        <v>19</v>
       </c>
       <c r="I77" t="s">
-        <v>97</v>
+        <v>18</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
@@ -3990,41 +3982,41 @@
         <v>125</v>
       </c>
       <c r="B78" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="G78" s="1"/>
       <c r="H78" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="I78" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>195</v>
+        <v>126</v>
       </c>
       <c r="B79" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="G79" s="1"/>
       <c r="H79" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="I79" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
@@ -4032,20 +4024,20 @@
         <v>127</v>
       </c>
       <c r="B80" t="s">
-        <v>113</v>
+        <v>173</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="G80" s="1"/>
       <c r="H80" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="I80" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
@@ -4053,20 +4045,20 @@
         <v>128</v>
       </c>
       <c r="B81" t="s">
-        <v>35</v>
+        <v>171</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>263</v>
+        <v>291</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="G81" s="1"/>
       <c r="H81" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="I81" t="s">
-        <v>86</v>
+        <v>49</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
@@ -4074,20 +4066,26 @@
         <v>129</v>
       </c>
       <c r="B82" t="s">
-        <v>176</v>
+        <v>124</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="G82" s="1"/>
       <c r="H82" t="s">
-        <v>49</v>
+        <v>284</v>
       </c>
       <c r="I82" t="s">
-        <v>50</v>
+        <v>18</v>
+      </c>
+      <c r="J82" t="s">
+        <v>36</v>
+      </c>
+      <c r="K82" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
@@ -4095,20 +4093,20 @@
         <v>130</v>
       </c>
       <c r="B83" t="s">
-        <v>174</v>
+        <v>8</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>296</v>
+        <v>261</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="G83" s="1"/>
       <c r="H83" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I83" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
@@ -4116,26 +4114,22 @@
         <v>131</v>
       </c>
       <c r="B84" t="s">
-        <v>126</v>
+        <v>168</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>265</v>
+        <v>306</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="G84" s="1"/>
+        <v>401</v>
+      </c>
+      <c r="G84" s="2">
+        <v>45718</v>
+      </c>
       <c r="H84" t="s">
-        <v>289</v>
+        <v>9</v>
       </c>
       <c r="I84" t="s">
-        <v>18</v>
-      </c>
-      <c r="J84" t="s">
-        <v>36</v>
-      </c>
-      <c r="K84" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
@@ -4143,20 +4137,28 @@
         <v>132</v>
       </c>
       <c r="B85" t="s">
-        <v>8</v>
+        <v>179</v>
+      </c>
+      <c r="C85" t="s">
+        <v>288</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="G85" s="1"/>
+        <v>402</v>
+      </c>
+      <c r="G85" s="2">
+        <v>45779</v>
+      </c>
       <c r="H85" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="I85" t="s">
         <v>18</v>
+      </c>
+      <c r="K85" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
@@ -4164,297 +4166,287 @@
         <v>133</v>
       </c>
       <c r="B86" t="s">
-        <v>171</v>
+        <v>181</v>
+      </c>
+      <c r="C86" t="s">
+        <v>286</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="G86" s="2">
-        <v>45718</v>
+        <v>45779</v>
       </c>
       <c r="H86" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="I86" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>134</v>
+        <v>323</v>
       </c>
       <c r="B87" t="s">
-        <v>182</v>
-      </c>
-      <c r="C87" t="s">
-        <v>293</v>
+        <v>57</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>267</v>
+        <v>314</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="G87" s="2">
-        <v>45779</v>
-      </c>
+        <v>404</v>
+      </c>
+      <c r="G87" s="1"/>
       <c r="H87" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I87" t="s">
-        <v>18</v>
-      </c>
-      <c r="K87" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>135</v>
+        <v>292</v>
       </c>
       <c r="B88" t="s">
-        <v>184</v>
-      </c>
-      <c r="C88" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>310</v>
+        <v>297</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="G88" s="2">
-        <v>45779</v>
-      </c>
+        <v>425</v>
+      </c>
+      <c r="G88" s="1"/>
       <c r="H88" t="s">
+        <v>48</v>
+      </c>
+      <c r="I88" t="s">
         <v>49</v>
-      </c>
-      <c r="I88" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>328</v>
+        <v>134</v>
       </c>
       <c r="B89" t="s">
-        <v>58</v>
+        <v>182</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="G89" s="1"/>
       <c r="H89" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="I89" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>297</v>
+        <v>134</v>
       </c>
       <c r="B90" t="s">
-        <v>298</v>
+        <v>183</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>431</v>
+        <v>406</v>
       </c>
       <c r="G90" s="1"/>
       <c r="H90" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="I90" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>136</v>
+        <v>189</v>
       </c>
       <c r="B91" t="s">
-        <v>185</v>
+        <v>35</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>327</v>
+        <v>263</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="G91" s="1"/>
       <c r="H91" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="I91" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="J91" t="s">
+        <v>285</v>
+      </c>
+      <c r="K91" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B92" t="s">
-        <v>186</v>
+        <v>124</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>315</v>
+        <v>264</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="G92" s="1"/>
       <c r="H92" t="s">
-        <v>65</v>
+        <v>279</v>
       </c>
       <c r="I92" t="s">
-        <v>54</v>
+        <v>280</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B93" t="s">
-        <v>35</v>
+        <v>303</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>268</v>
+        <v>304</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="G93" s="1"/>
       <c r="H93" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="I93" t="s">
-        <v>18</v>
-      </c>
-      <c r="J93" t="s">
-        <v>290</v>
-      </c>
-      <c r="K93" t="s">
-        <v>286</v>
+        <v>32</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>137</v>
+        <v>195</v>
       </c>
       <c r="B94" t="s">
-        <v>126</v>
+        <v>196</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="F94" s="1" t="s">
-        <v>414</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="F94" s="1"/>
       <c r="G94" s="1"/>
       <c r="H94" t="s">
-        <v>284</v>
+        <v>64</v>
       </c>
       <c r="I94" t="s">
-        <v>285</v>
+        <v>53</v>
       </c>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>198</v>
+        <v>136</v>
       </c>
       <c r="B95" t="s">
-        <v>308</v>
+        <v>184</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>435</v>
+        <v>409</v>
       </c>
       <c r="G95" s="1"/>
       <c r="H95" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="I95" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>198</v>
+        <v>137</v>
       </c>
       <c r="B96" t="s">
-        <v>199</v>
+        <v>138</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="F96" s="1"/>
+        <v>265</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>410</v>
+      </c>
       <c r="G96" s="1"/>
       <c r="H96" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="I96" t="s">
-        <v>54</v>
+        <v>18</v>
+      </c>
+      <c r="J96" t="s">
+        <v>66</v>
+      </c>
+      <c r="K96" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B97" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>320</v>
+        <v>275</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="G97" s="1"/>
       <c r="H97" t="s">
+        <v>48</v>
+      </c>
+      <c r="I97" t="s">
         <v>49</v>
-      </c>
-      <c r="I97" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B98" t="s">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="G98" s="1"/>
       <c r="H98" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="I98" t="s">
-        <v>18</v>
-      </c>
-      <c r="J98" t="s">
-        <v>67</v>
-      </c>
-      <c r="K98" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.2">
@@ -4462,41 +4454,39 @@
         <v>141</v>
       </c>
       <c r="B99" t="s">
-        <v>176</v>
+        <v>142</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="F99" s="1" t="s">
-        <v>417</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="F99" s="1"/>
       <c r="G99" s="1"/>
       <c r="H99" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="I99" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>142</v>
+        <v>197</v>
       </c>
       <c r="B100" t="s">
-        <v>113</v>
+        <v>29</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>283</v>
+        <v>267</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="G100" s="1"/>
       <c r="H100" t="s">
+        <v>48</v>
+      </c>
+      <c r="I100" t="s">
         <v>49</v>
-      </c>
-      <c r="I100" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.2">
@@ -4504,74 +4494,76 @@
         <v>143</v>
       </c>
       <c r="B101" t="s">
-        <v>144</v>
+        <v>185</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="F101" s="1"/>
+        <v>268</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>414</v>
+      </c>
       <c r="G101" s="1"/>
       <c r="H101" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="I101" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B102" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="G102" s="1"/>
       <c r="H102" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="I102" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>145</v>
+        <v>282</v>
       </c>
       <c r="B103" t="s">
-        <v>188</v>
+        <v>29</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="G103" s="1"/>
       <c r="H103" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="I103" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>197</v>
+        <v>144</v>
       </c>
       <c r="B104" t="s">
-        <v>8</v>
+        <v>171</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="G104" s="1"/>
       <c r="H104" t="s">
@@ -4580,41 +4572,45 @@
       <c r="I104" t="s">
         <v>18</v>
       </c>
+      <c r="J104" t="s">
+        <v>145</v>
+      </c>
+      <c r="K104" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>287</v>
+        <v>147</v>
       </c>
       <c r="B105" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>288</v>
+        <v>426</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="G105" s="1"/>
       <c r="H105" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="I105" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>146</v>
+        <v>190</v>
       </c>
       <c r="B106" t="s">
-        <v>174</v>
+        <v>191</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="F106" s="1" t="s">
-        <v>423</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="F106" s="1"/>
       <c r="G106" s="1"/>
       <c r="H106" t="s">
         <v>36</v>
@@ -4623,44 +4619,46 @@
         <v>18</v>
       </c>
       <c r="J106" t="s">
-        <v>147</v>
+        <v>19</v>
       </c>
       <c r="K106" t="s">
-        <v>148</v>
+        <v>18</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>149</v>
+        <v>324</v>
       </c>
       <c r="B107" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>432</v>
+        <v>325</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="G107" s="1"/>
       <c r="H107" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="I107" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>193</v>
+        <v>443</v>
       </c>
       <c r="B108" t="s">
-        <v>194</v>
+        <v>293</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="F108" s="1"/>
+        <v>444</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>445</v>
+      </c>
       <c r="G108" s="1"/>
       <c r="H108" t="s">
         <v>36</v>
@@ -4669,169 +4667,121 @@
         <v>18</v>
       </c>
       <c r="J108" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="K108" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>329</v>
+        <v>148</v>
       </c>
       <c r="B109" t="s">
-        <v>35</v>
+        <v>186</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>330</v>
+        <v>272</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="G109" s="1"/>
       <c r="H109" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="I109" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>449</v>
+        <v>294</v>
       </c>
       <c r="B110" t="s">
+        <v>295</v>
+      </c>
+      <c r="E110" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="E110" s="1" t="s">
-        <v>450</v>
-      </c>
       <c r="F110" s="1" t="s">
-        <v>451</v>
+        <v>421</v>
       </c>
       <c r="G110" s="1"/>
       <c r="H110" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="I110" t="s">
-        <v>18</v>
-      </c>
-      <c r="J110" t="s">
-        <v>59</v>
-      </c>
-      <c r="K110" t="s">
-        <v>86</v>
+        <v>49</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>150</v>
+      <c r="A111" s="3" t="s">
+        <v>449</v>
       </c>
       <c r="B111" t="s">
-        <v>189</v>
+        <v>450</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>277</v>
+        <v>451</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>426</v>
+        <v>454</v>
       </c>
       <c r="G111" s="1"/>
       <c r="H111" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="I111" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>299</v>
+        <v>149</v>
       </c>
       <c r="B112" t="s">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>303</v>
+        <v>273</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="G112" s="1"/>
       <c r="H112" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="I112" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A113" s="3" t="s">
-        <v>455</v>
+      <c r="A113" t="s">
+        <v>199</v>
       </c>
       <c r="B113" t="s">
-        <v>456</v>
+        <v>37</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>457</v>
+        <v>274</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>460</v>
+        <v>423</v>
       </c>
       <c r="G113" s="1"/>
       <c r="H113" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I113" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
-        <v>151</v>
-      </c>
-      <c r="B114" t="s">
-        <v>152</v>
-      </c>
-      <c r="E114" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="G114" s="1"/>
-      <c r="H114" t="s">
-        <v>13</v>
-      </c>
-      <c r="I114" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>202</v>
-      </c>
-      <c r="B115" t="s">
-        <v>37</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="G115" s="1"/>
-      <c r="H115" t="s">
-        <v>36</v>
-      </c>
-      <c r="I115" t="s">
         <v>18</v>
       </c>
-      <c r="J115" t="s">
-        <v>290</v>
-      </c>
-      <c r="K115" t="s">
-        <v>286</v>
+      <c r="J113" t="s">
+        <v>285</v>
+      </c>
+      <c r="K113" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -4842,116 +4792,114 @@
     <hyperlink ref="E13" r:id="rId4" xr:uid="{7BA53910-2895-8546-8C78-4ADAECEB1354}"/>
     <hyperlink ref="E14" r:id="rId5" xr:uid="{5B370D66-5FA2-8A4A-A92C-48946FC643B8}"/>
     <hyperlink ref="E15" r:id="rId6" xr:uid="{E1E20BC8-2BB4-C34E-8CA8-2ED92BB0838B}"/>
-    <hyperlink ref="E16" r:id="rId7" xr:uid="{77E75D5E-F948-2248-A233-77176542B4F7}"/>
-    <hyperlink ref="E22" r:id="rId8" xr:uid="{D9028AA5-E4C8-9E40-BF28-A681BB8D6B4F}"/>
-    <hyperlink ref="E26" r:id="rId9" xr:uid="{221B0995-0A38-FC4A-A9DC-9EFA0954E180}"/>
-    <hyperlink ref="E28" r:id="rId10" xr:uid="{2B53C67F-39F7-4A49-99C5-3CED9DB96DF6}"/>
-    <hyperlink ref="E31" r:id="rId11" xr:uid="{B022962F-480B-E242-A4EB-4B4743EC7105}"/>
-    <hyperlink ref="E33" r:id="rId12" xr:uid="{3503F030-FF3A-A74C-AECE-58009DA1DD3E}"/>
-    <hyperlink ref="E39" r:id="rId13" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
-    <hyperlink ref="E40" r:id="rId14" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
-    <hyperlink ref="E41" r:id="rId15" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
-    <hyperlink ref="E42" r:id="rId16" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
-    <hyperlink ref="E43" r:id="rId17" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
-    <hyperlink ref="E44" r:id="rId18" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
-    <hyperlink ref="E45" r:id="rId19" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
-    <hyperlink ref="E47" r:id="rId20" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
-    <hyperlink ref="E50" r:id="rId21" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
-    <hyperlink ref="E51" r:id="rId22" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
-    <hyperlink ref="E53" r:id="rId23" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
-    <hyperlink ref="E57" r:id="rId24" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
-    <hyperlink ref="E64" r:id="rId25" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
-    <hyperlink ref="E60" r:id="rId26" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
-    <hyperlink ref="E65" r:id="rId27" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
-    <hyperlink ref="E67" r:id="rId28" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
-    <hyperlink ref="E69" r:id="rId29" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
-    <hyperlink ref="E70" r:id="rId30" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
-    <hyperlink ref="E2" r:id="rId31" xr:uid="{3A3CFB2D-9550-DB47-876D-1CF2172ED36B}"/>
-    <hyperlink ref="E62" r:id="rId32" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
-    <hyperlink ref="E71" r:id="rId33" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
-    <hyperlink ref="E72" r:id="rId34" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
-    <hyperlink ref="E24" r:id="rId35" xr:uid="{403F5279-8F67-B64C-A27C-18563FED25F5}"/>
-    <hyperlink ref="E73" r:id="rId36" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
-    <hyperlink ref="E75" r:id="rId37" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
-    <hyperlink ref="E76" r:id="rId38" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
-    <hyperlink ref="E77" r:id="rId39" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
-    <hyperlink ref="E78" r:id="rId40" xr:uid="{C651F08A-4556-B04E-BEC5-BBBA98A040F7}"/>
-    <hyperlink ref="E79" r:id="rId41" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
-    <hyperlink ref="E80" r:id="rId42" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
-    <hyperlink ref="E82" r:id="rId43" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
-    <hyperlink ref="E84" r:id="rId44" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
-    <hyperlink ref="E85" r:id="rId45" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
-    <hyperlink ref="E86" r:id="rId46" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
-    <hyperlink ref="E87" r:id="rId47" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
-    <hyperlink ref="E91" r:id="rId48" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
-    <hyperlink ref="E93" r:id="rId49" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
-    <hyperlink ref="E98" r:id="rId50" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
-    <hyperlink ref="E100" r:id="rId51" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
-    <hyperlink ref="E101" r:id="rId52" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
-    <hyperlink ref="E102" r:id="rId53" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
-    <hyperlink ref="E103" r:id="rId54" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
-    <hyperlink ref="E104" r:id="rId55" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
-    <hyperlink ref="E106" r:id="rId56" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
-    <hyperlink ref="E107" r:id="rId57" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
-    <hyperlink ref="E111" r:id="rId58" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
-    <hyperlink ref="E114" r:id="rId59" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
-    <hyperlink ref="E115" r:id="rId60" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
-    <hyperlink ref="E56" r:id="rId61" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
-    <hyperlink ref="E68" r:id="rId62" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
-    <hyperlink ref="E92" r:id="rId63" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
-    <hyperlink ref="E99" r:id="rId64" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
-    <hyperlink ref="E10" r:id="rId65" xr:uid="{464857C2-993C-4144-9F79-68780529C7BD}"/>
-    <hyperlink ref="E59" r:id="rId66" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
-    <hyperlink ref="E5" r:id="rId67" display="mailto:isaac.arnquist@pnnl.gov" xr:uid="{308E6526-5B60-F34F-A8F5-559BEC15710C}"/>
-    <hyperlink ref="E54" r:id="rId68" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
-    <hyperlink ref="E55" r:id="rId69" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
-    <hyperlink ref="E6" r:id="rId70" xr:uid="{2D0C47D7-E74D-EA48-8223-B97B97694F84}"/>
-    <hyperlink ref="E52" r:id="rId71" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
-    <hyperlink ref="E66" r:id="rId72" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
-    <hyperlink ref="E94" r:id="rId73" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
-    <hyperlink ref="E108" r:id="rId74" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
-    <hyperlink ref="E81" r:id="rId75" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
-    <hyperlink ref="E3" r:id="rId76" xr:uid="{1407FD31-5939-8E40-B9DC-A0AC164EEEA9}"/>
-    <hyperlink ref="E105" r:id="rId77" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
-    <hyperlink ref="E25" r:id="rId78" xr:uid="{A1BB8086-1232-764F-9321-DBAFA8F4E6BC}"/>
-    <hyperlink ref="E83" r:id="rId79" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
-    <hyperlink ref="E90" r:id="rId80" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
-    <hyperlink ref="E112" r:id="rId81" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
-    <hyperlink ref="E23" r:id="rId82" xr:uid="{D75012BC-D5E3-6D46-B329-96A4CB35BA96}"/>
-    <hyperlink ref="E61" r:id="rId83" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
-    <hyperlink ref="E95" r:id="rId84" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
-    <hyperlink ref="E88" r:id="rId85" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
-    <hyperlink ref="E32" r:id="rId86" xr:uid="{137601BF-06D1-F948-9D79-A5FEE0032F25}"/>
-    <hyperlink ref="E96" r:id="rId87" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
-    <hyperlink ref="E89" r:id="rId88" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
-    <hyperlink ref="E97" r:id="rId89" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
-    <hyperlink ref="E58" r:id="rId90" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
-    <hyperlink ref="E27" r:id="rId91" xr:uid="{E24B841F-2272-CA43-9614-50B7F36AD8C5}"/>
-    <hyperlink ref="E11" r:id="rId92" xr:uid="{29460556-99EB-6943-BF02-EAF45B9A2438}"/>
-    <hyperlink ref="E109" r:id="rId93" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
-    <hyperlink ref="E19" r:id="rId94" xr:uid="{BFCD233B-85C4-684A-9E1F-CFD7E946453F}"/>
-    <hyperlink ref="F90" r:id="rId95" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
-    <hyperlink ref="F70" r:id="rId96" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
-    <hyperlink ref="F29" r:id="rId97" xr:uid="{232B5F00-F258-A24E-BDEA-CF2F2635A32D}"/>
-    <hyperlink ref="F95" r:id="rId98" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
-    <hyperlink ref="E48" r:id="rId99" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
-    <hyperlink ref="F48" r:id="rId100" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
-    <hyperlink ref="E49" r:id="rId101" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
-    <hyperlink ref="E8" r:id="rId102" xr:uid="{E4C80A26-9BBE-CE4E-A398-4F9C5F4955F3}"/>
-    <hyperlink ref="F8" r:id="rId103" xr:uid="{5914BE48-1B32-6F46-B075-BC630F5D8608}"/>
-    <hyperlink ref="E21" r:id="rId104" xr:uid="{D5AF8CE0-2466-6647-B572-C377DB7C2F3F}"/>
-    <hyperlink ref="F21" r:id="rId105" xr:uid="{0DDC6C1F-4537-7C4D-A53D-0EA66E740063}"/>
-    <hyperlink ref="E20" r:id="rId106" xr:uid="{7651A9F0-0FB9-AD45-8536-6DA2DBA419D4}"/>
-    <hyperlink ref="F20" r:id="rId107" xr:uid="{89D30D76-781B-4C4A-9D08-40BF96ECDA97}"/>
-    <hyperlink ref="E110" r:id="rId108" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
-    <hyperlink ref="F110" r:id="rId109" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
-    <hyperlink ref="E63" r:id="rId110" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
-    <hyperlink ref="E74" r:id="rId111" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
-    <hyperlink ref="E113" r:id="rId112" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
-    <hyperlink ref="F74" r:id="rId113" xr:uid="{22B55A5B-C73B-1740-B6AA-6B10A8B349F2}"/>
-    <hyperlink ref="F113" r:id="rId114" xr:uid="{E3192BBD-0D35-6F46-BD87-F7D47501BD47}"/>
-    <hyperlink ref="E17" r:id="rId115" xr:uid="{7282A957-59C7-2242-9B5C-B8EF75D9F7B7}"/>
-    <hyperlink ref="F17" r:id="rId116" xr:uid="{46335B35-EC75-1748-B7EA-F17851F56424}"/>
+    <hyperlink ref="E21" r:id="rId7" xr:uid="{D9028AA5-E4C8-9E40-BF28-A681BB8D6B4F}"/>
+    <hyperlink ref="E25" r:id="rId8" xr:uid="{221B0995-0A38-FC4A-A9DC-9EFA0954E180}"/>
+    <hyperlink ref="E27" r:id="rId9" xr:uid="{2B53C67F-39F7-4A49-99C5-3CED9DB96DF6}"/>
+    <hyperlink ref="E30" r:id="rId10" xr:uid="{B022962F-480B-E242-A4EB-4B4743EC7105}"/>
+    <hyperlink ref="E32" r:id="rId11" xr:uid="{3503F030-FF3A-A74C-AECE-58009DA1DD3E}"/>
+    <hyperlink ref="E38" r:id="rId12" xr:uid="{CEB8BAB9-B042-A34A-B635-6BCBB758D6F8}"/>
+    <hyperlink ref="E39" r:id="rId13" xr:uid="{8D9B2120-0137-C040-A53B-A370B9044CCB}"/>
+    <hyperlink ref="E40" r:id="rId14" xr:uid="{5EAE9946-74A0-2C4C-AF2E-8CC318946DFB}"/>
+    <hyperlink ref="E41" r:id="rId15" xr:uid="{414E8F76-C9B5-D043-B8F7-66A7AC4FE7F9}"/>
+    <hyperlink ref="E42" r:id="rId16" xr:uid="{966468A2-ECAE-E547-B0CC-F5EEA43C95E6}"/>
+    <hyperlink ref="E43" r:id="rId17" xr:uid="{AFBA781B-74EA-4D43-8C5C-3770401790AE}"/>
+    <hyperlink ref="E44" r:id="rId18" xr:uid="{C8972E3C-E75C-D849-9CB4-7D042B3A8058}"/>
+    <hyperlink ref="E46" r:id="rId19" xr:uid="{E94A7644-CFDA-1B41-B9B5-14C74A38FCFD}"/>
+    <hyperlink ref="E49" r:id="rId20" xr:uid="{13FE86C5-4070-A048-A059-C6DC8EEBBBCF}"/>
+    <hyperlink ref="E50" r:id="rId21" xr:uid="{5DCB360F-CBC0-3848-977E-6DFD9444FE4F}"/>
+    <hyperlink ref="E52" r:id="rId22" xr:uid="{A6AE4BE4-E884-1F4F-B788-7A25EF443B8B}"/>
+    <hyperlink ref="E56" r:id="rId23" xr:uid="{026C17E2-2748-6C44-8FE8-0DE2C3EB30ED}"/>
+    <hyperlink ref="E63" r:id="rId24" xr:uid="{095CF6B6-9288-374C-AD52-210A596D5626}"/>
+    <hyperlink ref="E59" r:id="rId25" xr:uid="{202BDED9-0922-6A41-B69F-23FD343F7EF9}"/>
+    <hyperlink ref="E64" r:id="rId26" xr:uid="{33C97671-253E-254F-B62A-44FA310DB5B1}"/>
+    <hyperlink ref="E66" r:id="rId27" xr:uid="{00ECC68F-EE1A-1D4B-BBA5-7072FC5E7FCD}"/>
+    <hyperlink ref="E68" r:id="rId28" xr:uid="{99B3B958-BD25-0447-8385-625DDAE1EBF7}"/>
+    <hyperlink ref="E69" r:id="rId29" xr:uid="{24414099-AF95-D943-813C-2818DFD559F1}"/>
+    <hyperlink ref="E2" r:id="rId30" xr:uid="{3A3CFB2D-9550-DB47-876D-1CF2172ED36B}"/>
+    <hyperlink ref="E61" r:id="rId31" xr:uid="{12E6E42C-6AD1-7B4D-9597-0E457430B2D1}"/>
+    <hyperlink ref="E70" r:id="rId32" xr:uid="{F84050AF-F022-0C4E-98B2-C03F3E8C81DA}"/>
+    <hyperlink ref="E71" r:id="rId33" xr:uid="{BBAA4BFB-60C1-4D46-9903-5C81869B2451}"/>
+    <hyperlink ref="E23" r:id="rId34" xr:uid="{403F5279-8F67-B64C-A27C-18563FED25F5}"/>
+    <hyperlink ref="E72" r:id="rId35" xr:uid="{05780F23-E974-A14B-A7BD-29C752AC1269}"/>
+    <hyperlink ref="E74" r:id="rId36" xr:uid="{26B47F7D-C147-3848-B38C-2D9A9DA0C33F}"/>
+    <hyperlink ref="E75" r:id="rId37" xr:uid="{2BF14A96-4081-2E46-827F-32E4EA8D0C53}"/>
+    <hyperlink ref="E76" r:id="rId38" xr:uid="{2685C65F-39CF-6249-84E6-BC878E3BBC05}"/>
+    <hyperlink ref="E77" r:id="rId39" xr:uid="{6EFE6D0A-2023-9A46-B153-528FD3B639BA}"/>
+    <hyperlink ref="E78" r:id="rId40" xr:uid="{E089342D-EADE-5144-85B4-5B221B6FB51B}"/>
+    <hyperlink ref="E80" r:id="rId41" xr:uid="{0FDDE15D-E614-8D41-81C5-58CDC38DE931}"/>
+    <hyperlink ref="E82" r:id="rId42" xr:uid="{474A574E-FBDA-FC4D-A145-8D4F1A4EB722}"/>
+    <hyperlink ref="E83" r:id="rId43" xr:uid="{7CA22AA8-EBC8-F64A-B96B-91E17E52D41B}"/>
+    <hyperlink ref="E84" r:id="rId44" xr:uid="{7FA7FE8F-9DD7-FF4D-84CA-598017C9D6C0}"/>
+    <hyperlink ref="E85" r:id="rId45" xr:uid="{46BBC652-4D86-A84E-878D-1AB9F86849D6}"/>
+    <hyperlink ref="E89" r:id="rId46" xr:uid="{118D17A4-70BB-814A-837E-BA9B4AF7AABC}"/>
+    <hyperlink ref="E91" r:id="rId47" xr:uid="{E6688BD5-536E-1F40-8D57-41F646FB3097}"/>
+    <hyperlink ref="E96" r:id="rId48" xr:uid="{A83786B8-4609-DB4C-B886-A0F508416DF4}"/>
+    <hyperlink ref="E98" r:id="rId49" xr:uid="{02EA66E6-2B70-4B41-BBC6-C0056CE95EF0}"/>
+    <hyperlink ref="E99" r:id="rId50" xr:uid="{D8FB3995-1FAB-FE49-921B-3834F08A9955}"/>
+    <hyperlink ref="E100" r:id="rId51" xr:uid="{8AE31660-08C0-7E4E-9CF5-75793EE4BAE8}"/>
+    <hyperlink ref="E101" r:id="rId52" xr:uid="{DB061F55-DBDE-A74E-8210-9FA1518AB3FA}"/>
+    <hyperlink ref="E102" r:id="rId53" xr:uid="{624DD26F-2C1E-7A49-BC32-8983E7AB5CE1}"/>
+    <hyperlink ref="E104" r:id="rId54" xr:uid="{F413B786-6B22-634A-AB2E-111579EA63C1}"/>
+    <hyperlink ref="E105" r:id="rId55" xr:uid="{E128C7BD-EB04-5940-B460-D15915636116}"/>
+    <hyperlink ref="E109" r:id="rId56" xr:uid="{92E5B0BF-1629-1544-9BF2-AA4DABAF3BE1}"/>
+    <hyperlink ref="E112" r:id="rId57" xr:uid="{A7ADBB2F-176B-C344-8322-5B13F2A3BDA1}"/>
+    <hyperlink ref="E113" r:id="rId58" xr:uid="{B1AB91E4-83D1-F449-AAB1-9585CE89E54D}"/>
+    <hyperlink ref="E55" r:id="rId59" xr:uid="{B8360AE4-856E-0F4D-ACF5-E39471D481E7}"/>
+    <hyperlink ref="E67" r:id="rId60" xr:uid="{1974D37E-5B37-7D4D-82A6-731A15D607BE}"/>
+    <hyperlink ref="E90" r:id="rId61" xr:uid="{0F240535-4B9A-0548-A68D-7A42A74ACDCC}"/>
+    <hyperlink ref="E97" r:id="rId62" xr:uid="{9E09B36A-3ADD-604B-82AD-2F401E55B19D}"/>
+    <hyperlink ref="E10" r:id="rId63" xr:uid="{464857C2-993C-4144-9F79-68780529C7BD}"/>
+    <hyperlink ref="E58" r:id="rId64" xr:uid="{2905F8A0-D72C-F846-B6E0-0A5993DFFA05}"/>
+    <hyperlink ref="E5" r:id="rId65" display="mailto:isaac.arnquist@pnnl.gov" xr:uid="{308E6526-5B60-F34F-A8F5-559BEC15710C}"/>
+    <hyperlink ref="E53" r:id="rId66" xr:uid="{1CACE84F-E2CD-C74C-AEA1-D2928BFA4503}"/>
+    <hyperlink ref="E54" r:id="rId67" xr:uid="{3D7385AE-56EF-A342-A0D1-586DDD8AF4BE}"/>
+    <hyperlink ref="E6" r:id="rId68" xr:uid="{2D0C47D7-E74D-EA48-8223-B97B97694F84}"/>
+    <hyperlink ref="E51" r:id="rId69" display="mailto:amaia.larumbe@ehu.eus" xr:uid="{6DF6911F-00F3-E547-A8E6-08C387F269CA}"/>
+    <hyperlink ref="E65" r:id="rId70" xr:uid="{F661AF17-C778-0149-A0C7-3F0217DCC29E}"/>
+    <hyperlink ref="E92" r:id="rId71" xr:uid="{FFEAF516-B00C-E44B-83AC-7EED5FF2AB67}"/>
+    <hyperlink ref="E106" r:id="rId72" display="mailto:pablo.garcia@dipc.org" xr:uid="{0C4389B2-D44C-654A-B498-6115532471C9}"/>
+    <hyperlink ref="E79" r:id="rId73" xr:uid="{235A1856-CF13-5048-90E7-01FB7EBCF01C}"/>
+    <hyperlink ref="E3" r:id="rId74" xr:uid="{1407FD31-5939-8E40-B9DC-A0AC164EEEA9}"/>
+    <hyperlink ref="E103" r:id="rId75" xr:uid="{4A109917-0016-FD4E-AB5E-85042C64CC96}"/>
+    <hyperlink ref="E24" r:id="rId76" xr:uid="{A1BB8086-1232-764F-9321-DBAFA8F4E6BC}"/>
+    <hyperlink ref="E81" r:id="rId77" xr:uid="{720C49FB-E08F-A243-B2BF-818E9A279FFC}"/>
+    <hyperlink ref="E88" r:id="rId78" xr:uid="{E83E3204-222C-E341-B533-0F6F3E031F74}"/>
+    <hyperlink ref="E110" r:id="rId79" xr:uid="{5890E7DE-8C5A-194A-850D-5CB1D18110D7}"/>
+    <hyperlink ref="E22" r:id="rId80" xr:uid="{D75012BC-D5E3-6D46-B329-96A4CB35BA96}"/>
+    <hyperlink ref="E60" r:id="rId81" xr:uid="{27C23B05-0062-D141-9CB5-F38A5E2A5615}"/>
+    <hyperlink ref="E93" r:id="rId82" xr:uid="{300B6594-95C8-694A-BC49-79F88D1B7938}"/>
+    <hyperlink ref="E86" r:id="rId83" xr:uid="{A89D8FB9-300E-A44D-A6C9-40183C323D05}"/>
+    <hyperlink ref="E31" r:id="rId84" xr:uid="{137601BF-06D1-F948-9D79-A5FEE0032F25}"/>
+    <hyperlink ref="E94" r:id="rId85" xr:uid="{401FA1E7-B57D-8A46-888A-7FC359B3E8BE}"/>
+    <hyperlink ref="E87" r:id="rId86" xr:uid="{0A20642F-D23C-0A40-A68A-C1EEFE73BFC5}"/>
+    <hyperlink ref="E95" r:id="rId87" xr:uid="{1EAA3F68-BBAB-EB46-A913-60F8E2C47D13}"/>
+    <hyperlink ref="E57" r:id="rId88" xr:uid="{3695667B-23BA-B649-937C-EFF9527A0FD1}"/>
+    <hyperlink ref="E26" r:id="rId89" xr:uid="{E24B841F-2272-CA43-9614-50B7F36AD8C5}"/>
+    <hyperlink ref="E11" r:id="rId90" xr:uid="{29460556-99EB-6943-BF02-EAF45B9A2438}"/>
+    <hyperlink ref="E107" r:id="rId91" xr:uid="{31EA1686-1B20-3342-8310-E26369FFF7C2}"/>
+    <hyperlink ref="E18" r:id="rId92" xr:uid="{BFCD233B-85C4-684A-9E1F-CFD7E946453F}"/>
+    <hyperlink ref="F88" r:id="rId93" xr:uid="{8A532988-D04F-D445-B8FD-AA64E787BB24}"/>
+    <hyperlink ref="F69" r:id="rId94" xr:uid="{D54F73F6-B34C-4044-9163-D80E3A8D31D1}"/>
+    <hyperlink ref="F28" r:id="rId95" xr:uid="{232B5F00-F258-A24E-BDEA-CF2F2635A32D}"/>
+    <hyperlink ref="F93" r:id="rId96" xr:uid="{219994FD-4BE4-D040-8000-FA1EAB97BA79}"/>
+    <hyperlink ref="E47" r:id="rId97" xr:uid="{5120D118-05B0-D540-BE4F-B9DCCD52040C}"/>
+    <hyperlink ref="F47" r:id="rId98" xr:uid="{BCA8D2A5-D5BD-AF4B-8D5E-2A79F1997BDF}"/>
+    <hyperlink ref="E48" r:id="rId99" xr:uid="{2D132A55-81FD-AD46-B0BE-C908F8D920E8}"/>
+    <hyperlink ref="E8" r:id="rId100" xr:uid="{E4C80A26-9BBE-CE4E-A398-4F9C5F4955F3}"/>
+    <hyperlink ref="F8" r:id="rId101" xr:uid="{5914BE48-1B32-6F46-B075-BC630F5D8608}"/>
+    <hyperlink ref="E20" r:id="rId102" xr:uid="{D5AF8CE0-2466-6647-B572-C377DB7C2F3F}"/>
+    <hyperlink ref="F20" r:id="rId103" xr:uid="{0DDC6C1F-4537-7C4D-A53D-0EA66E740063}"/>
+    <hyperlink ref="E19" r:id="rId104" xr:uid="{7651A9F0-0FB9-AD45-8536-6DA2DBA419D4}"/>
+    <hyperlink ref="F19" r:id="rId105" xr:uid="{89D30D76-781B-4C4A-9D08-40BF96ECDA97}"/>
+    <hyperlink ref="E108" r:id="rId106" xr:uid="{026E2B8D-FB9A-F942-A358-7A96EA60AAE6}"/>
+    <hyperlink ref="F108" r:id="rId107" xr:uid="{5D581E56-6F6D-CB4C-81EB-3C2041C0974B}"/>
+    <hyperlink ref="E62" r:id="rId108" xr:uid="{6CDD9F24-D4B4-D646-8B31-5DDB7E06C54F}"/>
+    <hyperlink ref="E73" r:id="rId109" xr:uid="{A055B258-CFB3-274F-A1B8-E8DFAF801887}"/>
+    <hyperlink ref="E111" r:id="rId110" xr:uid="{24D2F24E-7FAE-D744-896E-B75BD10607F0}"/>
+    <hyperlink ref="F73" r:id="rId111" xr:uid="{22B55A5B-C73B-1740-B6AA-6B10A8B349F2}"/>
+    <hyperlink ref="F111" r:id="rId112" xr:uid="{E3192BBD-0D35-6F46-BD87-F7D47501BD47}"/>
+    <hyperlink ref="E16" r:id="rId113" xr:uid="{7282A957-59C7-2242-9B5C-B8EF75D9F7B7}"/>
+    <hyperlink ref="F16" r:id="rId114" xr:uid="{46335B35-EC75-1748-B7EA-F17851F56424}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Afiliation Gonzalo M. L. upated: now at IFIC
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -1429,7 +1429,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1466,6 +1466,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1520,8 +1526,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1529,7 +1539,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1549,7 +1559,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1806,2519 +1820,2520 @@
   <dimension ref="A1:K113"/>
   <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="33.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="112.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="2" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="2" t="s">
+      <c r="G3" s="2"/>
+      <c r="H3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="2" t="s">
+      <c r="G4" s="2"/>
+      <c r="H4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" s="4" t="n">
         <v>46174</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="2" t="s">
+      <c r="G6" s="2"/>
+      <c r="H6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="2" t="s">
+      <c r="G7" s="2"/>
+      <c r="H7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="2" t="s">
+      <c r="G8" s="2"/>
+      <c r="H8" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="1"/>
-      <c r="H9" s="2" t="s">
+      <c r="G9" s="2"/>
+      <c r="H9" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="2" t="s">
+      <c r="G10" s="2"/>
+      <c r="H10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="0" t="s">
+      <c r="H12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I12" s="0" t="s">
+      <c r="I12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J12" s="0" t="s">
+      <c r="J12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="K12" s="0" t="s">
+      <c r="K12" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="G13" s="1"/>
-      <c r="H13" s="2" t="s">
+      <c r="G13" s="2"/>
+      <c r="H13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G14" s="1"/>
-      <c r="H14" s="2" t="s">
+      <c r="G14" s="2"/>
+      <c r="H14" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="3" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="J15" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G16" s="1"/>
-      <c r="H16" s="2" t="s">
+      <c r="G16" s="2"/>
+      <c r="H16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="F17" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="H17" s="0" t="s">
+      <c r="H17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I17" s="0" t="s">
+      <c r="I17" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="G18" s="4" t="n">
         <v>46174</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="I18" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="G19" s="3"/>
-      <c r="H19" s="2" t="s">
+      <c r="G19" s="4"/>
+      <c r="H19" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I19" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="J19" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K19" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="G20" s="3"/>
-      <c r="H20" s="2" t="s">
+      <c r="G20" s="4"/>
+      <c r="H20" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="I20" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G21" s="1"/>
-      <c r="H21" s="2" t="s">
+      <c r="G21" s="2"/>
+      <c r="H21" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="I21" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F22" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G22" s="1"/>
-      <c r="H22" s="2" t="s">
+      <c r="G22" s="2"/>
+      <c r="H22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="I22" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F23" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="G23" s="1"/>
-      <c r="H23" s="2" t="s">
+      <c r="G23" s="2"/>
+      <c r="H23" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="I23" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F24" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G24" s="1"/>
-      <c r="H24" s="2" t="s">
+      <c r="G24" s="2"/>
+      <c r="H24" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="I24" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="G25" s="1"/>
-      <c r="H25" s="2" t="s">
+      <c r="G25" s="2"/>
+      <c r="H25" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="I25" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G26" s="5" t="s">
+      <c r="G26" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H26" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="I26" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="F27" s="1"/>
-      <c r="G27" s="6" t="n">
+      <c r="F27" s="2"/>
+      <c r="G27" s="7" t="n">
         <v>46240</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H27" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="I27" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E28" s="0" t="s">
+      <c r="E28" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="H28" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="I28" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="J28" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="K28" s="3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E29" s="0" t="s">
+      <c r="E29" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="F29" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="H29" s="0" t="s">
+      <c r="H29" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I29" s="0" t="s">
+      <c r="I29" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F30" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="G30" s="4" t="n">
         <v>45779</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="I30" s="3" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E31" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F31" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="G31" s="1"/>
-      <c r="H31" s="2" t="s">
+      <c r="G31" s="2"/>
+      <c r="H31" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="I31" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E32" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="G32" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H32" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="I32" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J32" s="2" t="s">
+      <c r="J32" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="K32" s="2" t="s">
+      <c r="K32" s="3" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="F33" s="1"/>
-      <c r="G33" s="3" t="s">
+      <c r="F33" s="2"/>
+      <c r="G33" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="H33" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="I33" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E34" s="0" t="s">
+      <c r="E34" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="F34" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="H34" s="0" t="s">
+      <c r="H34" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I34" s="0" t="s">
+      <c r="I34" s="1" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="E35" s="0" t="s">
+      <c r="E35" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="F35" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="H35" s="0" t="s">
+      <c r="H35" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="I35" s="0" t="s">
+      <c r="I35" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J35" s="0" t="s">
+      <c r="J35" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="K35" s="0" t="s">
+      <c r="K35" s="1" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="E36" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="F36" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="H36" s="0" t="s">
+      <c r="H36" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I36" s="0" t="s">
+      <c r="I36" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="C37" s="0" t="s">
+      <c r="C37" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="E37" s="0" t="s">
+      <c r="E37" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="F37" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="H37" s="0" t="s">
+      <c r="H37" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I37" s="0" t="s">
+      <c r="I37" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J37" s="0" t="s">
+      <c r="J37" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="K37" s="0" t="s">
+      <c r="K37" s="1" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+      <c r="A38" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B38" s="0" t="s">
+      <c r="B38" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F38" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="G38" s="1"/>
-      <c r="H38" s="2" t="s">
+      <c r="G38" s="2"/>
+      <c r="H38" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="I38" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="B39" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F39" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="G39" s="1"/>
-      <c r="H39" s="2" t="s">
+      <c r="G39" s="2"/>
+      <c r="H39" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="I39" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="A40" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B40" s="0" t="s">
+      <c r="B40" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F40" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="G40" s="1"/>
-      <c r="H40" s="2" t="s">
+      <c r="G40" s="2"/>
+      <c r="H40" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="I40" s="2" t="s">
+      <c r="I40" s="3" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="A41" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="B41" s="0" t="s">
+      <c r="B41" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="E41" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="F41" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="G41" s="1"/>
-      <c r="H41" s="2" t="s">
+      <c r="G41" s="2"/>
+      <c r="H41" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="I41" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="A42" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B42" s="0" t="s">
+      <c r="B42" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E42" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F42" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="G42" s="1"/>
-      <c r="H42" s="2" t="s">
+      <c r="G42" s="2"/>
+      <c r="H42" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="I42" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
+      <c r="A43" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="B43" s="0" t="s">
+      <c r="B43" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="F43" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="G43" s="1"/>
-      <c r="H43" s="2" t="s">
+      <c r="G43" s="2"/>
+      <c r="H43" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="I43" s="3" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+      <c r="A44" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B44" s="0" t="s">
+      <c r="B44" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="E44" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="G44" s="1"/>
-      <c r="H44" s="2" t="s">
+      <c r="G44" s="2"/>
+      <c r="H44" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="I44" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+      <c r="A45" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="B45" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E45" s="0" t="s">
+      <c r="E45" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F45" s="0" t="s">
+      <c r="F45" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="H45" s="0" t="s">
+      <c r="H45" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="I45" s="0" t="s">
+      <c r="I45" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
+      <c r="A46" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B46" s="0" t="s">
+      <c r="B46" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F46" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="G46" s="1"/>
-      <c r="H46" s="2" t="s">
+      <c r="G46" s="2"/>
+      <c r="H46" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="I46" s="3" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+      <c r="A47" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B47" s="0" t="s">
+      <c r="B47" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="E47" s="1" t="s">
+      <c r="E47" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="F47" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="G47" s="1"/>
-      <c r="H47" s="2" t="s">
+      <c r="G47" s="2"/>
+      <c r="H47" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I47" s="2" t="s">
+      <c r="I47" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
+      <c r="A48" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="B48" s="0" t="s">
+      <c r="B48" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="E48" s="1" t="s">
+      <c r="E48" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="F48" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="H48" s="2" t="s">
+      <c r="H48" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="I48" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="J48" s="2" t="s">
+      <c r="J48" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="K48" s="2" t="s">
+      <c r="K48" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
+      <c r="A49" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="B49" s="0" t="s">
+      <c r="B49" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="F49" s="1" t="s">
+      <c r="F49" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="G49" s="1"/>
-      <c r="H49" s="2" t="s">
+      <c r="G49" s="2"/>
+      <c r="H49" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="I49" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
+      <c r="A50" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B50" s="0" t="s">
+      <c r="B50" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="E50" s="1" t="s">
+      <c r="E50" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F50" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="G50" s="4" t="s">
+      <c r="G50" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="H50" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="I50" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0" t="s">
+      <c r="A51" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="B51" s="0" t="s">
+      <c r="B51" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E51" s="1" t="s">
+      <c r="E51" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="F51" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="G51" s="1"/>
-      <c r="H51" s="2" t="s">
+      <c r="G51" s="2"/>
+      <c r="H51" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="I51" s="2" t="s">
+      <c r="I51" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
+      <c r="A52" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="B52" s="0" t="s">
+      <c r="B52" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="F52" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="G52" s="1"/>
-      <c r="H52" s="2" t="s">
+      <c r="G52" s="2"/>
+      <c r="H52" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="I52" s="2" t="s">
+      <c r="I52" s="3" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0" t="s">
+      <c r="A53" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B53" s="0" t="s">
+      <c r="B53" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E53" s="1" t="s">
+      <c r="E53" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="F53" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G53" s="1"/>
-      <c r="H53" s="2" t="s">
+      <c r="G53" s="2"/>
+      <c r="H53" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I53" s="2" t="s">
+      <c r="I53" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0" t="s">
+      <c r="A54" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="B54" s="0" t="s">
+      <c r="B54" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="E54" s="1" t="s">
+      <c r="E54" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="F54" s="1" t="s">
+      <c r="F54" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G54" s="1"/>
-      <c r="H54" s="2" t="s">
+      <c r="G54" s="2"/>
+      <c r="H54" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I54" s="2" t="s">
+      <c r="I54" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0" t="s">
+      <c r="A55" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="B55" s="0" t="s">
+      <c r="B55" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F55" s="1" t="s">
+      <c r="F55" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="G55" s="1"/>
-      <c r="H55" s="2" t="s">
+      <c r="G55" s="2"/>
+      <c r="H55" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="I55" s="2" t="s">
+      <c r="I55" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0" t="s">
+      <c r="A56" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="B56" s="0" t="s">
+      <c r="B56" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E56" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="F56" s="1" t="s">
+      <c r="F56" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="G56" s="1"/>
-      <c r="H56" s="2" t="s">
+      <c r="G56" s="2"/>
+      <c r="H56" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I56" s="2" t="s">
+      <c r="I56" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0" t="s">
+      <c r="A57" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="B57" s="0" t="s">
+      <c r="B57" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E57" s="1" t="s">
+      <c r="E57" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="F57" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="G57" s="1"/>
-      <c r="H57" s="2" t="s">
+      <c r="G57" s="2"/>
+      <c r="H57" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="I57" s="2" t="s">
+      <c r="I57" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0" t="s">
+      <c r="A58" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="B58" s="0" t="s">
+      <c r="B58" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="E58" s="1" t="s">
+      <c r="E58" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="F58" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="G58" s="1"/>
-      <c r="H58" s="2" t="s">
+      <c r="G58" s="2"/>
+      <c r="H58" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="I58" s="2" t="s">
+      <c r="I58" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0" t="s">
+      <c r="A59" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="B59" s="0" t="s">
+      <c r="B59" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="E59" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="F59" s="1" t="s">
+      <c r="F59" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="G59" s="1"/>
-      <c r="H59" s="2" t="s">
+      <c r="G59" s="2"/>
+      <c r="H59" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I59" s="2" t="s">
+      <c r="I59" s="3" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0" t="s">
+      <c r="A60" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B60" s="0" t="s">
+      <c r="B60" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="E60" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="F60" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="G60" s="1"/>
-      <c r="H60" s="2" t="s">
+      <c r="G60" s="2"/>
+      <c r="H60" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I60" s="2" t="s">
+      <c r="I60" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0" t="s">
+      <c r="A61" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="B61" s="0" t="s">
+      <c r="B61" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="F61" s="1" t="s">
+      <c r="F61" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="G61" s="1"/>
-      <c r="H61" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>28</v>
+      <c r="G61" s="2"/>
+      <c r="H61" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I61" s="8" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
+      <c r="A62" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B62" s="0" t="s">
+      <c r="B62" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="E62" s="1" t="s">
+      <c r="E62" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F62" s="1" t="s">
+      <c r="F62" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="G62" s="1"/>
-      <c r="H62" s="2" t="s">
+      <c r="G62" s="2"/>
+      <c r="H62" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I62" s="2" t="s">
+      <c r="I62" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
+      <c r="A63" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B63" s="0" t="s">
+      <c r="B63" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="E63" s="1" t="s">
+      <c r="E63" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="F63" s="1" t="s">
+      <c r="F63" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="G63" s="1"/>
-      <c r="H63" s="2" t="s">
+      <c r="G63" s="2"/>
+      <c r="H63" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="I63" s="2" t="s">
+      <c r="I63" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
+      <c r="A64" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B64" s="0" t="s">
+      <c r="B64" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="E64" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="F64" s="1" t="s">
+      <c r="F64" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="G64" s="1"/>
-      <c r="H64" s="2" t="s">
+      <c r="G64" s="2"/>
+      <c r="H64" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I64" s="2" t="s">
+      <c r="I64" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
+      <c r="A65" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="B65" s="0" t="s">
+      <c r="B65" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E65" s="1" t="s">
+      <c r="E65" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="F65" s="1" t="s">
+      <c r="F65" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="G65" s="1"/>
-      <c r="H65" s="2" t="s">
+      <c r="G65" s="2"/>
+      <c r="H65" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="I65" s="2" t="s">
+      <c r="I65" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="0" t="s">
+      <c r="A66" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B66" s="0" t="s">
+      <c r="B66" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="E66" s="1" t="s">
+      <c r="E66" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="F66" s="1" t="s">
+      <c r="F66" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="G66" s="1"/>
-      <c r="H66" s="2" t="s">
+      <c r="G66" s="2"/>
+      <c r="H66" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I66" s="2" t="s">
+      <c r="I66" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J66" s="2" t="s">
+      <c r="J66" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="K66" s="2" t="s">
+      <c r="K66" s="3" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="0" t="s">
+      <c r="A67" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="B67" s="0" t="s">
+      <c r="B67" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="E67" s="1" t="s">
+      <c r="E67" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="F67" s="1" t="s">
+      <c r="F67" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="G67" s="1"/>
-      <c r="H67" s="2" t="s">
+      <c r="G67" s="2"/>
+      <c r="H67" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I67" s="2" t="s">
+      <c r="I67" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
+      <c r="A68" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="B68" s="0" t="s">
+      <c r="B68" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="E68" s="1" t="s">
+      <c r="E68" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="F68" s="1" t="s">
+      <c r="F68" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="G68" s="1"/>
-      <c r="H68" s="2" t="s">
+      <c r="G68" s="2"/>
+      <c r="H68" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I68" s="2" t="s">
+      <c r="I68" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="s">
+      <c r="A69" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="B69" s="0" t="s">
+      <c r="B69" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="E69" s="1" t="s">
+      <c r="E69" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="F69" s="1" t="s">
+      <c r="F69" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="G69" s="1"/>
-      <c r="H69" s="2" t="s">
+      <c r="G69" s="2"/>
+      <c r="H69" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I69" s="2" t="s">
+      <c r="I69" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="0" t="s">
+      <c r="A70" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="B70" s="0" t="s">
+      <c r="B70" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="E70" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="F70" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="G70" s="1"/>
-      <c r="H70" s="2" t="s">
+      <c r="G70" s="2"/>
+      <c r="H70" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I70" s="2" t="s">
+      <c r="I70" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0" t="s">
+      <c r="A71" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B71" s="0" t="s">
+      <c r="B71" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="E71" s="1" t="s">
+      <c r="E71" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="F71" s="1" t="s">
+      <c r="F71" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="G71" s="1"/>
-      <c r="H71" s="2" t="s">
+      <c r="G71" s="2"/>
+      <c r="H71" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="I71" s="2" t="s">
+      <c r="I71" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
+      <c r="A72" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="B72" s="0" t="s">
+      <c r="B72" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E72" s="1" t="s">
+      <c r="E72" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="F72" s="1" t="s">
+      <c r="F72" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="G72" s="1"/>
-      <c r="H72" s="2" t="s">
+      <c r="G72" s="2"/>
+      <c r="H72" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I72" s="2" t="s">
+      <c r="I72" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="s">
+      <c r="A73" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B73" s="0" t="s">
+      <c r="B73" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="E73" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="F73" s="1" t="s">
+      <c r="F73" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="G73" s="1"/>
-      <c r="H73" s="2" t="s">
+      <c r="G73" s="2"/>
+      <c r="H73" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I73" s="2" t="s">
+      <c r="I73" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0" t="s">
+      <c r="A74" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B74" s="0" t="s">
+      <c r="B74" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E74" s="1" t="s">
+      <c r="E74" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="F74" s="1" t="s">
+      <c r="F74" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="G74" s="1"/>
-      <c r="H74" s="2" t="s">
+      <c r="G74" s="2"/>
+      <c r="H74" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="I74" s="2" t="s">
+      <c r="I74" s="3" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0" t="s">
+      <c r="A75" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="B75" s="0" t="s">
+      <c r="B75" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="E75" s="1" t="s">
+      <c r="E75" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="F75" s="1" t="s">
+      <c r="F75" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="G75" s="1"/>
-      <c r="H75" s="2" t="s">
+      <c r="G75" s="2"/>
+      <c r="H75" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I75" s="2" t="s">
+      <c r="I75" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="0" t="s">
+      <c r="A76" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="B76" s="0" t="s">
+      <c r="B76" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="E76" s="1" t="s">
+      <c r="E76" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="2" t="s">
+      <c r="F76" s="2"/>
+      <c r="G76" s="2"/>
+      <c r="H76" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="I76" s="2" t="s">
+      <c r="I76" s="3" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0" t="s">
+      <c r="A77" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B77" s="0" t="s">
+      <c r="B77" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E77" s="1" t="s">
+      <c r="E77" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="F77" s="1" t="s">
+      <c r="F77" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="G77" s="1"/>
-      <c r="H77" s="2" t="s">
+      <c r="G77" s="2"/>
+      <c r="H77" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="I77" s="2" t="s">
+      <c r="I77" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0" t="s">
+      <c r="A78" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="B78" s="0" t="s">
+      <c r="B78" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E78" s="1" t="s">
+      <c r="E78" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="F78" s="1" t="s">
+      <c r="F78" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="G78" s="1"/>
-      <c r="H78" s="2" t="s">
+      <c r="G78" s="2"/>
+      <c r="H78" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I78" s="2" t="s">
+      <c r="I78" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0" t="s">
+      <c r="A79" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="B79" s="0" t="s">
+      <c r="B79" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E79" s="1" t="s">
+      <c r="E79" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="F79" s="1" t="s">
+      <c r="F79" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="G79" s="1"/>
-      <c r="H79" s="2" t="s">
+      <c r="G79" s="2"/>
+      <c r="H79" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I79" s="2" t="s">
+      <c r="I79" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0" t="s">
+      <c r="A80" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="B80" s="0" t="s">
+      <c r="B80" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="E80" s="1" t="s">
+      <c r="E80" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="F80" s="1" t="s">
+      <c r="F80" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="G80" s="1"/>
-      <c r="H80" s="2" t="s">
+      <c r="G80" s="2"/>
+      <c r="H80" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I80" s="2" t="s">
+      <c r="I80" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0" t="s">
+      <c r="A81" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="B81" s="0" t="s">
+      <c r="B81" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="E81" s="1" t="s">
+      <c r="E81" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="F81" s="1" t="s">
+      <c r="F81" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="G81" s="1"/>
-      <c r="H81" s="2" t="s">
+      <c r="G81" s="2"/>
+      <c r="H81" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I81" s="2" t="s">
+      <c r="I81" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="0" t="s">
+      <c r="A82" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="B82" s="0" t="s">
+      <c r="B82" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="E82" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="F82" s="1" t="s">
+      <c r="F82" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="G82" s="1"/>
-      <c r="H82" s="2" t="s">
+      <c r="G82" s="2"/>
+      <c r="H82" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="I82" s="2" t="s">
+      <c r="I82" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J82" s="2" t="s">
+      <c r="J82" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K82" s="2" t="s">
+      <c r="K82" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="0" t="s">
+      <c r="A83" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="B83" s="0" t="s">
+      <c r="B83" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E83" s="1" t="s">
+      <c r="E83" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="F83" s="1" t="s">
+      <c r="F83" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="G83" s="1"/>
-      <c r="H83" s="2" t="s">
+      <c r="G83" s="2"/>
+      <c r="H83" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="I83" s="2" t="s">
+      <c r="I83" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="0" t="s">
+      <c r="A84" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="B84" s="0" t="s">
+      <c r="B84" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="E84" s="1" t="s">
+      <c r="E84" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="F84" s="1" t="s">
+      <c r="F84" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="G84" s="3" t="n">
+      <c r="G84" s="4" t="n">
         <v>45718</v>
       </c>
-      <c r="H84" s="2" t="s">
+      <c r="H84" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="I84" s="2" t="s">
+      <c r="I84" s="3" t="s">
         <v>364</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="0" t="s">
+      <c r="A85" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="B85" s="0" t="s">
+      <c r="B85" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="C85" s="0" t="s">
+      <c r="C85" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="E85" s="1" t="s">
+      <c r="E85" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="F85" s="1" t="s">
+      <c r="F85" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="G85" s="3" t="n">
+      <c r="G85" s="4" t="n">
         <v>45779</v>
       </c>
-      <c r="H85" s="2" t="s">
+      <c r="H85" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I85" s="2" t="s">
+      <c r="I85" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="K85" s="2" t="s">
+      <c r="K85" s="3" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="0" t="s">
+      <c r="A86" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="B86" s="0" t="s">
+      <c r="B86" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="C86" s="0" t="s">
+      <c r="C86" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="E86" s="1" t="s">
+      <c r="E86" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="F86" s="1" t="s">
+      <c r="F86" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="G86" s="3" t="n">
+      <c r="G86" s="4" t="n">
         <v>45779</v>
       </c>
-      <c r="H86" s="2" t="s">
+      <c r="H86" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I86" s="2" t="s">
+      <c r="I86" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="0" t="s">
+      <c r="A87" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="B87" s="0" t="s">
+      <c r="B87" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E87" s="1" t="s">
+      <c r="E87" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="F87" s="1" t="s">
+      <c r="F87" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="G87" s="1"/>
-      <c r="H87" s="2" t="s">
+      <c r="G87" s="2"/>
+      <c r="H87" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="I87" s="2" t="s">
+      <c r="I87" s="3" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="0" t="s">
+      <c r="A88" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="B88" s="0" t="s">
+      <c r="B88" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E88" s="1" t="s">
+      <c r="E88" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="F88" s="1" t="s">
+      <c r="F88" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="G88" s="1"/>
-      <c r="H88" s="2" t="s">
+      <c r="G88" s="2"/>
+      <c r="H88" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I88" s="2" t="s">
+      <c r="I88" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0" t="s">
+      <c r="A89" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B89" s="0" t="s">
+      <c r="B89" s="1" t="s">
         <v>381</v>
       </c>
-      <c r="E89" s="1" t="s">
+      <c r="E89" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="F89" s="1" t="s">
+      <c r="F89" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="G89" s="1"/>
-      <c r="H89" s="2" t="s">
+      <c r="G89" s="2"/>
+      <c r="H89" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="I89" s="2" t="s">
+      <c r="I89" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="0" t="s">
+      <c r="A90" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B90" s="0" t="s">
+      <c r="B90" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="E90" s="1" t="s">
+      <c r="E90" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="F90" s="1" t="s">
+      <c r="F90" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="G90" s="1"/>
-      <c r="H90" s="2" t="s">
+      <c r="G90" s="2"/>
+      <c r="H90" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I90" s="2" t="s">
+      <c r="I90" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="0" t="s">
+      <c r="A91" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="B91" s="0" t="s">
+      <c r="B91" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E91" s="1" t="s">
+      <c r="E91" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="F91" s="1" t="s">
+      <c r="F91" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="G91" s="1"/>
-      <c r="H91" s="2" t="s">
+      <c r="G91" s="2"/>
+      <c r="H91" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I91" s="2" t="s">
+      <c r="I91" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J91" s="2" t="s">
+      <c r="J91" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="K91" s="2" t="s">
+      <c r="K91" s="3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="0" t="s">
+      <c r="A92" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="B92" s="0" t="s">
+      <c r="B92" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="E92" s="1" t="s">
+      <c r="E92" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="F92" s="1" t="s">
+      <c r="F92" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="G92" s="1"/>
-      <c r="H92" s="2" t="s">
+      <c r="G92" s="2"/>
+      <c r="H92" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="I92" s="2" t="s">
+      <c r="I92" s="3" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="0" t="s">
+      <c r="A93" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="B93" s="0" t="s">
+      <c r="B93" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="E93" s="1" t="s">
+      <c r="E93" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="F93" s="1" t="s">
+      <c r="F93" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="G93" s="1"/>
-      <c r="H93" s="2" t="s">
+      <c r="G93" s="2"/>
+      <c r="H93" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="I93" s="2" t="s">
+      <c r="I93" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="0" t="s">
+      <c r="A94" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="B94" s="0" t="s">
+      <c r="B94" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="E94" s="1" t="s">
+      <c r="E94" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="F94" s="1"/>
-      <c r="G94" s="1"/>
-      <c r="H94" s="2" t="s">
+      <c r="F94" s="2"/>
+      <c r="G94" s="2"/>
+      <c r="H94" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I94" s="2" t="s">
+      <c r="I94" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="0" t="s">
+      <c r="A95" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="B95" s="0" t="s">
+      <c r="B95" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E95" s="1" t="s">
+      <c r="E95" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="F95" s="1" t="s">
+      <c r="F95" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="G95" s="1"/>
-      <c r="H95" s="2" t="s">
+      <c r="G95" s="2"/>
+      <c r="H95" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I95" s="2" t="s">
+      <c r="I95" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="0" t="s">
+      <c r="A96" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B96" s="0" t="s">
+      <c r="B96" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="E96" s="1" t="s">
+      <c r="E96" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="F96" s="1" t="s">
+      <c r="F96" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="G96" s="1"/>
-      <c r="H96" s="2" t="s">
+      <c r="G96" s="2"/>
+      <c r="H96" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I96" s="2" t="s">
+      <c r="I96" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J96" s="2" t="s">
+      <c r="J96" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="K96" s="2" t="s">
+      <c r="K96" s="3" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="0" t="s">
+      <c r="A97" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B97" s="0" t="s">
+      <c r="B97" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="E97" s="1" t="s">
+      <c r="E97" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="F97" s="1" t="s">
+      <c r="F97" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="G97" s="1"/>
-      <c r="H97" s="2" t="s">
+      <c r="G97" s="2"/>
+      <c r="H97" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I97" s="2" t="s">
+      <c r="I97" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="0" t="s">
+      <c r="A98" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="B98" s="0" t="s">
+      <c r="B98" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E98" s="1" t="s">
+      <c r="E98" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="F98" s="1" t="s">
+      <c r="F98" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="G98" s="1"/>
-      <c r="H98" s="2" t="s">
+      <c r="G98" s="2"/>
+      <c r="H98" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I98" s="2" t="s">
+      <c r="I98" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="0" t="s">
+      <c r="A99" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B99" s="0" t="s">
+      <c r="B99" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="E99" s="1" t="s">
+      <c r="E99" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="F99" s="1"/>
-      <c r="G99" s="1"/>
-      <c r="H99" s="2" t="s">
+      <c r="F99" s="2"/>
+      <c r="G99" s="2"/>
+      <c r="H99" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I99" s="2" t="s">
+      <c r="I99" s="3" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="0" t="s">
+      <c r="A100" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="B100" s="0" t="s">
+      <c r="B100" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E100" s="1" t="s">
+      <c r="E100" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="F100" s="1" t="s">
+      <c r="F100" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="G100" s="1"/>
-      <c r="H100" s="2" t="s">
+      <c r="G100" s="2"/>
+      <c r="H100" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I100" s="2" t="s">
+      <c r="I100" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="0" t="s">
+      <c r="A101" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B101" s="0" t="s">
+      <c r="B101" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="E101" s="1" t="s">
+      <c r="E101" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="F101" s="1" t="s">
+      <c r="F101" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="G101" s="1"/>
-      <c r="H101" s="2" t="s">
+      <c r="G101" s="2"/>
+      <c r="H101" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I101" s="2" t="s">
+      <c r="I101" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="0" t="s">
+      <c r="A102" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="B102" s="0" t="s">
+      <c r="B102" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="E102" s="1" t="s">
+      <c r="E102" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="F102" s="1" t="s">
+      <c r="F102" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="G102" s="1"/>
-      <c r="H102" s="2" t="s">
+      <c r="G102" s="2"/>
+      <c r="H102" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I102" s="2" t="s">
+      <c r="I102" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="0" t="s">
+      <c r="A103" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="B103" s="0" t="s">
+      <c r="B103" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E103" s="1" t="s">
+      <c r="E103" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="F103" s="1" t="s">
+      <c r="F103" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="G103" s="1"/>
-      <c r="H103" s="2" t="s">
+      <c r="G103" s="2"/>
+      <c r="H103" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I103" s="2" t="s">
+      <c r="I103" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="0" t="s">
+      <c r="A104" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="B104" s="0" t="s">
+      <c r="B104" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="E104" s="1" t="s">
+      <c r="E104" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="F104" s="1" t="s">
+      <c r="F104" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="G104" s="4" t="s">
+      <c r="G104" s="5" t="s">
         <v>431</v>
       </c>
-      <c r="H104" s="2" t="s">
+      <c r="H104" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I104" s="2" t="s">
+      <c r="I104" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J104" s="2" t="s">
+      <c r="J104" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="K104" s="2" t="s">
+      <c r="K104" s="3" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="0" t="s">
+      <c r="A105" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="B105" s="0" t="s">
+      <c r="B105" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E105" s="1" t="s">
+      <c r="E105" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="F105" s="1" t="s">
+      <c r="F105" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="G105" s="1"/>
-      <c r="H105" s="2" t="s">
+      <c r="G105" s="2"/>
+      <c r="H105" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I105" s="2" t="s">
+      <c r="I105" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="0" t="s">
+      <c r="A106" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="B106" s="0" t="s">
+      <c r="B106" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="E106" s="1" t="s">
+      <c r="E106" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="F106" s="1"/>
-      <c r="G106" s="1"/>
-      <c r="H106" s="2" t="s">
+      <c r="F106" s="2"/>
+      <c r="G106" s="2"/>
+      <c r="H106" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I106" s="2" t="s">
+      <c r="I106" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J106" s="2" t="s">
+      <c r="J106" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="K106" s="2" t="s">
+      <c r="K106" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="0" t="s">
+      <c r="A107" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="B107" s="0" t="s">
+      <c r="B107" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E107" s="1" t="s">
+      <c r="E107" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="F107" s="1" t="s">
+      <c r="F107" s="2" t="s">
         <v>442</v>
       </c>
-      <c r="G107" s="1"/>
-      <c r="H107" s="2" t="s">
+      <c r="G107" s="2"/>
+      <c r="H107" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="I107" s="2" t="s">
+      <c r="I107" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="0" t="s">
+      <c r="A108" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="B108" s="0" t="s">
+      <c r="B108" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E108" s="1" t="s">
+      <c r="E108" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="F108" s="1" t="s">
+      <c r="F108" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="G108" s="1"/>
-      <c r="H108" s="2" t="s">
+      <c r="G108" s="2"/>
+      <c r="H108" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I108" s="2" t="s">
+      <c r="I108" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J108" s="2" t="s">
+      <c r="J108" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="K108" s="2" t="s">
+      <c r="K108" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="0" t="s">
+      <c r="A109" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="B109" s="0" t="s">
+      <c r="B109" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="E109" s="1" t="s">
+      <c r="E109" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="F109" s="1" t="s">
+      <c r="F109" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="G109" s="1"/>
-      <c r="H109" s="2" t="s">
+      <c r="G109" s="2"/>
+      <c r="H109" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="I109" s="2" t="s">
+      <c r="I109" s="3" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="0" t="s">
+      <c r="A110" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="B110" s="0" t="s">
+      <c r="B110" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="E110" s="1" t="s">
+      <c r="E110" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="F110" s="1" t="s">
+      <c r="F110" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="G110" s="1"/>
-      <c r="H110" s="2" t="s">
+      <c r="G110" s="2"/>
+      <c r="H110" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="I110" s="2" t="s">
+      <c r="I110" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="7" t="s">
+      <c r="A111" s="9" t="s">
         <v>455</v>
       </c>
-      <c r="B111" s="2" t="s">
+      <c r="B111" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="E111" s="1" t="s">
+      <c r="E111" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="F111" s="1" t="s">
+      <c r="F111" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="G111" s="1"/>
-      <c r="H111" s="2" t="s">
+      <c r="G111" s="2"/>
+      <c r="H111" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I111" s="2" t="s">
+      <c r="I111" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="0" t="s">
+      <c r="A112" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="B112" s="0" t="s">
+      <c r="B112" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="E112" s="1" t="s">
+      <c r="E112" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="F112" s="1" t="s">
+      <c r="F112" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="G112" s="1"/>
-      <c r="H112" s="2" t="s">
+      <c r="G112" s="2"/>
+      <c r="H112" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="I112" s="2" t="s">
+      <c r="I112" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="0" t="s">
+      <c r="A113" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="B113" s="0" t="s">
+      <c r="B113" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E113" s="1" t="s">
+      <c r="E113" s="2" t="s">
         <v>464</v>
       </c>
-      <c r="F113" s="1" t="s">
+      <c r="F113" s="2" t="s">
         <v>465</v>
       </c>
-      <c r="G113" s="1"/>
-      <c r="H113" s="2" t="s">
+      <c r="G113" s="2"/>
+      <c r="H113" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I113" s="2" t="s">
+      <c r="I113" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J113" s="2" t="s">
+      <c r="J113" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="K113" s="2" t="s">
+      <c r="K113" s="3" t="s">
         <v>72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Last active date for S. Ayet
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="467">
   <si>
     <t xml:space="preserve">LastName</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://orcid.org/0000-0002-0053-1691</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31/08/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Instituto de F\'isica Corpuscular (IFIC), CSIC \&amp; Universitat de Val\`encia, Calle Catedr\'atico Jos\'e Beltr\'an, 2 </t>
@@ -1429,7 +1432,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1466,12 +1469,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1526,7 +1523,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1560,10 +1557,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1824,7 +1817,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="112.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="112.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1982,68 +1975,70 @@
       <c r="F7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="2"/>
+      <c r="G7" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="H7" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="3" t="s">
@@ -2055,19 +2050,19 @@
     </row>
     <row r="11" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>15</v>
@@ -2078,16 +2073,16 @@
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>15</v>
@@ -2096,24 +2091,24 @@
         <v>16</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="3" t="s">
@@ -2125,40 +2120,40 @@
     </row>
     <row r="14" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>15</v>
@@ -2167,7 +2162,7 @@
         <v>16</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>16</v>
@@ -2175,37 +2170,37 @@
     </row>
     <row r="16" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>15</v>
@@ -2216,16 +2211,16 @@
     </row>
     <row r="18" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>46174</v>
@@ -2239,109 +2234,109 @@
     </row>
     <row r="19" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G19" s="4"/>
       <c r="H19" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="3" t="s">
@@ -2353,61 +2348,61 @@
     </row>
     <row r="24" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>15</v>
@@ -2418,13 +2413,13 @@
     </row>
     <row r="27" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="7" t="n">
@@ -2439,16 +2434,16 @@
     </row>
     <row r="28" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>15</v>
@@ -2457,24 +2452,24 @@
         <v>16</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>21</v>
@@ -2485,19 +2480,19 @@
     </row>
     <row r="30" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>45779</v>
@@ -2506,48 +2501,48 @@
         <v>27</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>15</v>
@@ -2556,25 +2551,25 @@
         <v>16</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>15</v>
@@ -2585,62 +2580,62 @@
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>16</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>21</v>
@@ -2651,19 +2646,19 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H37" s="1" t="s">
         <v>15</v>
@@ -2672,150 +2667,150 @@
         <v>16</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G40" s="2"/>
       <c r="H40" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G43" s="2"/>
       <c r="H43" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="3" t="s">
@@ -2827,128 +2822,128 @@
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G47" s="2"/>
       <c r="H47" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>36</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>15</v>
@@ -2959,16 +2954,16 @@
     </row>
     <row r="51" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="3" t="s">
@@ -2980,37 +2975,37 @@
     </row>
     <row r="52" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G52" s="2"/>
       <c r="H52" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>36</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G53" s="2"/>
       <c r="H53" s="3" t="s">
@@ -3022,79 +3017,79 @@
     </row>
     <row r="54" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G54" s="2"/>
       <c r="H54" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G55" s="2"/>
       <c r="H55" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G56" s="2"/>
       <c r="H56" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G57" s="2"/>
       <c r="H57" s="3" t="s">
@@ -3106,58 +3101,58 @@
     </row>
     <row r="58" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G58" s="2"/>
       <c r="H58" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G59" s="2"/>
       <c r="H59" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G60" s="2"/>
       <c r="H60" s="3" t="s">
@@ -3169,100 +3164,100 @@
     </row>
     <row r="61" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G61" s="2"/>
-      <c r="H61" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="I61" s="8" t="s">
-        <v>272</v>
+      <c r="H61" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G62" s="2"/>
       <c r="H62" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G63" s="2"/>
       <c r="H63" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="G64" s="2"/>
       <c r="H64" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G65" s="2"/>
       <c r="H65" s="3" t="s">
@@ -3274,16 +3269,16 @@
     </row>
     <row r="66" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G66" s="2"/>
       <c r="H66" s="3" t="s">
@@ -3293,45 +3288,45 @@
         <v>16</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K66" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G67" s="2"/>
       <c r="H67" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G68" s="2"/>
       <c r="H68" s="3" t="s">
@@ -3343,79 +3338,79 @@
     </row>
     <row r="69" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G69" s="2"/>
       <c r="H69" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G70" s="2"/>
       <c r="H70" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G71" s="2"/>
       <c r="H71" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="3" t="s">
@@ -3427,102 +3422,102 @@
     </row>
     <row r="73" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G73" s="2"/>
       <c r="H73" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G74" s="2"/>
       <c r="H74" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G75" s="2"/>
       <c r="H75" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
       <c r="H76" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G77" s="2"/>
       <c r="H77" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I77" s="3" t="s">
         <v>16</v>
@@ -3530,16 +3525,16 @@
     </row>
     <row r="78" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G78" s="2"/>
       <c r="H78" s="3" t="s">
@@ -3551,79 +3546,79 @@
     </row>
     <row r="79" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G79" s="2"/>
       <c r="H79" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G80" s="2"/>
       <c r="H80" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G81" s="2"/>
       <c r="H81" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G82" s="2"/>
       <c r="H82" s="3" t="s">
@@ -3641,20 +3636,20 @@
     </row>
     <row r="83" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G83" s="2"/>
       <c r="H83" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I83" s="3" t="s">
         <v>16</v>
@@ -3662,42 +3657,42 @@
     </row>
     <row r="84" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G84" s="4" t="n">
         <v>45718</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G85" s="4" t="n">
         <v>45779</v>
@@ -3709,131 +3704,131 @@
         <v>16</v>
       </c>
       <c r="K85" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G86" s="4" t="n">
         <v>45779</v>
       </c>
       <c r="H86" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G87" s="2"/>
       <c r="H87" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G88" s="2"/>
       <c r="H88" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G89" s="2"/>
       <c r="H89" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F90" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G90" s="2"/>
       <c r="H90" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G91" s="2"/>
       <c r="H91" s="3" t="s">
@@ -3843,106 +3838,106 @@
         <v>16</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K91" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G92" s="2"/>
       <c r="H92" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G93" s="2"/>
       <c r="H93" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
       <c r="H94" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="G95" s="2"/>
       <c r="H95" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I95" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G96" s="2"/>
       <c r="H96" s="3" t="s">
@@ -3952,106 +3947,106 @@
         <v>16</v>
       </c>
       <c r="J96" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K96" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G97" s="2"/>
       <c r="H97" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F98" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G98" s="2"/>
       <c r="H98" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I98" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
       <c r="H99" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I99" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F100" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G100" s="2"/>
       <c r="H100" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I100" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="G101" s="2"/>
       <c r="H101" s="3" t="s">
@@ -4063,16 +4058,16 @@
     </row>
     <row r="102" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G102" s="2"/>
       <c r="H102" s="3" t="s">
@@ -4084,16 +4079,16 @@
     </row>
     <row r="103" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G103" s="2"/>
       <c r="H103" s="3" t="s">
@@ -4105,19 +4100,19 @@
     </row>
     <row r="104" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G104" s="5" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="H104" s="3" t="s">
         <v>15</v>
@@ -4126,42 +4121,42 @@
         <v>16</v>
       </c>
       <c r="J104" s="3" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K104" s="3" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G105" s="2"/>
       <c r="H105" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I105" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
@@ -4172,7 +4167,7 @@
         <v>16</v>
       </c>
       <c r="J106" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K106" s="3" t="s">
         <v>16</v>
@@ -4180,37 +4175,37 @@
     </row>
     <row r="107" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G107" s="2"/>
       <c r="H107" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G108" s="2"/>
       <c r="H108" s="3" t="s">
@@ -4220,108 +4215,108 @@
         <v>16</v>
       </c>
       <c r="J108" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K108" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G109" s="2"/>
       <c r="H109" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I109" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G110" s="2"/>
       <c r="H110" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="9" t="s">
-        <v>455</v>
+      <c r="A111" s="8" t="s">
+        <v>456</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G111" s="2"/>
       <c r="H111" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I111" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="G112" s="2"/>
       <c r="H112" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I112" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G113" s="2"/>
       <c r="H113" s="3" t="s">
@@ -4331,10 +4326,10 @@
         <v>16</v>
       </c>
       <c r="J113" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K113" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates in UoM, IFIC and UPV
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="471">
   <si>
     <t xml:space="preserve">LastName</t>
   </si>
@@ -1325,6 +1325,18 @@
   </si>
   <si>
     <t xml:space="preserve"> Girona, E-17071, Spain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Torres-Curado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rutorcu@upv.es</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://orcid.org/0000-0002-7621-5804</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instituto de Instrumentaci\'on para Imagen Molecular (I3M), Centro Mixto CSIC - Universitat Polit\`ecnica de Val\`encia, Camino de Vera s/n</t>
   </si>
   <si>
     <t xml:space="preserve">Trettin</t>
@@ -1432,7 +1444,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1469,6 +1481,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1523,7 +1548,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1556,7 +1581,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1810,14 +1843,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K114"/>
   <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="20.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="112.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="125.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="56.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="100.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="29.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2686,7 +2722,9 @@
       <c r="F38" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="G38" s="2"/>
+      <c r="G38" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H38" s="3" t="s">
         <v>125</v>
       </c>
@@ -2921,7 +2959,9 @@
       <c r="F49" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="G49" s="2"/>
+      <c r="G49" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H49" s="3" t="s">
         <v>45</v>
       </c>
@@ -3966,7 +4006,9 @@
       <c r="F97" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="G97" s="2"/>
+      <c r="G97" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H97" s="3" t="s">
         <v>45</v>
       </c>
@@ -4127,106 +4169,104 @@
         <v>434</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
         <v>435</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="F105" s="2" t="s">
+      <c r="F105" s="8" t="s">
         <v>437</v>
       </c>
-      <c r="G105" s="2"/>
-      <c r="H105" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="I105" s="3" t="s">
-        <v>126</v>
-      </c>
+      <c r="G105" s="5"/>
+      <c r="H105" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="I105" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="J105" s="3"/>
+      <c r="K105" s="3"/>
     </row>
     <row r="106" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>439</v>
+        <v>85</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="F106" s="2"/>
-      <c r="G106" s="2"/>
+      <c r="F106" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="G106" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H106" s="3" t="s">
-        <v>15</v>
+        <v>125</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J106" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="K106" s="3" t="s">
-        <v>16</v>
+        <v>126</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>69</v>
+        <v>443</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="F107" s="2" t="s">
-        <v>443</v>
-      </c>
+        <v>444</v>
+      </c>
+      <c r="F107" s="2"/>
       <c r="G107" s="2"/>
       <c r="H107" s="3" t="s">
-        <v>172</v>
+        <v>15</v>
       </c>
       <c r="I107" s="3" t="s">
-        <v>132</v>
+        <v>16</v>
+      </c>
+      <c r="J107" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="K107" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>134</v>
+        <v>69</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="G108" s="2"/>
       <c r="H108" s="3" t="s">
-        <v>15</v>
+        <v>172</v>
       </c>
       <c r="I108" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J108" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="K108" s="3" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>448</v>
+        <v>134</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>449</v>
@@ -4236,38 +4276,44 @@
       </c>
       <c r="G109" s="2"/>
       <c r="H109" s="3" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="I109" s="3" t="s">
-        <v>451</v>
+        <v>16</v>
+      </c>
+      <c r="J109" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K109" s="3" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B110" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="E110" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="E110" s="2" t="s">
+      <c r="F110" s="2" t="s">
         <v>454</v>
-      </c>
-      <c r="F110" s="2" t="s">
-        <v>455</v>
       </c>
       <c r="G110" s="2"/>
       <c r="H110" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="I110" s="3" t="s">
-        <v>46</v>
+        <v>455</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="8" t="s">
+      <c r="A111" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="B111" s="3" t="s">
+      <c r="B111" s="1" t="s">
         <v>457</v>
       </c>
       <c r="E111" s="2" t="s">
@@ -4278,17 +4324,17 @@
       </c>
       <c r="G111" s="2"/>
       <c r="H111" s="3" t="s">
-        <v>125</v>
+        <v>45</v>
       </c>
       <c r="I111" s="3" t="s">
-        <v>126</v>
+        <v>46</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="1" t="s">
+      <c r="A112" s="10" t="s">
         <v>460</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="B112" s="3" t="s">
         <v>461</v>
       </c>
       <c r="E112" s="2" t="s">
@@ -4297,7 +4343,9 @@
       <c r="F112" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="G112" s="2"/>
+      <c r="G112" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H112" s="3" t="s">
         <v>125</v>
       </c>
@@ -4310,25 +4358,46 @@
         <v>464</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>85</v>
+        <v>465</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="G113" s="2"/>
       <c r="H113" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I113" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="G114" s="2"/>
+      <c r="H114" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I113" s="3" t="s">
+      <c r="I114" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J113" s="3" t="s">
+      <c r="J114" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K113" s="3" t="s">
+      <c r="K114" s="3" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4437,17 +4506,18 @@
     <hyperlink ref="E102" r:id="rId101" display="claire.tonnele@dipc.org"/>
     <hyperlink ref="E103" r:id="rId102" display="samuele.torelli@dipc.org"/>
     <hyperlink ref="E104" r:id="rId103" display="jordi.torrent@udg.edu"/>
-    <hyperlink ref="E105" r:id="rId104" display="alexandra.trettin@manchester.ac.uk"/>
-    <hyperlink ref="E106" r:id="rId105" display="pablo.garcia@dipc.org"/>
-    <hyperlink ref="E107" r:id="rId106" display="mukundam.vanga@uta.edu"/>
-    <hyperlink ref="E108" r:id="rId107" display="pablo.vazquez@dipc.org"/>
-    <hyperlink ref="F108" r:id="rId108" display="https://orcid.org/0009-0007-0098-8927"/>
-    <hyperlink ref="E109" r:id="rId109" display="joao.veloso@ua.pt"/>
-    <hyperlink ref="E110" r:id="rId110" display="Juan.Villamil@ific.uv.es"/>
-    <hyperlink ref="E111" r:id="rId111" display="luismiguel.villarpadruno@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="F111" r:id="rId112" display="https://orcid.org/0009-0002-5335-0891"/>
-    <hyperlink ref="E112" r:id="rId113" display="john.waiton@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="E113" r:id="rId114" display="alfonso.yubero@dipc.org"/>
+    <hyperlink ref="F105" r:id="rId104" display="https://orcid.org/0000-0002-7621-5804"/>
+    <hyperlink ref="E106" r:id="rId105" display="alexandra.trettin@manchester.ac.uk"/>
+    <hyperlink ref="E107" r:id="rId106" display="pablo.garcia@dipc.org"/>
+    <hyperlink ref="E108" r:id="rId107" display="mukundam.vanga@uta.edu"/>
+    <hyperlink ref="E109" r:id="rId108" display="pablo.vazquez@dipc.org"/>
+    <hyperlink ref="F109" r:id="rId109" display="https://orcid.org/0009-0007-0098-8927"/>
+    <hyperlink ref="E110" r:id="rId110" display="joao.veloso@ua.pt"/>
+    <hyperlink ref="E111" r:id="rId111" display="Juan.Villamil@ific.uv.es"/>
+    <hyperlink ref="E112" r:id="rId112" display="luismiguel.villarpadruno@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="F112" r:id="rId113" display="https://orcid.org/0009-0002-5335-0891"/>
+    <hyperlink ref="E113" r:id="rId114" display="john.waiton@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="E114" r:id="rId115" display="alfonso.yubero@dipc.org"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Updates from Coimbra group
</commit_message>
<xml_diff>
--- a/AuthorList.xlsx
+++ b/AuthorList.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="454">
   <si>
     <t xml:space="preserve">LastName</t>
   </si>
@@ -622,18 +622,6 @@
     <t xml:space="preserve"> Ames, IA 50011-3160, USA</t>
   </si>
   <si>
-    <t xml:space="preserve">Henriques                   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">C.A.O.     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">henriques@uc.pt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0002-1218-181X</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hernando~Morata             </t>
   </si>
   <si>
@@ -694,18 +682,6 @@
     <t xml:space="preserve">https://orcid.org/0000-0002-6876-8089</t>
   </si>
   <si>
-    <t xml:space="preserve">Isabel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A.F.B.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">afbisabel@fis.uc.pt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0001-8025-8375</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jones                       </t>
   </si>
   <si>
@@ -796,18 +772,6 @@
     <t xml:space="preserve">https://orcid.org/0009-0003-0256-052X</t>
   </si>
   <si>
-    <t xml:space="preserve">Mano                        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">R.D.P.     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">rdpmano@uc.pt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://orcid.org/0000-0003-2920-7067</t>
-  </si>
-  <si>
     <t xml:space="preserve">Marauri</t>
   </si>
   <si>
@@ -1216,12 +1180,6 @@
     <t xml:space="preserve">https://orcid.org/0000-0002-8363-0109</t>
   </si>
   <si>
-    <t xml:space="preserve">P.A.O.C.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pesilva@uc.pt</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sim\'on                     </t>
   </si>
   <si>
@@ -1259,15 +1217,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://orcid.org/0000-0001-6804-9810</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teixeira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J.M.R.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jmrt@uc.pt</t>
   </si>
   <si>
     <t xml:space="preserve">Teruel-Pardo</t>
@@ -1444,7 +1393,7 @@
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1488,12 +1437,7 @@
       <color theme="10"/>
       <name val="Courier New"/>
       <family val="3"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1548,7 +1492,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1586,10 +1530,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1843,7 +1783,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K1048576"/>
   <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.71"/>
@@ -1851,9 +1791,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="33.36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="36.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="125.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="56.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="100.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="29.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="56.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="100.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="29.64"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2789,10 +2729,10 @@
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="3" t="s">
-        <v>156</v>
+        <v>51</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>113</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2810,93 +2750,98 @@
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="3" t="s">
-        <v>51</v>
+        <v>208</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>52</v>
+        <v>209</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G43" s="2"/>
       <c r="H43" s="3" t="s">
-        <v>212</v>
+        <v>21</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
         <v>214</v>
       </c>
       <c r="B44" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="F44" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="H44" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="G44" s="2"/>
-      <c r="H44" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
+      <c r="B45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E45" s="1" t="s">
+      <c r="F45" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="F45" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="H45" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>52</v>
+      <c r="G45" s="2"/>
+      <c r="H45" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>221</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="F46" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="G46" s="2"/>
       <c r="H46" s="3" t="s">
-        <v>27</v>
+        <v>131</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>151</v>
+        <v>132</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2904,46 +2849,45 @@
         <v>224</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="F47" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="F47" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="G47" s="2"/>
+      <c r="G47" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H47" s="3" t="s">
-        <v>156</v>
+        <v>45</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>113</v>
+        <v>46</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="E48" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="F48" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="G48" s="5" t="s">
         <v>231</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>131</v>
+        <v>15</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="J48" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="K48" s="3" t="s">
-        <v>126</v>
+        <v>16</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2951,7 +2895,7 @@
         <v>232</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>233</v>
@@ -2959,14 +2903,12 @@
       <c r="F49" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="G49" s="7" t="n">
-        <v>46366</v>
-      </c>
+      <c r="G49" s="2"/>
       <c r="H49" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2974,22 +2916,20 @@
         <v>235</v>
       </c>
       <c r="B50" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="F50" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="G50" s="2"/>
+      <c r="H50" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="G50" s="5" t="s">
+      <c r="I50" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I50" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2997,7 +2937,7 @@
         <v>240</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>85</v>
+        <v>36</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>241</v>
@@ -3007,7 +2947,7 @@
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="3" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>16</v>
@@ -3018,104 +2958,104 @@
         <v>243</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>209</v>
+        <v>244</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G52" s="2"/>
       <c r="H52" s="3" t="s">
-        <v>246</v>
+        <v>45</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>247</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E53" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B53" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E53" s="2" t="s">
+      <c r="F53" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>250</v>
       </c>
       <c r="G53" s="2"/>
       <c r="H53" s="3" t="s">
-        <v>15</v>
+        <v>172</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>16</v>
+        <v>132</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="F54" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>254</v>
       </c>
       <c r="G54" s="2"/>
       <c r="H54" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="E55" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B55" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E55" s="2" t="s">
+      <c r="F55" s="2" t="s">
         <v>256</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>257</v>
       </c>
       <c r="G55" s="2"/>
       <c r="H55" s="3" t="s">
-        <v>172</v>
+        <v>82</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="E56" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="F56" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>261</v>
       </c>
       <c r="G56" s="2"/>
       <c r="H56" s="3" t="s">
-        <v>156</v>
+        <v>45</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>113</v>
+        <v>261</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3133,10 +3073,10 @@
       </c>
       <c r="G57" s="2"/>
       <c r="H57" s="3" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3154,10 +3094,10 @@
       </c>
       <c r="G58" s="2"/>
       <c r="H58" s="3" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>113</v>
+        <v>261</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3178,15 +3118,15 @@
         <v>45</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>273</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>274</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>275</v>
@@ -3196,10 +3136,10 @@
       </c>
       <c r="G60" s="2"/>
       <c r="H60" s="3" t="s">
-        <v>21</v>
+        <v>172</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>22</v>
+        <v>132</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3217,10 +3157,10 @@
       </c>
       <c r="G61" s="2"/>
       <c r="H61" s="3" t="s">
-        <v>45</v>
+        <v>131</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>273</v>
+        <v>132</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3228,70 +3168,76 @@
         <v>281</v>
       </c>
       <c r="B62" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E62" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="E62" s="2" t="s">
+      <c r="F62" s="2" t="s">
         <v>283</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>284</v>
       </c>
       <c r="G62" s="2"/>
       <c r="H62" s="3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="E63" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="F63" s="2" t="s">
         <v>287</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>288</v>
       </c>
       <c r="G63" s="2"/>
       <c r="H63" s="3" t="s">
-        <v>172</v>
+        <v>15</v>
       </c>
       <c r="I63" s="3" t="s">
-        <v>132</v>
+        <v>16</v>
+      </c>
+      <c r="J63" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="K63" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="E64" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="F64" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>292</v>
       </c>
       <c r="G64" s="2"/>
       <c r="H64" s="3" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>293</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>294</v>
@@ -3301,10 +3247,10 @@
       </c>
       <c r="G65" s="2"/>
       <c r="H65" s="3" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3322,16 +3268,10 @@
       </c>
       <c r="G66" s="2"/>
       <c r="H66" s="3" t="s">
-        <v>15</v>
+        <v>131</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J66" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="K66" s="3" t="s">
-        <v>164</v>
+        <v>132</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3349,10 +3289,10 @@
       </c>
       <c r="G67" s="2"/>
       <c r="H67" s="3" t="s">
-        <v>156</v>
+        <v>45</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>113</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3370,10 +3310,10 @@
       </c>
       <c r="G68" s="2"/>
       <c r="H68" s="3" t="s">
-        <v>21</v>
+        <v>131</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>22</v>
+        <v>132</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3381,62 +3321,62 @@
         <v>308</v>
       </c>
       <c r="B69" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="E69" s="2" t="s">
+      <c r="F69" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="G69" s="2"/>
       <c r="H69" s="3" t="s">
-        <v>131</v>
+        <v>15</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>132</v>
+        <v>16</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="E70" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="E70" s="2" t="s">
+      <c r="F70" s="2" t="s">
         <v>314</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>315</v>
       </c>
       <c r="G70" s="2"/>
       <c r="H70" s="3" t="s">
-        <v>45</v>
+        <v>125</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>46</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E71" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="F71" s="2" t="s">
         <v>317</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>319</v>
       </c>
       <c r="G71" s="2"/>
       <c r="H71" s="3" t="s">
-        <v>131</v>
+        <v>318</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>132</v>
+        <v>319</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3444,41 +3384,39 @@
         <v>320</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>128</v>
+        <v>321</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="3" t="s">
-        <v>15</v>
+        <v>125</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>16</v>
+        <v>126</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="F73" s="2" t="s">
         <v>326</v>
       </c>
+      <c r="F73" s="2"/>
       <c r="G73" s="2"/>
       <c r="H73" s="3" t="s">
-        <v>125</v>
+        <v>238</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>126</v>
+        <v>239</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3486,7 +3424,7 @@
         <v>327</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>179</v>
+        <v>85</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>328</v>
@@ -3496,155 +3434,165 @@
       </c>
       <c r="G74" s="2"/>
       <c r="H74" s="3" t="s">
-        <v>330</v>
+        <v>177</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>331</v>
+        <v>16</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="F75" s="2" t="s">
         <v>332</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>335</v>
       </c>
       <c r="G75" s="2"/>
       <c r="H75" s="3" t="s">
-        <v>125</v>
+        <v>15</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>126</v>
+        <v>16</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>337</v>
+        <v>69</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="F76" s="2"/>
+        <v>334</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>335</v>
+      </c>
       <c r="G76" s="2"/>
       <c r="H76" s="3" t="s">
-        <v>246</v>
+        <v>51</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>247</v>
+        <v>52</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>85</v>
+        <v>270</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="G77" s="2"/>
       <c r="H77" s="3" t="s">
-        <v>177</v>
+        <v>45</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>179</v>
+        <v>258</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="G78" s="2"/>
       <c r="H78" s="3" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>69</v>
+        <v>312</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="G79" s="2"/>
       <c r="H79" s="3" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>52</v>
+        <v>16</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K79" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>282</v>
+        <v>91</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="G80" s="2"/>
       <c r="H80" s="3" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F81" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="B81" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="E81" s="2" t="s">
+      <c r="G81" s="4" t="n">
+        <v>45718</v>
+      </c>
+      <c r="H81" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="I81" s="3" t="s">
         <v>353</v>
-      </c>
-      <c r="G81" s="2"/>
-      <c r="H81" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I81" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3652,70 +3600,75 @@
         <v>354</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>324</v>
+        <v>321</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>355</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="G82" s="2"/>
+        <v>357</v>
+      </c>
+      <c r="G82" s="4" t="n">
+        <v>45779</v>
+      </c>
       <c r="H82" s="3" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="I82" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J82" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="K82" s="3" t="s">
-        <v>16</v>
+        <v>319</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>91</v>
+        <v>359</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>360</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="G83" s="2"/>
+        <v>362</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>45779</v>
+      </c>
       <c r="H83" s="3" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>361</v>
+        <v>128</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="G84" s="4" t="n">
-        <v>45718</v>
-      </c>
+        <v>365</v>
+      </c>
+      <c r="G84" s="2"/>
       <c r="H84" s="3" t="s">
-        <v>364</v>
+        <v>318</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3723,240 +3676,237 @@
         <v>366</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="C85" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E85" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="E85" s="2" t="s">
+      <c r="F85" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="F85" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="G85" s="4" t="n">
-        <v>45779</v>
-      </c>
+      <c r="G85" s="2"/>
       <c r="H85" s="3" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I85" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K85" s="3" t="s">
-        <v>331</v>
+        <v>46</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B86" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="E86" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="C86" s="1" t="s">
+      <c r="F86" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="E86" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="F86" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="G86" s="4" t="n">
-        <v>45779</v>
-      </c>
+      <c r="G86" s="2"/>
       <c r="H86" s="3" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>46</v>
+        <v>113</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F87" s="2" t="s">
         <v>375</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="F87" s="2" t="s">
-        <v>377</v>
       </c>
       <c r="G87" s="2"/>
       <c r="H87" s="3" t="s">
-        <v>330</v>
+        <v>156</v>
       </c>
       <c r="I87" s="3" t="s">
-        <v>331</v>
+        <v>113</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F88" s="2" t="s">
         <v>378</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>379</v>
-      </c>
-      <c r="F88" s="2" t="s">
-        <v>380</v>
       </c>
       <c r="G88" s="2"/>
       <c r="H88" s="3" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>46</v>
+        <v>16</v>
+      </c>
+      <c r="J88" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="K88" s="3" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="F89" s="2" t="s">
         <v>381</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="F89" s="2" t="s">
-        <v>384</v>
       </c>
       <c r="G89" s="2"/>
       <c r="H89" s="3" t="s">
-        <v>82</v>
+        <v>208</v>
       </c>
       <c r="I89" s="3" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B90" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="E90" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F90" s="2" t="s">
         <v>385</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="F90" s="2" t="s">
-        <v>387</v>
       </c>
       <c r="G90" s="2"/>
       <c r="H90" s="3" t="s">
-        <v>156</v>
+        <v>57</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F91" s="2" t="s">
         <v>388</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="F91" s="2" t="s">
-        <v>390</v>
       </c>
       <c r="G91" s="2"/>
       <c r="H91" s="3" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J91" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="K91" s="3" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="E92" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="B92" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="E92" s="2" t="s">
+      <c r="F92" s="2" t="s">
         <v>392</v>
-      </c>
-      <c r="F92" s="2" t="s">
-        <v>393</v>
       </c>
       <c r="G92" s="2"/>
       <c r="H92" s="3" t="s">
-        <v>212</v>
+        <v>15</v>
       </c>
       <c r="I92" s="3" t="s">
-        <v>213</v>
+        <v>16</v>
+      </c>
+      <c r="J92" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="K92" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E93" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="F93" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="E93" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="F93" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="G93" s="2"/>
+      <c r="G93" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H93" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="I93" s="3" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B94" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="F94" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="E94" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="F94" s="2"/>
       <c r="G94" s="2"/>
       <c r="H94" s="3" t="s">
-        <v>156</v>
+        <v>45</v>
       </c>
       <c r="I94" s="3" t="s">
-        <v>113</v>
+        <v>46</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E95" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="B95" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="E95" s="2" t="s">
+      <c r="F95" s="2" t="s">
         <v>401</v>
-      </c>
-      <c r="F95" s="2" t="s">
-        <v>402</v>
       </c>
       <c r="G95" s="2"/>
       <c r="H95" s="3" t="s">
@@ -3968,149 +3918,153 @@
     </row>
     <row r="96" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B96" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="E96" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="E96" s="2" t="s">
+      <c r="F96" s="2" t="s">
         <v>405</v>
-      </c>
-      <c r="F96" s="2" t="s">
-        <v>406</v>
       </c>
       <c r="G96" s="2"/>
       <c r="H96" s="3" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I96" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J96" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="K96" s="3" t="s">
-        <v>164</v>
+        <v>22</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E97" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="B97" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="E97" s="2" t="s">
+      <c r="F97" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="F97" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="G97" s="7" t="n">
-        <v>46366</v>
-      </c>
+      <c r="G97" s="2"/>
       <c r="H97" s="3" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I97" s="3" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E98" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="B98" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="E98" s="2" t="s">
+      <c r="F98" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>412</v>
       </c>
       <c r="G98" s="2"/>
       <c r="H98" s="3" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I98" s="3" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E99" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="F99" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="E99" s="2" t="s">
+      <c r="G99" s="5" t="s">
         <v>415</v>
       </c>
-      <c r="F99" s="2"/>
-      <c r="G99" s="2"/>
       <c r="H99" s="3" t="s">
-        <v>156</v>
+        <v>15</v>
       </c>
       <c r="I99" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="J99" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="K99" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>41</v>
+        <v>122</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="F100" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="G100" s="2"/>
+        <v>419</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="G100" s="5"/>
       <c r="H100" s="3" t="s">
-        <v>45</v>
+        <v>421</v>
       </c>
       <c r="I100" s="3" t="s">
-        <v>46</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="J100" s="3"/>
+      <c r="K100" s="3"/>
     </row>
     <row r="101" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>420</v>
+        <v>85</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="G101" s="2"/>
+        <v>424</v>
+      </c>
+      <c r="G101" s="7" t="n">
+        <v>46366</v>
+      </c>
       <c r="H101" s="3" t="s">
-        <v>21</v>
+        <v>125</v>
       </c>
       <c r="I101" s="3" t="s">
-        <v>22</v>
+        <v>126</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>91</v>
+        <v>426</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="F102" s="2" t="s">
-        <v>425</v>
-      </c>
+        <v>427</v>
+      </c>
+      <c r="F102" s="2"/>
       <c r="G102" s="2"/>
       <c r="H102" s="3" t="s">
         <v>15</v>
@@ -4118,44 +4072,48 @@
       <c r="I102" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="J102" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="K102" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="G103" s="2"/>
       <c r="H103" s="3" t="s">
-        <v>15</v>
+        <v>172</v>
       </c>
       <c r="I103" s="3" t="s">
-        <v>16</v>
+        <v>132</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>270</v>
+        <v>134</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="G104" s="5" t="s">
-        <v>432</v>
-      </c>
+        <v>433</v>
+      </c>
+      <c r="G104" s="2"/>
       <c r="H104" s="3" t="s">
         <v>15</v>
       </c>
@@ -4163,116 +4121,110 @@
         <v>16</v>
       </c>
       <c r="J104" s="3" t="s">
-        <v>433</v>
+        <v>51</v>
       </c>
       <c r="K104" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="s">
         <v>434</v>
       </c>
-    </row>
-    <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="1" t="s">
+      <c r="B105" s="1" t="s">
         <v>435</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>122</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="F105" s="8" t="s">
+      <c r="F105" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="G105" s="5"/>
-      <c r="H105" s="9" t="s">
+      <c r="G105" s="2"/>
+      <c r="H105" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I105" s="3" t="s">
         <v>438</v>
       </c>
-      <c r="I105" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="J105" s="3"/>
-      <c r="K105" s="3"/>
     </row>
     <row r="106" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
         <v>439</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>85</v>
+        <v>440</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F106" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="G106" s="7" t="n">
+        <v>442</v>
+      </c>
+      <c r="G106" s="2"/>
+      <c r="H106" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I106" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="G107" s="7" t="n">
         <v>46366</v>
       </c>
-      <c r="H106" s="3" t="s">
+      <c r="H107" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="I106" s="3" t="s">
+      <c r="I107" s="3" t="s">
         <v>126</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="E107" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F107" s="2"/>
-      <c r="G107" s="2"/>
-      <c r="H107" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I107" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J107" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="K107" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>69</v>
+        <v>448</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="G108" s="2"/>
       <c r="H108" s="3" t="s">
-        <v>172</v>
+        <v>125</v>
       </c>
       <c r="I108" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>134</v>
+        <v>85</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="G109" s="2"/>
       <c r="H109" s="3" t="s">
@@ -4282,125 +4234,17 @@
         <v>16</v>
       </c>
       <c r="J109" s="3" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="K109" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="B110" s="1" t="s">
-        <v>452</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="F110" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="G110" s="2"/>
-      <c r="H110" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="I110" s="3" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="1" t="s">
-        <v>456</v>
-      </c>
-      <c r="B111" s="1" t="s">
-        <v>457</v>
-      </c>
-      <c r="E111" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="F111" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="G111" s="2"/>
-      <c r="H111" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I111" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="10" t="s">
-        <v>460</v>
-      </c>
-      <c r="B112" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="E112" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="F112" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="G112" s="7" t="n">
-        <v>46366</v>
-      </c>
-      <c r="H112" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="I112" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="113" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="B113" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="F113" s="2" t="s">
-        <v>467</v>
-      </c>
-      <c r="G113" s="2"/>
-      <c r="H113" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="I113" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="B114" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="G114" s="2"/>
-      <c r="H114" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I114" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J114" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="K114" s="3" t="s">
         <v>73</v>
       </c>
     </row>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" display="helena.almazan@dipc.org"/>
@@ -4438,86 +4282,80 @@
     <hyperlink ref="E38" r:id="rId33" display="joshua.grocott@postgrad.manchester.ac.uk"/>
     <hyperlink ref="E39" r:id="rId34" display="roxanne.guenette@manchester.ac.uk"/>
     <hyperlink ref="E40" r:id="rId35" display="hauptman@iastate.edu"/>
-    <hyperlink ref="E41" r:id="rId36" display="henriques@uc.pt"/>
-    <hyperlink ref="E42" r:id="rId37" display="jose.hernando@usc.es"/>
-    <hyperlink ref="E43" r:id="rId38" display="pablo.herrero-gomez@mail.huji.ac.il"/>
-    <hyperlink ref="E44" r:id="rId39" display="viherbos@eln.upv.es"/>
-    <hyperlink ref="E46" r:id="rId40" display="yairifergan@gmail.com"/>
-    <hyperlink ref="E47" r:id="rId41" display="afbisabel@fis.uc.pt"/>
-    <hyperlink ref="F47" r:id="rId42" display="https://orcid.org/0000-0001-8025-8375"/>
-    <hyperlink ref="E48" r:id="rId43" display="benjamin.jones-7@manchester.ac.uk"/>
-    <hyperlink ref="E49" r:id="rId44" display="fabian.kellerer@ific.uv.es"/>
-    <hyperlink ref="E50" r:id="rId45" display="leire.larizgoitia@dipc.org"/>
-    <hyperlink ref="E51" r:id="rId46" display="amaia.larumbe@ehu.eus"/>
-    <hyperlink ref="E52" r:id="rId47" display="lebrun@fnal.gov"/>
-    <hyperlink ref="E53" r:id="rId48" display="francisco.lopez@dipc.org"/>
-    <hyperlink ref="E54" r:id="rId49" display="lopezneu@ific.uv.es"/>
-    <hyperlink ref="E55" r:id="rId50" display="ryan.madigan@mavs.uta.edu"/>
-    <hyperlink ref="E56" r:id="rId51" display="rdpmano@uc.pt"/>
-    <hyperlink ref="E57" r:id="rId52" display="aimar.marauri@ehu.eus"/>
-    <hyperlink ref="E58" r:id="rId53" display="afonso.marques97@gmail.com"/>
-    <hyperlink ref="E59" r:id="rId54" display="justo.martin-albo@ific.uv.es"/>
-    <hyperlink ref="E60" r:id="rId55" display="alberto.martinez.perez@ific.uv.es"/>
-    <hyperlink ref="E61" r:id="rId56" display="gonzaponte@gmail.com"/>
-    <hyperlink ref="E62" r:id="rId57" display="miryam.martinez@ific.uv.es"/>
-    <hyperlink ref="E63" r:id="rId58" display="rlm6389@mavs.uta.edu"/>
-    <hyperlink ref="E64" r:id="rId59" display="krishan.mistry@uta.edu"/>
-    <hyperlink ref="E65" r:id="rId60" display="juan.molina@ehu.eus"/>
-    <hyperlink ref="E66" r:id="rId61" display="francesc.monrabal@dipc.org"/>
-    <hyperlink ref="E67" r:id="rId62" display="cristinam@uc.pt"/>
-    <hyperlink ref="E68" r:id="rId63" display="fjmora@eln.upv.es"/>
-    <hyperlink ref="E69" r:id="rId64" display="ken6461@mavs.uta.edu"/>
-    <hyperlink ref="F69" r:id="rId65" display="https://orcid.org/0009-0009-0971-5559"/>
-    <hyperlink ref="E70" r:id="rId66" display="pau.novella@ific.uv.es"/>
-    <hyperlink ref="E71" r:id="rId67" display="nygren@uta.edu"/>
-    <hyperlink ref="E72" r:id="rId68" display="eva.oblak@dipc.org"/>
-    <hyperlink ref="E73" r:id="rId69" display="ian.osborne@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="F73" r:id="rId70" display="https://orcid.org/0009-0002-2780-2399"/>
-    <hyperlink ref="E74" r:id="rId71" display="jpalacio@lsc-canfranc.es"/>
-    <hyperlink ref="E75" r:id="rId72" display="brais.palmeiro@manchester.ac.uk"/>
-    <hyperlink ref="E76" r:id="rId73" display="para@fnal.gov"/>
-    <hyperlink ref="E77" r:id="rId74" display="ariadna.pazos@ehu.eus"/>
-    <hyperlink ref="E78" r:id="rId75" display="jorge.pelegrin@dipc.org"/>
-    <hyperlink ref="E79" r:id="rId76" display="martin.maneiro@usc.es"/>
-    <hyperlink ref="E80" r:id="rId77" display="marcque@ific.uv.es"/>
-    <hyperlink ref="E81" r:id="rId78" display="jrenner@ific.uv.es"/>
-    <hyperlink ref="E82" r:id="rId79" display="ivan.rivilla@ehu.es"/>
-    <hyperlink ref="E83" r:id="rId80" display="celia.rogero@csic.es"/>
-    <hyperlink ref="E84" r:id="rId81" display="Leslie.rogers776@gmail.com"/>
-    <hyperlink ref="E85" r:id="rId82" display="bromeo@dipc.org"/>
-    <hyperlink ref="E86" r:id="rId83" display="romoluque_c@lanl.gov"/>
-    <hyperlink ref="E87" r:id="rId84" display="eruiz@lsc-canfranc.es"/>
-    <hyperlink ref="E88" r:id="rId85" display="Pokhee.Saharia@ific.uv.es"/>
-    <hyperlink ref="F88" r:id="rId86" display="https://orcid.org/0009-0006-7366-4950"/>
-    <hyperlink ref="E89" r:id="rId87" display="filomena.santos@coimbra.lip.pt"/>
-    <hyperlink ref="E90" r:id="rId88" display="jmf@uc.pt"/>
-    <hyperlink ref="E91" r:id="rId89" display="marc.seemann@dipc.org"/>
-    <hyperlink ref="E92" r:id="rId90" display="itay.shomroni@mail.huji.ac.il"/>
-    <hyperlink ref="E93" r:id="rId91" display="analuisa.silva@ua.pt"/>
-    <hyperlink ref="F93" r:id="rId92" display="https://orcid.org/0000-0002-8363-0109"/>
-    <hyperlink ref="E94" r:id="rId93" display="pesilva@uc.pt"/>
-    <hyperlink ref="E95" r:id="rId94" display="ander.simon@ific.uv.es"/>
-    <hyperlink ref="E96" r:id="rId95" display="roberto.soleti@dipc.org"/>
-    <hyperlink ref="E97" r:id="rId96" display="sorel@ific.uv.es"/>
-    <hyperlink ref="E98" r:id="rId97" display="josealfonso.soto@ific.uv.es"/>
-    <hyperlink ref="E99" r:id="rId98" display="jmrt@uc.pt"/>
-    <hyperlink ref="E100" r:id="rId99" display="steruel@ific.uv.es"/>
-    <hyperlink ref="E101" r:id="rId100" display="jtoledo@eln.upv.es"/>
-    <hyperlink ref="E102" r:id="rId101" display="claire.tonnele@dipc.org"/>
-    <hyperlink ref="E103" r:id="rId102" display="samuele.torelli@dipc.org"/>
-    <hyperlink ref="E104" r:id="rId103" display="jordi.torrent@udg.edu"/>
-    <hyperlink ref="F105" r:id="rId104" display="https://orcid.org/0000-0002-7621-5804"/>
-    <hyperlink ref="E106" r:id="rId105" display="alexandra.trettin@manchester.ac.uk"/>
-    <hyperlink ref="E107" r:id="rId106" display="pablo.garcia@dipc.org"/>
-    <hyperlink ref="E108" r:id="rId107" display="mukundam.vanga@uta.edu"/>
-    <hyperlink ref="E109" r:id="rId108" display="pablo.vazquez@dipc.org"/>
-    <hyperlink ref="F109" r:id="rId109" display="https://orcid.org/0009-0007-0098-8927"/>
-    <hyperlink ref="E110" r:id="rId110" display="joao.veloso@ua.pt"/>
-    <hyperlink ref="E111" r:id="rId111" display="Juan.Villamil@ific.uv.es"/>
-    <hyperlink ref="E112" r:id="rId112" display="luismiguel.villarpadruno@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="F112" r:id="rId113" display="https://orcid.org/0009-0002-5335-0891"/>
-    <hyperlink ref="E113" r:id="rId114" display="john.waiton@postgrad.manchester.ac.uk"/>
-    <hyperlink ref="E114" r:id="rId115" display="alfonso.yubero@dipc.org"/>
+    <hyperlink ref="E41" r:id="rId36" display="jose.hernando@usc.es"/>
+    <hyperlink ref="E42" r:id="rId37" display="pablo.herrero-gomez@mail.huji.ac.il"/>
+    <hyperlink ref="E43" r:id="rId38" display="viherbos@eln.upv.es"/>
+    <hyperlink ref="E45" r:id="rId39" display="yairifergan@gmail.com"/>
+    <hyperlink ref="E46" r:id="rId40" display="benjamin.jones-7@manchester.ac.uk"/>
+    <hyperlink ref="E47" r:id="rId41" display="fabian.kellerer@ific.uv.es"/>
+    <hyperlink ref="E48" r:id="rId42" display="leire.larizgoitia@dipc.org"/>
+    <hyperlink ref="E49" r:id="rId43" display="amaia.larumbe@ehu.eus"/>
+    <hyperlink ref="E50" r:id="rId44" display="lebrun@fnal.gov"/>
+    <hyperlink ref="E51" r:id="rId45" display="francisco.lopez@dipc.org"/>
+    <hyperlink ref="E52" r:id="rId46" display="lopezneu@ific.uv.es"/>
+    <hyperlink ref="E53" r:id="rId47" display="ryan.madigan@mavs.uta.edu"/>
+    <hyperlink ref="E54" r:id="rId48" display="aimar.marauri@ehu.eus"/>
+    <hyperlink ref="E55" r:id="rId49" display="afonso.marques97@gmail.com"/>
+    <hyperlink ref="E56" r:id="rId50" display="justo.martin-albo@ific.uv.es"/>
+    <hyperlink ref="E57" r:id="rId51" display="alberto.martinez.perez@ific.uv.es"/>
+    <hyperlink ref="E58" r:id="rId52" display="gonzaponte@gmail.com"/>
+    <hyperlink ref="E59" r:id="rId53" display="miryam.martinez@ific.uv.es"/>
+    <hyperlink ref="E60" r:id="rId54" display="rlm6389@mavs.uta.edu"/>
+    <hyperlink ref="E61" r:id="rId55" display="krishan.mistry@uta.edu"/>
+    <hyperlink ref="E62" r:id="rId56" display="juan.molina@ehu.eus"/>
+    <hyperlink ref="E63" r:id="rId57" display="francesc.monrabal@dipc.org"/>
+    <hyperlink ref="E64" r:id="rId58" display="cristinam@uc.pt"/>
+    <hyperlink ref="E65" r:id="rId59" display="fjmora@eln.upv.es"/>
+    <hyperlink ref="E66" r:id="rId60" display="ken6461@mavs.uta.edu"/>
+    <hyperlink ref="F66" r:id="rId61" display="https://orcid.org/0009-0009-0971-5559"/>
+    <hyperlink ref="E67" r:id="rId62" display="pau.novella@ific.uv.es"/>
+    <hyperlink ref="E68" r:id="rId63" display="nygren@uta.edu"/>
+    <hyperlink ref="E69" r:id="rId64" display="eva.oblak@dipc.org"/>
+    <hyperlink ref="E70" r:id="rId65" display="ian.osborne@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="F70" r:id="rId66" display="https://orcid.org/0009-0002-2780-2399"/>
+    <hyperlink ref="E71" r:id="rId67" display="jpalacio@lsc-canfranc.es"/>
+    <hyperlink ref="E72" r:id="rId68" display="brais.palmeiro@manchester.ac.uk"/>
+    <hyperlink ref="E73" r:id="rId69" display="para@fnal.gov"/>
+    <hyperlink ref="E74" r:id="rId70" display="ariadna.pazos@ehu.eus"/>
+    <hyperlink ref="E75" r:id="rId71" display="jorge.pelegrin@dipc.org"/>
+    <hyperlink ref="E76" r:id="rId72" display="martin.maneiro@usc.es"/>
+    <hyperlink ref="E77" r:id="rId73" display="marcque@ific.uv.es"/>
+    <hyperlink ref="E78" r:id="rId74" display="jrenner@ific.uv.es"/>
+    <hyperlink ref="E79" r:id="rId75" display="ivan.rivilla@ehu.es"/>
+    <hyperlink ref="E80" r:id="rId76" display="celia.rogero@csic.es"/>
+    <hyperlink ref="E81" r:id="rId77" display="Leslie.rogers776@gmail.com"/>
+    <hyperlink ref="E82" r:id="rId78" display="bromeo@dipc.org"/>
+    <hyperlink ref="E83" r:id="rId79" display="romoluque_c@lanl.gov"/>
+    <hyperlink ref="E84" r:id="rId80" display="eruiz@lsc-canfranc.es"/>
+    <hyperlink ref="E85" r:id="rId81" display="Pokhee.Saharia@ific.uv.es"/>
+    <hyperlink ref="F85" r:id="rId82" display="https://orcid.org/0009-0006-7366-4950"/>
+    <hyperlink ref="E86" r:id="rId83" display="filomena.santos@coimbra.lip.pt"/>
+    <hyperlink ref="E87" r:id="rId84" display="jmf@uc.pt"/>
+    <hyperlink ref="E88" r:id="rId85" display="marc.seemann@dipc.org"/>
+    <hyperlink ref="E89" r:id="rId86" display="itay.shomroni@mail.huji.ac.il"/>
+    <hyperlink ref="E90" r:id="rId87" display="analuisa.silva@ua.pt"/>
+    <hyperlink ref="F90" r:id="rId88" display="https://orcid.org/0000-0002-8363-0109"/>
+    <hyperlink ref="E91" r:id="rId89" display="ander.simon@ific.uv.es"/>
+    <hyperlink ref="E92" r:id="rId90" display="roberto.soleti@dipc.org"/>
+    <hyperlink ref="E93" r:id="rId91" display="sorel@ific.uv.es"/>
+    <hyperlink ref="E94" r:id="rId92" display="josealfonso.soto@ific.uv.es"/>
+    <hyperlink ref="E95" r:id="rId93" display="steruel@ific.uv.es"/>
+    <hyperlink ref="E96" r:id="rId94" display="jtoledo@eln.upv.es"/>
+    <hyperlink ref="E97" r:id="rId95" display="claire.tonnele@dipc.org"/>
+    <hyperlink ref="E98" r:id="rId96" display="samuele.torelli@dipc.org"/>
+    <hyperlink ref="E99" r:id="rId97" display="jordi.torrent@udg.edu"/>
+    <hyperlink ref="F100" r:id="rId98" display="https://orcid.org/0000-0002-7621-5804"/>
+    <hyperlink ref="E101" r:id="rId99" display="alexandra.trettin@manchester.ac.uk"/>
+    <hyperlink ref="E102" r:id="rId100" display="pablo.garcia@dipc.org"/>
+    <hyperlink ref="E103" r:id="rId101" display="mukundam.vanga@uta.edu"/>
+    <hyperlink ref="E104" r:id="rId102" display="pablo.vazquez@dipc.org"/>
+    <hyperlink ref="F104" r:id="rId103" display="https://orcid.org/0009-0007-0098-8927"/>
+    <hyperlink ref="E105" r:id="rId104" display="joao.veloso@ua.pt"/>
+    <hyperlink ref="E106" r:id="rId105" display="Juan.Villamil@ific.uv.es"/>
+    <hyperlink ref="E107" r:id="rId106" display="luismiguel.villarpadruno@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="F107" r:id="rId107" display="https://orcid.org/0009-0002-5335-0891"/>
+    <hyperlink ref="E108" r:id="rId108" display="john.waiton@postgrad.manchester.ac.uk"/>
+    <hyperlink ref="E109" r:id="rId109" display="alfonso.yubero@dipc.org"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>